<commit_message>
Backtest: add B&H benchmarks for all 4 ETFs + month-by-month table on tab
</commit_message>
<xml_diff>
--- a/backtest.xlsx
+++ b/backtest.xlsx
@@ -3075,7 +3075,7 @@
         <v>6375.7</v>
       </c>
       <c r="R32" t="n">
-        <v>131676.3</v>
+        <v>131676.4</v>
       </c>
       <c r="S32" t="n">
         <v>0</v>
@@ -3399,7 +3399,7 @@
         <v>6375.7</v>
       </c>
       <c r="R36" t="n">
-        <v>180876.5</v>
+        <v>180876.6</v>
       </c>
       <c r="S36" t="n">
         <v>0</v>
@@ -3486,10 +3486,10 @@
         <v>0</v>
       </c>
       <c r="T37" t="n">
-        <v>434750</v>
+        <v>434751</v>
       </c>
       <c r="U37" t="n">
-        <v>434750</v>
+        <v>434751</v>
       </c>
       <c r="V37" t="n">
         <v>360000</v>
@@ -3744,7 +3744,7 @@
         <v>1.715</v>
       </c>
       <c r="Y40" t="n">
-        <v>503926</v>
+        <v>503927</v>
       </c>
     </row>
     <row r="41">
@@ -3987,7 +3987,7 @@
         <v>1.721</v>
       </c>
       <c r="Y43" t="n">
-        <v>551361</v>
+        <v>551360</v>
       </c>
     </row>
     <row r="44">
@@ -4068,7 +4068,7 @@
         <v>1.957</v>
       </c>
       <c r="Y44" t="n">
-        <v>587993</v>
+        <v>587994</v>
       </c>
     </row>
     <row r="45">
@@ -4149,7 +4149,7 @@
         <v>2.141</v>
       </c>
       <c r="Y45" t="n">
-        <v>627130</v>
+        <v>627129</v>
       </c>
     </row>
     <row r="46">
@@ -4296,10 +4296,10 @@
         <v>0</v>
       </c>
       <c r="T47" t="n">
-        <v>880929</v>
+        <v>880930</v>
       </c>
       <c r="U47" t="n">
-        <v>880929</v>
+        <v>880930</v>
       </c>
       <c r="V47" t="n">
         <v>460000</v>
@@ -4620,10 +4620,10 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>974912</v>
+        <v>974913</v>
       </c>
       <c r="U51" t="n">
-        <v>974912</v>
+        <v>974913</v>
       </c>
       <c r="V51" t="n">
         <v>500000</v>
@@ -4635,7 +4635,7 @@
         <v>2.608</v>
       </c>
       <c r="Y51" t="n">
-        <v>728448</v>
+        <v>728449</v>
       </c>
     </row>
     <row r="52">
@@ -4878,7 +4878,7 @@
         <v>3.097</v>
       </c>
       <c r="Y54" t="n">
-        <v>824700</v>
+        <v>824699</v>
       </c>
     </row>
     <row r="55">
@@ -5187,10 +5187,10 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>1607745</v>
+        <v>1607746</v>
       </c>
       <c r="U58" t="n">
-        <v>1607745</v>
+        <v>1607746</v>
       </c>
       <c r="V58" t="n">
         <v>570000</v>
@@ -5418,7 +5418,7 @@
         <v>1797.9</v>
       </c>
       <c r="P61" t="n">
-        <v>330024.6</v>
+        <v>330024.5</v>
       </c>
       <c r="Q61" t="n">
         <v>6588.2</v>
@@ -5430,10 +5430,10 @@
         <v>0</v>
       </c>
       <c r="T61" t="n">
-        <v>1756343</v>
+        <v>1756344</v>
       </c>
       <c r="U61" t="n">
-        <v>1756343</v>
+        <v>1756344</v>
       </c>
       <c r="V61" t="n">
         <v>600000</v>
@@ -5499,7 +5499,7 @@
         <v>1797.9</v>
       </c>
       <c r="P62" t="n">
-        <v>332467</v>
+        <v>332466.9</v>
       </c>
       <c r="Q62" t="n">
         <v>6588.2</v>
@@ -5592,10 +5592,10 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>1661897</v>
+        <v>1661896</v>
       </c>
       <c r="U63" t="n">
-        <v>1661897</v>
+        <v>1661896</v>
       </c>
       <c r="V63" t="n">
         <v>620000</v>
@@ -6228,7 +6228,7 @@
         <v>1950.3</v>
       </c>
       <c r="P71" t="n">
-        <v>345701.8</v>
+        <v>345701.7</v>
       </c>
       <c r="Q71" t="n">
         <v>7245.6</v>
@@ -6255,7 +6255,7 @@
         <v>3.921</v>
       </c>
       <c r="Y71" t="n">
-        <v>1167298</v>
+        <v>1167297</v>
       </c>
     </row>
     <row r="72">
@@ -6309,7 +6309,7 @@
         <v>2002</v>
       </c>
       <c r="P72" t="n">
-        <v>345701.8</v>
+        <v>345701.7</v>
       </c>
       <c r="Q72" t="n">
         <v>7466.2</v>
@@ -6390,7 +6390,7 @@
         <v>2054.4</v>
       </c>
       <c r="P73" t="n">
-        <v>345701.8</v>
+        <v>345701.7</v>
       </c>
       <c r="Q73" t="n">
         <v>7683.6</v>
@@ -6417,7 +6417,7 @@
         <v>3.133</v>
       </c>
       <c r="Y73" t="n">
-        <v>1089446</v>
+        <v>1089447</v>
       </c>
     </row>
     <row r="74">
@@ -6471,7 +6471,7 @@
         <v>2103.5</v>
       </c>
       <c r="P74" t="n">
-        <v>345701.8</v>
+        <v>345701.7</v>
       </c>
       <c r="Q74" t="n">
         <v>7882.7</v>
@@ -6645,10 +6645,10 @@
         <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>1726274</v>
+        <v>1726273</v>
       </c>
       <c r="U76" t="n">
-        <v>1726274</v>
+        <v>1726273</v>
       </c>
       <c r="V76" t="n">
         <v>750000</v>
@@ -6714,7 +6714,7 @@
         <v>2103.5</v>
       </c>
       <c r="P77" t="n">
-        <v>353436.6</v>
+        <v>353436.5</v>
       </c>
       <c r="Q77" t="n">
         <v>7882.7</v>
@@ -6741,7 +6741,7 @@
         <v>3.694</v>
       </c>
       <c r="Y77" t="n">
-        <v>1189265</v>
+        <v>1189266</v>
       </c>
     </row>
     <row r="78">
@@ -6822,7 +6822,7 @@
         <v>4.553</v>
       </c>
       <c r="Y78" t="n">
-        <v>1284298</v>
+        <v>1284297</v>
       </c>
     </row>
     <row r="79">
@@ -6903,7 +6903,7 @@
         <v>4.88</v>
       </c>
       <c r="Y79" t="n">
-        <v>1307773</v>
+        <v>1307774</v>
       </c>
     </row>
     <row r="80">
@@ -6969,10 +6969,10 @@
         <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>2371550</v>
+        <v>2371549</v>
       </c>
       <c r="U80" t="n">
-        <v>2371550</v>
+        <v>2371549</v>
       </c>
       <c r="V80" t="n">
         <v>790000</v>
@@ -7050,10 +7050,10 @@
         <v>0</v>
       </c>
       <c r="T81" t="n">
-        <v>2284298</v>
+        <v>2284299</v>
       </c>
       <c r="U81" t="n">
-        <v>2284298</v>
+        <v>2284299</v>
       </c>
       <c r="V81" t="n">
         <v>800000</v>
@@ -7131,10 +7131,10 @@
         <v>0</v>
       </c>
       <c r="T82" t="n">
-        <v>2516509</v>
+        <v>2516508</v>
       </c>
       <c r="U82" t="n">
-        <v>2516509</v>
+        <v>2516508</v>
       </c>
       <c r="V82" t="n">
         <v>810000</v>
@@ -7551,7 +7551,7 @@
         <v>7.837</v>
       </c>
       <c r="Y87" t="n">
-        <v>1626828</v>
+        <v>1626829</v>
       </c>
     </row>
     <row r="88">
@@ -7713,7 +7713,7 @@
         <v>8.175000000000001</v>
       </c>
       <c r="Y89" t="n">
-        <v>1670802</v>
+        <v>1670801</v>
       </c>
     </row>
     <row r="90">
@@ -7794,7 +7794,7 @@
         <v>9.17</v>
       </c>
       <c r="Y90" t="n">
-        <v>1748648</v>
+        <v>1748649</v>
       </c>
     </row>
     <row r="91">
@@ -8022,10 +8022,10 @@
         <v>0</v>
       </c>
       <c r="T93" t="n">
-        <v>5877481</v>
+        <v>5877482</v>
       </c>
       <c r="U93" t="n">
-        <v>5877481</v>
+        <v>5877482</v>
       </c>
       <c r="V93" t="n">
         <v>920000</v>
@@ -8172,7 +8172,7 @@
         <v>2103.5</v>
       </c>
       <c r="P95" t="n">
-        <v>380207.3</v>
+        <v>380207.2</v>
       </c>
       <c r="Q95" t="n">
         <v>7882.7</v>
@@ -8346,10 +8346,10 @@
         <v>0</v>
       </c>
       <c r="T97" t="n">
-        <v>6984217</v>
+        <v>6984218</v>
       </c>
       <c r="U97" t="n">
-        <v>6984217</v>
+        <v>6984218</v>
       </c>
       <c r="V97" t="n">
         <v>960000</v>
@@ -8427,10 +8427,10 @@
         <v>0</v>
       </c>
       <c r="T98" t="n">
-        <v>6277672</v>
+        <v>6277671</v>
       </c>
       <c r="U98" t="n">
-        <v>6277672</v>
+        <v>6277671</v>
       </c>
       <c r="V98" t="n">
         <v>970000</v>
@@ -8496,7 +8496,7 @@
         <v>2103.5</v>
       </c>
       <c r="P99" t="n">
-        <v>383425.4</v>
+        <v>383425.3</v>
       </c>
       <c r="Q99" t="n">
         <v>7882.7</v>
@@ -8508,10 +8508,10 @@
         <v>0</v>
       </c>
       <c r="T99" t="n">
-        <v>5568499</v>
+        <v>5568498</v>
       </c>
       <c r="U99" t="n">
-        <v>5568499</v>
+        <v>5568498</v>
       </c>
       <c r="V99" t="n">
         <v>980000</v>
@@ -8523,7 +8523,7 @@
         <v>11.772</v>
       </c>
       <c r="Y99" t="n">
-        <v>2069155</v>
+        <v>2069156</v>
       </c>
     </row>
     <row r="100">
@@ -8604,7 +8604,7 @@
         <v>14.706</v>
       </c>
       <c r="Y100" t="n">
-        <v>2196528</v>
+        <v>2196527</v>
       </c>
     </row>
     <row r="101">
@@ -8658,7 +8658,7 @@
         <v>2103.5</v>
       </c>
       <c r="P101" t="n">
-        <v>384909.6</v>
+        <v>384909.5</v>
       </c>
       <c r="Q101" t="n">
         <v>7882.7</v>
@@ -8670,10 +8670,10 @@
         <v>0</v>
       </c>
       <c r="T101" t="n">
-        <v>6498414</v>
+        <v>6498413</v>
       </c>
       <c r="U101" t="n">
-        <v>6498414</v>
+        <v>6498413</v>
       </c>
       <c r="V101" t="n">
         <v>1000000</v>
@@ -8685,7 +8685,7 @@
         <v>13.697</v>
       </c>
       <c r="Y101" t="n">
-        <v>2231669</v>
+        <v>2231668</v>
       </c>
     </row>
     <row r="102">
@@ -8751,10 +8751,10 @@
         <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>7078887</v>
+        <v>7078886</v>
       </c>
       <c r="U102" t="n">
-        <v>7078887</v>
+        <v>7078886</v>
       </c>
       <c r="V102" t="n">
         <v>1010000</v>
@@ -8766,7 +8766,7 @@
         <v>14.9</v>
       </c>
       <c r="Y102" t="n">
-        <v>2304065</v>
+        <v>2304064</v>
       </c>
     </row>
     <row r="103">
@@ -8913,10 +8913,10 @@
         <v>0</v>
       </c>
       <c r="T104" t="n">
-        <v>7517181</v>
+        <v>7517180</v>
       </c>
       <c r="U104" t="n">
-        <v>7517181</v>
+        <v>7517180</v>
       </c>
       <c r="V104" t="n">
         <v>1030000</v>
@@ -9009,7 +9009,7 @@
         <v>11.231</v>
       </c>
       <c r="Y105" t="n">
-        <v>2249709</v>
+        <v>2249708</v>
       </c>
     </row>
     <row r="106">
@@ -9063,7 +9063,7 @@
         <v>2134.4</v>
       </c>
       <c r="P106" t="n">
-        <v>387588.3</v>
+        <v>387588.2</v>
       </c>
       <c r="Q106" t="n">
         <v>7997.5</v>
@@ -9144,7 +9144,7 @@
         <v>2168.3</v>
       </c>
       <c r="P107" t="n">
-        <v>387588.3</v>
+        <v>387588.2</v>
       </c>
       <c r="Q107" t="n">
         <v>8118</v>
@@ -9156,10 +9156,10 @@
         <v>0</v>
       </c>
       <c r="T107" t="n">
-        <v>4252568</v>
+        <v>4252567</v>
       </c>
       <c r="U107" t="n">
-        <v>4252568</v>
+        <v>4252567</v>
       </c>
       <c r="V107" t="n">
         <v>1060000</v>
@@ -9318,10 +9318,10 @@
         <v>0</v>
       </c>
       <c r="T109" t="n">
-        <v>6004060</v>
+        <v>6004059</v>
       </c>
       <c r="U109" t="n">
-        <v>6004060</v>
+        <v>6004059</v>
       </c>
       <c r="V109" t="n">
         <v>1080000</v>
@@ -9399,10 +9399,10 @@
         <v>0</v>
       </c>
       <c r="T110" t="n">
-        <v>6552313</v>
+        <v>6552312</v>
       </c>
       <c r="U110" t="n">
-        <v>6552313</v>
+        <v>6552312</v>
       </c>
       <c r="V110" t="n">
         <v>1090000</v>
@@ -9414,7 +9414,7 @@
         <v>13.603</v>
       </c>
       <c r="Y110" t="n">
-        <v>2444586</v>
+        <v>2444585</v>
       </c>
     </row>
     <row r="111">
@@ -9642,10 +9642,10 @@
         <v>0</v>
       </c>
       <c r="T113" t="n">
-        <v>7101970</v>
+        <v>7101971</v>
       </c>
       <c r="U113" t="n">
-        <v>7101970</v>
+        <v>7101971</v>
       </c>
       <c r="V113" t="n">
         <v>1120000</v>
@@ -9738,7 +9738,7 @@
         <v>16.261</v>
       </c>
       <c r="Y114" t="n">
-        <v>2647303</v>
+        <v>2647302</v>
       </c>
     </row>
     <row r="115">
@@ -9885,10 +9885,10 @@
         <v>0</v>
       </c>
       <c r="T116" t="n">
-        <v>7674559</v>
+        <v>7674558</v>
       </c>
       <c r="U116" t="n">
-        <v>7674559</v>
+        <v>7674558</v>
       </c>
       <c r="V116" t="n">
         <v>1150000</v>
@@ -9966,10 +9966,10 @@
         <v>0</v>
       </c>
       <c r="T117" t="n">
-        <v>8740736</v>
+        <v>8740737</v>
       </c>
       <c r="U117" t="n">
-        <v>8740736</v>
+        <v>8740737</v>
       </c>
       <c r="V117" t="n">
         <v>1160000</v>
@@ -9981,7 +9981,7 @@
         <v>17.974</v>
       </c>
       <c r="Y117" t="n">
-        <v>2766590</v>
+        <v>2766589</v>
       </c>
     </row>
     <row r="118">
@@ -10035,7 +10035,7 @@
         <v>2168.3</v>
       </c>
       <c r="P118" t="n">
-        <v>395333.4</v>
+        <v>395333.3</v>
       </c>
       <c r="Q118" t="n">
         <v>8118</v>
@@ -10047,10 +10047,10 @@
         <v>0</v>
       </c>
       <c r="T118" t="n">
-        <v>9720972</v>
+        <v>9720973</v>
       </c>
       <c r="U118" t="n">
-        <v>9720972</v>
+        <v>9720973</v>
       </c>
       <c r="V118" t="n">
         <v>1170000</v>
@@ -10128,10 +10128,10 @@
         <v>0</v>
       </c>
       <c r="T119" t="n">
-        <v>11444854</v>
+        <v>11444855</v>
       </c>
       <c r="U119" t="n">
-        <v>11444854</v>
+        <v>11444855</v>
       </c>
       <c r="V119" t="n">
         <v>1180000</v>
@@ -10209,10 +10209,10 @@
         <v>0</v>
       </c>
       <c r="T120" t="n">
-        <v>11066394</v>
+        <v>11066393</v>
       </c>
       <c r="U120" t="n">
-        <v>11066394</v>
+        <v>11066393</v>
       </c>
       <c r="V120" t="n">
         <v>1190000</v>
@@ -10224,7 +10224,7 @@
         <v>22.693</v>
       </c>
       <c r="Y120" t="n">
-        <v>3112927</v>
+        <v>3112928</v>
       </c>
     </row>
     <row r="121">
@@ -10290,10 +10290,10 @@
         <v>0</v>
       </c>
       <c r="T121" t="n">
-        <v>9345551</v>
+        <v>9345549</v>
       </c>
       <c r="U121" t="n">
-        <v>9345551</v>
+        <v>9345549</v>
       </c>
       <c r="V121" t="n">
         <v>1200000</v>
@@ -10305,7 +10305,7 @@
         <v>19.144</v>
       </c>
       <c r="Y121" t="n">
-        <v>2934354</v>
+        <v>2934355</v>
       </c>
     </row>
     <row r="122">
@@ -10386,7 +10386,7 @@
         <v>10.882</v>
       </c>
       <c r="Y122" t="n">
-        <v>2730551</v>
+        <v>2730552</v>
       </c>
     </row>
     <row r="123">
@@ -10533,10 +10533,10 @@
         <v>0</v>
       </c>
       <c r="T124" t="n">
-        <v>8576081</v>
+        <v>8576082</v>
       </c>
       <c r="U124" t="n">
-        <v>8576081</v>
+        <v>8576082</v>
       </c>
       <c r="V124" t="n">
         <v>1230000</v>
@@ -10548,7 +10548,7 @@
         <v>17.49</v>
       </c>
       <c r="Y124" t="n">
-        <v>3367286</v>
+        <v>3367287</v>
       </c>
     </row>
     <row r="125">
@@ -10614,10 +10614,10 @@
         <v>0</v>
       </c>
       <c r="T125" t="n">
-        <v>10167704</v>
+        <v>10167703</v>
       </c>
       <c r="U125" t="n">
-        <v>10167704</v>
+        <v>10167703</v>
       </c>
       <c r="V125" t="n">
         <v>1240000</v>
@@ -10629,7 +10629,7 @@
         <v>20.716</v>
       </c>
       <c r="Y125" t="n">
-        <v>3588968</v>
+        <v>3588967</v>
       </c>
     </row>
     <row r="126">
@@ -10695,10 +10695,10 @@
         <v>0</v>
       </c>
       <c r="T126" t="n">
-        <v>12195956</v>
+        <v>12195955</v>
       </c>
       <c r="U126" t="n">
-        <v>12195956</v>
+        <v>12195955</v>
       </c>
       <c r="V126" t="n">
         <v>1250000</v>
@@ -10710,7 +10710,7 @@
         <v>24.828</v>
       </c>
       <c r="Y126" t="n">
-        <v>3862620</v>
+        <v>3862621</v>
       </c>
     </row>
     <row r="127">
@@ -10743,7 +10743,7 @@
         <v>0</v>
       </c>
       <c r="I127" t="n">
-        <v>767293</v>
+        <v>767294</v>
       </c>
       <c r="J127" t="n">
         <v>1245048</v>
@@ -10776,10 +10776,10 @@
         <v>2010329</v>
       </c>
       <c r="T127" t="n">
-        <v>13235306</v>
+        <v>13235309</v>
       </c>
       <c r="U127" t="n">
-        <v>15245635</v>
+        <v>15245638</v>
       </c>
       <c r="V127" t="n">
         <v>1260000</v>
@@ -10791,7 +10791,7 @@
         <v>31.02</v>
       </c>
       <c r="Y127" t="n">
-        <v>4295364</v>
+        <v>4295365</v>
       </c>
     </row>
     <row r="128">
@@ -10857,10 +10857,10 @@
         <v>2010329</v>
       </c>
       <c r="T128" t="n">
-        <v>11640571</v>
+        <v>11640572</v>
       </c>
       <c r="U128" t="n">
-        <v>13650900</v>
+        <v>13650901</v>
       </c>
       <c r="V128" t="n">
         <v>1270000</v>
@@ -10872,7 +10872,7 @@
         <v>27.755</v>
       </c>
       <c r="Y128" t="n">
-        <v>4057142</v>
+        <v>4057143</v>
       </c>
     </row>
     <row r="129">
@@ -10938,10 +10938,10 @@
         <v>2010329</v>
       </c>
       <c r="T129" t="n">
-        <v>10980388</v>
+        <v>10980389</v>
       </c>
       <c r="U129" t="n">
-        <v>12990717</v>
+        <v>12990718</v>
       </c>
       <c r="V129" t="n">
         <v>1280000</v>
@@ -10953,7 +10953,7 @@
         <v>26.393</v>
       </c>
       <c r="Y129" t="n">
-        <v>3943594</v>
+        <v>3943595</v>
       </c>
     </row>
     <row r="130">
@@ -11019,10 +11019,10 @@
         <v>2010329</v>
       </c>
       <c r="T130" t="n">
-        <v>15859052</v>
+        <v>15859051</v>
       </c>
       <c r="U130" t="n">
-        <v>17869381</v>
+        <v>17869380</v>
       </c>
       <c r="V130" t="n">
         <v>1290000</v>
@@ -11034,7 +11034,7 @@
         <v>36.284</v>
       </c>
       <c r="Y130" t="n">
-        <v>4396285</v>
+        <v>4396283</v>
       </c>
     </row>
     <row r="131">
@@ -11100,10 +11100,10 @@
         <v>2010329</v>
       </c>
       <c r="T131" t="n">
-        <v>18095378</v>
+        <v>18095381</v>
       </c>
       <c r="U131" t="n">
-        <v>20105707</v>
+        <v>20105711</v>
       </c>
       <c r="V131" t="n">
         <v>1300000</v>
@@ -11181,10 +11181,10 @@
         <v>2010329</v>
       </c>
       <c r="T132" t="n">
-        <v>18748465</v>
+        <v>18748462</v>
       </c>
       <c r="U132" t="n">
-        <v>20758794</v>
+        <v>20758792</v>
       </c>
       <c r="V132" t="n">
         <v>1310000</v>
@@ -11262,7 +11262,7 @@
         <v>2010329</v>
       </c>
       <c r="T133" t="n">
-        <v>20195912</v>
+        <v>20195911</v>
       </c>
       <c r="U133" t="n">
         <v>22206241</v>
@@ -11277,7 +11277,7 @@
         <v>45.026</v>
       </c>
       <c r="Y133" t="n">
-        <v>4647657</v>
+        <v>4647660</v>
       </c>
     </row>
     <row r="134">
@@ -11343,10 +11343,10 @@
         <v>2010329</v>
       </c>
       <c r="T134" t="n">
-        <v>20268339</v>
+        <v>20268341</v>
       </c>
       <c r="U134" t="n">
-        <v>22278668</v>
+        <v>22278671</v>
       </c>
       <c r="V134" t="n">
         <v>1330000</v>
@@ -11424,7 +11424,7 @@
         <v>2010329</v>
       </c>
       <c r="T135" t="n">
-        <v>21356496</v>
+        <v>21356495</v>
       </c>
       <c r="U135" t="n">
         <v>23366824</v>
@@ -11493,7 +11493,7 @@
         <v>2368.5</v>
       </c>
       <c r="P136" t="n">
-        <v>358854.5</v>
+        <v>358854.4</v>
       </c>
       <c r="Q136" t="n">
         <v>8727</v>
@@ -11505,10 +11505,10 @@
         <v>2010329</v>
       </c>
       <c r="T136" t="n">
-        <v>21475513</v>
+        <v>21475511</v>
       </c>
       <c r="U136" t="n">
-        <v>23485842</v>
+        <v>23485840</v>
       </c>
       <c r="V136" t="n">
         <v>1350000</v>
@@ -11586,10 +11586,10 @@
         <v>2010329</v>
       </c>
       <c r="T137" t="n">
-        <v>24908233</v>
+        <v>24908235</v>
       </c>
       <c r="U137" t="n">
-        <v>26918562</v>
+        <v>26918564</v>
       </c>
       <c r="V137" t="n">
         <v>1360000</v>
@@ -11601,7 +11601,7 @@
         <v>54.49</v>
       </c>
       <c r="Y137" t="n">
-        <v>5298659</v>
+        <v>5298658</v>
       </c>
     </row>
     <row r="138">
@@ -11667,10 +11667,10 @@
         <v>2010329</v>
       </c>
       <c r="T138" t="n">
-        <v>25781199</v>
+        <v>25781200</v>
       </c>
       <c r="U138" t="n">
-        <v>27791528</v>
+        <v>27791530</v>
       </c>
       <c r="V138" t="n">
         <v>1370000</v>
@@ -11748,10 +11748,10 @@
         <v>2010329</v>
       </c>
       <c r="T139" t="n">
-        <v>27901227</v>
+        <v>27901224</v>
       </c>
       <c r="U139" t="n">
-        <v>29911556</v>
+        <v>29911553</v>
       </c>
       <c r="V139" t="n">
         <v>1380000</v>
@@ -11763,7 +11763,7 @@
         <v>60.506</v>
       </c>
       <c r="Y139" t="n">
-        <v>5700580</v>
+        <v>5700579</v>
       </c>
     </row>
     <row r="140">
@@ -11844,7 +11844,7 @@
         <v>52.263</v>
       </c>
       <c r="Y140" t="n">
-        <v>5386597</v>
+        <v>5386596</v>
       </c>
     </row>
     <row r="141">
@@ -11910,10 +11910,10 @@
         <v>2010329</v>
       </c>
       <c r="T141" t="n">
-        <v>28743962</v>
+        <v>28743957</v>
       </c>
       <c r="U141" t="n">
-        <v>30754291</v>
+        <v>30754286</v>
       </c>
       <c r="V141" t="n">
         <v>1400000</v>
@@ -11925,7 +11925,7 @@
         <v>62.167</v>
       </c>
       <c r="Y141" t="n">
-        <v>5820189</v>
+        <v>5820188</v>
       </c>
     </row>
     <row r="142">
@@ -11991,10 +11991,10 @@
         <v>2010329</v>
       </c>
       <c r="T142" t="n">
-        <v>34394466</v>
+        <v>34394463</v>
       </c>
       <c r="U142" t="n">
-        <v>36404795</v>
+        <v>36404792</v>
       </c>
       <c r="V142" t="n">
         <v>1410000</v>
@@ -12006,7 +12006,7 @@
         <v>73.568</v>
       </c>
       <c r="Y142" t="n">
-        <v>5946398</v>
+        <v>5946399</v>
       </c>
     </row>
     <row r="143">
@@ -12072,10 +12072,10 @@
         <v>2010329</v>
       </c>
       <c r="T143" t="n">
-        <v>35624100</v>
+        <v>35624097</v>
       </c>
       <c r="U143" t="n">
-        <v>37634429</v>
+        <v>37634427</v>
       </c>
       <c r="V143" t="n">
         <v>1420000</v>
@@ -12153,10 +12153,10 @@
         <v>2010329</v>
       </c>
       <c r="T144" t="n">
-        <v>25169555</v>
+        <v>25169557</v>
       </c>
       <c r="U144" t="n">
-        <v>27179884</v>
+        <v>27179886</v>
       </c>
       <c r="V144" t="n">
         <v>1430000</v>
@@ -12168,7 +12168,7 @@
         <v>54.891</v>
       </c>
       <c r="Y144" t="n">
-        <v>5507900</v>
+        <v>5507902</v>
       </c>
     </row>
     <row r="145">
@@ -12234,10 +12234,10 @@
         <v>2010329</v>
       </c>
       <c r="T145" t="n">
-        <v>22499078</v>
+        <v>22499081</v>
       </c>
       <c r="U145" t="n">
-        <v>24509407</v>
+        <v>24509410</v>
       </c>
       <c r="V145" t="n">
         <v>1440000</v>
@@ -12249,7 +12249,7 @@
         <v>49.478</v>
       </c>
       <c r="Y145" t="n">
-        <v>5271359</v>
+        <v>5271360</v>
       </c>
     </row>
     <row r="146">
@@ -12315,10 +12315,10 @@
         <v>2010329</v>
       </c>
       <c r="T146" t="n">
-        <v>22912706</v>
+        <v>22912703</v>
       </c>
       <c r="U146" t="n">
-        <v>24923035</v>
+        <v>24923032</v>
       </c>
       <c r="V146" t="n">
         <v>1450000</v>
@@ -12330,7 +12330,7 @@
         <v>50.293</v>
       </c>
       <c r="Y146" t="n">
-        <v>5527410</v>
+        <v>5527411</v>
       </c>
     </row>
     <row r="147">
@@ -12396,10 +12396,10 @@
         <v>2010329</v>
       </c>
       <c r="T147" t="n">
-        <v>14270760</v>
+        <v>14270759</v>
       </c>
       <c r="U147" t="n">
-        <v>16281089</v>
+        <v>16281088</v>
       </c>
       <c r="V147" t="n">
         <v>1460000</v>
@@ -12411,7 +12411,7 @@
         <v>32.834</v>
       </c>
       <c r="Y147" t="n">
-        <v>4785908</v>
+        <v>4785907</v>
       </c>
     </row>
     <row r="148">
@@ -12477,10 +12477,10 @@
         <v>2010329</v>
       </c>
       <c r="T148" t="n">
-        <v>14471121</v>
+        <v>14471120</v>
       </c>
       <c r="U148" t="n">
-        <v>16481450</v>
+        <v>16481449</v>
       </c>
       <c r="V148" t="n">
         <v>1470000</v>
@@ -12492,7 +12492,7 @@
         <v>33.218</v>
       </c>
       <c r="Y148" t="n">
-        <v>4719965</v>
+        <v>4719966</v>
       </c>
     </row>
     <row r="149">
@@ -12558,10 +12558,10 @@
         <v>2010329</v>
       </c>
       <c r="T149" t="n">
-        <v>9384856</v>
+        <v>9384857</v>
       </c>
       <c r="U149" t="n">
-        <v>11395185</v>
+        <v>11395187</v>
       </c>
       <c r="V149" t="n">
         <v>1480000</v>
@@ -12639,10 +12639,10 @@
         <v>2010329</v>
       </c>
       <c r="T150" t="n">
-        <v>13127072</v>
+        <v>13127070</v>
       </c>
       <c r="U150" t="n">
-        <v>15137401</v>
+        <v>15137400</v>
       </c>
       <c r="V150" t="n">
         <v>1490000</v>
@@ -12735,7 +12735,7 @@
         <v>24.988</v>
       </c>
       <c r="Y151" t="n">
-        <v>4620958</v>
+        <v>4620959</v>
       </c>
     </row>
     <row r="152">
@@ -12801,10 +12801,10 @@
         <v>2010329</v>
       </c>
       <c r="T152" t="n">
-        <v>7311771</v>
+        <v>7311772</v>
       </c>
       <c r="U152" t="n">
-        <v>9322100</v>
+        <v>9322101</v>
       </c>
       <c r="V152" t="n">
         <v>1510000</v>
@@ -12816,7 +12816,7 @@
         <v>18.724</v>
       </c>
       <c r="Y152" t="n">
-        <v>4144105</v>
+        <v>4144106</v>
       </c>
     </row>
     <row r="153">
@@ -12882,10 +12882,10 @@
         <v>2010329</v>
       </c>
       <c r="T153" t="n">
-        <v>7663586</v>
+        <v>7663587</v>
       </c>
       <c r="U153" t="n">
-        <v>9673915</v>
+        <v>9673916</v>
       </c>
       <c r="V153" t="n">
         <v>1520000</v>
@@ -12897,7 +12897,7 @@
         <v>19.411</v>
       </c>
       <c r="Y153" t="n">
-        <v>4319853</v>
+        <v>4319854</v>
       </c>
     </row>
     <row r="154">
@@ -12966,7 +12966,7 @@
         <v>9716005</v>
       </c>
       <c r="U154" t="n">
-        <v>11726334</v>
+        <v>11726335</v>
       </c>
       <c r="V154" t="n">
         <v>1530000</v>
@@ -12978,7 +12978,7 @@
         <v>23.509</v>
       </c>
       <c r="Y154" t="n">
-        <v>4569343</v>
+        <v>4569342</v>
       </c>
     </row>
     <row r="155">
@@ -13044,7 +13044,7 @@
         <v>2010329</v>
       </c>
       <c r="T155" t="n">
-        <v>7337149</v>
+        <v>7337148</v>
       </c>
       <c r="U155" t="n">
         <v>9347477</v>
@@ -13059,7 +13059,7 @@
         <v>18.72</v>
       </c>
       <c r="Y155" t="n">
-        <v>4167466</v>
+        <v>4167468</v>
       </c>
     </row>
     <row r="156">
@@ -13125,7 +13125,7 @@
         <v>2010329</v>
       </c>
       <c r="T156" t="n">
-        <v>9917836</v>
+        <v>9917835</v>
       </c>
       <c r="U156" t="n">
         <v>11928165</v>
@@ -13206,10 +13206,10 @@
         <v>2010329</v>
       </c>
       <c r="T157" t="n">
-        <v>9837909</v>
+        <v>9837910</v>
       </c>
       <c r="U157" t="n">
-        <v>11848238</v>
+        <v>11848239</v>
       </c>
       <c r="V157" t="n">
         <v>1560000</v>
@@ -13221,7 +13221,7 @@
         <v>23.688</v>
       </c>
       <c r="Y157" t="n">
-        <v>4614362</v>
+        <v>4614363</v>
       </c>
     </row>
     <row r="158">
@@ -13290,7 +13290,7 @@
         <v>12157915</v>
       </c>
       <c r="U158" t="n">
-        <v>14168243</v>
+        <v>14168244</v>
       </c>
       <c r="V158" t="n">
         <v>1570000</v>
@@ -13371,7 +13371,7 @@
         <v>10941510</v>
       </c>
       <c r="U159" t="n">
-        <v>12951838</v>
+        <v>12951839</v>
       </c>
       <c r="V159" t="n">
         <v>1580000</v>
@@ -13449,10 +13449,10 @@
         <v>2010329</v>
       </c>
       <c r="T160" t="n">
-        <v>14306485</v>
+        <v>14306486</v>
       </c>
       <c r="U160" t="n">
-        <v>16316814</v>
+        <v>16316816</v>
       </c>
       <c r="V160" t="n">
         <v>1590000</v>
@@ -13464,7 +13464,7 @@
         <v>32.554</v>
       </c>
       <c r="Y160" t="n">
-        <v>5509996</v>
+        <v>5509995</v>
       </c>
     </row>
     <row r="161">
@@ -13530,10 +13530,10 @@
         <v>2020329</v>
       </c>
       <c r="T161" t="n">
-        <v>16604859</v>
+        <v>16604858</v>
       </c>
       <c r="U161" t="n">
-        <v>18625188</v>
+        <v>18625187</v>
       </c>
       <c r="V161" t="n">
         <v>1600000</v>
@@ -13611,10 +13611,10 @@
         <v>2020329</v>
       </c>
       <c r="T162" t="n">
-        <v>18501853</v>
+        <v>18501854</v>
       </c>
       <c r="U162" t="n">
-        <v>20522182</v>
+        <v>20522184</v>
       </c>
       <c r="V162" t="n">
         <v>1610000</v>
@@ -13707,7 +13707,7 @@
         <v>37.208</v>
       </c>
       <c r="Y163" t="n">
-        <v>6023272</v>
+        <v>6023273</v>
       </c>
     </row>
     <row r="164">
@@ -13776,7 +13776,7 @@
         <v>13929153</v>
       </c>
       <c r="U164" t="n">
-        <v>15949482</v>
+        <v>15949483</v>
       </c>
       <c r="V164" t="n">
         <v>1630000</v>
@@ -13842,7 +13842,7 @@
         <v>2632.1</v>
       </c>
       <c r="P165" t="n">
-        <v>361685.9</v>
+        <v>361685.8</v>
       </c>
       <c r="Q165" t="n">
         <v>9431.200000000001</v>
@@ -13854,10 +13854,10 @@
         <v>2020329</v>
       </c>
       <c r="T165" t="n">
-        <v>12230111</v>
+        <v>12230112</v>
       </c>
       <c r="U165" t="n">
-        <v>14250440</v>
+        <v>14250441</v>
       </c>
       <c r="V165" t="n">
         <v>1640000</v>
@@ -13869,7 +13869,7 @@
         <v>28.35</v>
       </c>
       <c r="Y165" t="n">
-        <v>5618981</v>
+        <v>5618982</v>
       </c>
     </row>
     <row r="166">
@@ -13935,10 +13935,10 @@
         <v>2020329</v>
       </c>
       <c r="T166" t="n">
-        <v>16752394</v>
+        <v>16752395</v>
       </c>
       <c r="U166" t="n">
-        <v>18772723</v>
+        <v>18772725</v>
       </c>
       <c r="V166" t="n">
         <v>1650000</v>
@@ -14016,10 +14016,10 @@
         <v>4716204</v>
       </c>
       <c r="T167" t="n">
-        <v>17985073</v>
+        <v>17985074</v>
       </c>
       <c r="U167" t="n">
-        <v>22701277</v>
+        <v>22701278</v>
       </c>
       <c r="V167" t="n">
         <v>1660000</v>
@@ -14085,7 +14085,7 @@
         <v>2632.1</v>
       </c>
       <c r="P168" t="n">
-        <v>326124.3</v>
+        <v>326124.2</v>
       </c>
       <c r="Q168" t="n">
         <v>9431.200000000001</v>
@@ -14097,7 +14097,7 @@
         <v>4716204</v>
       </c>
       <c r="T168" t="n">
-        <v>18586961</v>
+        <v>18586959</v>
       </c>
       <c r="U168" t="n">
         <v>23303164</v>
@@ -14166,7 +14166,7 @@
         <v>2632.1</v>
       </c>
       <c r="P169" t="n">
-        <v>326293.8</v>
+        <v>326293.7</v>
       </c>
       <c r="Q169" t="n">
         <v>9431.200000000001</v>
@@ -14178,10 +14178,10 @@
         <v>4716204</v>
       </c>
       <c r="T169" t="n">
-        <v>22597310</v>
+        <v>22597309</v>
       </c>
       <c r="U169" t="n">
-        <v>27313514</v>
+        <v>27313513</v>
       </c>
       <c r="V169" t="n">
         <v>1680000</v>
@@ -14259,10 +14259,10 @@
         <v>4716204</v>
       </c>
       <c r="T170" t="n">
-        <v>23828267</v>
+        <v>23828268</v>
       </c>
       <c r="U170" t="n">
-        <v>28544471</v>
+        <v>28544472</v>
       </c>
       <c r="V170" t="n">
         <v>1690000</v>
@@ -14328,7 +14328,7 @@
         <v>2632.1</v>
       </c>
       <c r="P171" t="n">
-        <v>326652.7</v>
+        <v>326652.6</v>
       </c>
       <c r="Q171" t="n">
         <v>9431.200000000001</v>
@@ -14421,10 +14421,10 @@
         <v>4716204</v>
       </c>
       <c r="T172" t="n">
-        <v>24642705</v>
+        <v>24642707</v>
       </c>
       <c r="U172" t="n">
-        <v>29358909</v>
+        <v>29358911</v>
       </c>
       <c r="V172" t="n">
         <v>1710000</v>
@@ -14502,10 +14502,10 @@
         <v>4716204</v>
       </c>
       <c r="T173" t="n">
-        <v>28368035</v>
+        <v>28368036</v>
       </c>
       <c r="U173" t="n">
-        <v>33084239</v>
+        <v>33084240</v>
       </c>
       <c r="V173" t="n">
         <v>1720000</v>
@@ -14517,7 +14517,7 @@
         <v>65.61799999999999</v>
       </c>
       <c r="Y173" t="n">
-        <v>7803713</v>
+        <v>7803714</v>
       </c>
     </row>
     <row r="174">
@@ -14583,10 +14583,10 @@
         <v>4716204</v>
       </c>
       <c r="T174" t="n">
-        <v>24799953</v>
+        <v>24799955</v>
       </c>
       <c r="U174" t="n">
-        <v>29516156</v>
+        <v>29516159</v>
       </c>
       <c r="V174" t="n">
         <v>1730000</v>
@@ -14637,7 +14637,7 @@
         <v>0</v>
       </c>
       <c r="K175" t="n">
-        <v>471.84</v>
+        <v>471.85</v>
       </c>
       <c r="L175" t="n">
         <v>33.75</v>
@@ -14679,7 +14679,7 @@
         <v>56.018</v>
       </c>
       <c r="Y175" t="n">
-        <v>7777545</v>
+        <v>7777546</v>
       </c>
     </row>
     <row r="176">
@@ -14745,7 +14745,7 @@
         <v>4716204</v>
       </c>
       <c r="T176" t="n">
-        <v>23797033</v>
+        <v>23797032</v>
       </c>
       <c r="U176" t="n">
         <v>28513236</v>
@@ -14826,10 +14826,10 @@
         <v>4716204</v>
       </c>
       <c r="T177" t="n">
-        <v>21739845</v>
+        <v>21739846</v>
       </c>
       <c r="U177" t="n">
-        <v>26456049</v>
+        <v>26456050</v>
       </c>
       <c r="V177" t="n">
         <v>1760000</v>
@@ -14910,7 +14910,7 @@
         <v>23037207</v>
       </c>
       <c r="U178" t="n">
-        <v>27753410</v>
+        <v>27753411</v>
       </c>
       <c r="V178" t="n">
         <v>1770000</v>
@@ -14922,7 +14922,7 @@
         <v>54.947</v>
       </c>
       <c r="Y178" t="n">
-        <v>8366760</v>
+        <v>8366761</v>
       </c>
     </row>
     <row r="179">
@@ -15003,7 +15003,7 @@
         <v>54.511</v>
       </c>
       <c r="Y179" t="n">
-        <v>8414739</v>
+        <v>8414738</v>
       </c>
     </row>
     <row r="180">
@@ -15057,7 +15057,7 @@
         <v>2642.5</v>
       </c>
       <c r="P180" t="n">
-        <v>327765.9</v>
+        <v>327765.8</v>
       </c>
       <c r="Q180" t="n">
         <v>9452</v>
@@ -15069,10 +15069,10 @@
         <v>4716204</v>
       </c>
       <c r="T180" t="n">
-        <v>23394495</v>
+        <v>23394493</v>
       </c>
       <c r="U180" t="n">
-        <v>28110698</v>
+        <v>28110697</v>
       </c>
       <c r="V180" t="n">
         <v>1790000</v>
@@ -15144,7 +15144,7 @@
         <v>9452</v>
       </c>
       <c r="R181" t="n">
-        <v>235092.5</v>
+        <v>235092.6</v>
       </c>
       <c r="S181" t="n">
         <v>4716204</v>
@@ -15225,13 +15225,13 @@
         <v>9475.700000000001</v>
       </c>
       <c r="R182" t="n">
-        <v>235092.5</v>
+        <v>235092.6</v>
       </c>
       <c r="S182" t="n">
         <v>4716204</v>
       </c>
       <c r="T182" t="n">
-        <v>16301703</v>
+        <v>16301702</v>
       </c>
       <c r="U182" t="n">
         <v>21017906</v>
@@ -15306,7 +15306,7 @@
         <v>9499.4</v>
       </c>
       <c r="R183" t="n">
-        <v>235092.5</v>
+        <v>235092.6</v>
       </c>
       <c r="S183" t="n">
         <v>4716204</v>
@@ -15387,13 +15387,13 @@
         <v>9520.299999999999</v>
       </c>
       <c r="R184" t="n">
-        <v>235092.5</v>
+        <v>235092.6</v>
       </c>
       <c r="S184" t="n">
         <v>4716204</v>
       </c>
       <c r="T184" t="n">
-        <v>18841733</v>
+        <v>18841732</v>
       </c>
       <c r="U184" t="n">
         <v>23557936</v>
@@ -15477,7 +15477,7 @@
         <v>23578764</v>
       </c>
       <c r="U185" t="n">
-        <v>28294967</v>
+        <v>28294968</v>
       </c>
       <c r="V185" t="n">
         <v>1840000</v>
@@ -15549,7 +15549,7 @@
         <v>9520.299999999999</v>
       </c>
       <c r="R186" t="n">
-        <v>235491.5</v>
+        <v>235491.6</v>
       </c>
       <c r="S186" t="n">
         <v>4716204</v>
@@ -15636,7 +15636,7 @@
         <v>4716204</v>
       </c>
       <c r="T187" t="n">
-        <v>25014802</v>
+        <v>25014801</v>
       </c>
       <c r="U187" t="n">
         <v>29731005</v>
@@ -15798,10 +15798,10 @@
         <v>4716204</v>
       </c>
       <c r="T189" t="n">
-        <v>35501262</v>
+        <v>35501261</v>
       </c>
       <c r="U189" t="n">
-        <v>40217465</v>
+        <v>40217466</v>
       </c>
       <c r="V189" t="n">
         <v>1880000</v>
@@ -15867,7 +15867,7 @@
         <v>2673.4</v>
       </c>
       <c r="P190" t="n">
-        <v>328522.1</v>
+        <v>328522</v>
       </c>
       <c r="Q190" t="n">
         <v>9520.299999999999</v>
@@ -15879,7 +15879,7 @@
         <v>4716204</v>
       </c>
       <c r="T190" t="n">
-        <v>32594289</v>
+        <v>32594288</v>
       </c>
       <c r="U190" t="n">
         <v>37310492</v>
@@ -15948,7 +15948,7 @@
         <v>2673.4</v>
       </c>
       <c r="P191" t="n">
-        <v>328617</v>
+        <v>328616.9</v>
       </c>
       <c r="Q191" t="n">
         <v>9520.299999999999</v>
@@ -16038,13 +16038,13 @@
         <v>189017.8</v>
       </c>
       <c r="S192" t="n">
-        <v>9401720</v>
+        <v>9401721</v>
       </c>
       <c r="T192" t="n">
         <v>33130320</v>
       </c>
       <c r="U192" t="n">
-        <v>42532040</v>
+        <v>42532041</v>
       </c>
       <c r="V192" t="n">
         <v>1910000</v>
@@ -16119,13 +16119,13 @@
         <v>189097.4</v>
       </c>
       <c r="S193" t="n">
-        <v>9401720</v>
+        <v>9401721</v>
       </c>
       <c r="T193" t="n">
         <v>31991112</v>
       </c>
       <c r="U193" t="n">
-        <v>41392832</v>
+        <v>41392833</v>
       </c>
       <c r="V193" t="n">
         <v>1920000</v>
@@ -16200,13 +16200,13 @@
         <v>189097.4</v>
       </c>
       <c r="S194" t="n">
-        <v>9401720</v>
+        <v>9401721</v>
       </c>
       <c r="T194" t="n">
         <v>26597931</v>
       </c>
       <c r="U194" t="n">
-        <v>35999651</v>
+        <v>35999652</v>
       </c>
       <c r="V194" t="n">
         <v>1930000</v>
@@ -16281,10 +16281,10 @@
         <v>189136.7</v>
       </c>
       <c r="S195" t="n">
-        <v>9401720</v>
+        <v>9401721</v>
       </c>
       <c r="T195" t="n">
-        <v>49447839</v>
+        <v>49447838</v>
       </c>
       <c r="U195" t="n">
         <v>58849559</v>
@@ -16443,10 +16443,10 @@
         <v>121047.5</v>
       </c>
       <c r="S197" t="n">
-        <v>27852893</v>
+        <v>27852894</v>
       </c>
       <c r="T197" t="n">
-        <v>46944175</v>
+        <v>46944174</v>
       </c>
       <c r="U197" t="n">
         <v>74797068</v>
@@ -16475,11 +16475,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16490,7 +16494,27 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Value</t>
+          <t>Adaptive strategy</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>B&amp;H QQQ</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>B&amp;H TQQQ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>B&amp;H SMH</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>B&amp;H SOXL</t>
         </is>
       </c>
     </row>
@@ -16505,6 +16529,10 @@
           <t>2010-03-31 → 2026-06-30 (16.2 yrs, 196 months)</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -16517,6 +16545,10 @@
           <t>$10,000</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -16529,230 +16561,462 @@
           <t>$1,960,000</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>METRIC</t>
+          <t>Final NAV</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ADAPTIVE STRATEGY  |  BUY &amp; HOLD QQQ</t>
+          <t>$74,797,068</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>$11,898,665</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>$101,660,685</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>$34,886,610</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>$205,415,389</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Final NAV</t>
+          <t>Total profit</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$74,797,068   |   $11,898,665</t>
+          <t>$72,837,068</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>$9,938,665</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>$99,700,685</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>$32,926,610</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>$203,455,389</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Total profit (NAV − contributed)</t>
+          <t>Multiple on invested</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>$72,837,068   |   $9,938,665</t>
+          <t>38.16x</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>6.07x</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>51.87x</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>17.8x</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>104.8x</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Multiple on invested</t>
+          <t>Time-weighted CAGR</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>38.16x   |   6.07x</t>
+          <t>36.0%/yr</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>19.0%/yr</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>41.0%/yr</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>26.9%/yr</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>41.6%/yr</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Time-weighted CAGR</t>
+          <t>Money-weighted IRR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>36.0%/yr   |   18.8%/yr</t>
+          <t>38.3%/yr</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>19.6%/yr</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>41.5%/yr</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>30.5%/yr</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>49.0%/yr</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Money-weighted IRR</t>
+          <t>Investment Sharpe (equal-wt)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>38.3%/yr   |   19.6%/yr</t>
+          <t>0.86</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1.08</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.08</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0.79</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Investment Sharpe (equal-wt)</t>
+          <t>Contribution Sharpe (capital-wt)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.86   |   1.09</t>
+          <t>0.67</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0.61</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1.29</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.64</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Contribution Sharpe (capital-wt)</t>
+          <t>Sortino</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0.67   |   1.01</t>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1.17</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1.23</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>1.04</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sortino</t>
+          <t>Max drawdown (time-weighted)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0.94   |   1.19</t>
+          <t>-75.4%</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>-32.6%</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>-79.1%</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>-40.0%</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>-86.9%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Max drawdown (time-weighted)</t>
+          <t>Win rate (positive months)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>-75.4%   |   -32.5%</t>
+          <t>62%</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>63%</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>61%</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>64%</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>56%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Win rate (positive months)</t>
+          <t>Best month</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>62%   |   63%</t>
+          <t>63.4%</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>15.7%</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>52.4%</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>32.2%</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>165.0%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Best / worst month</t>
+          <t>Worst month</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>63.4% / -43.2%   |   15.7% / -13.6%</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Growth = $ from market</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>$72,837,068 (97.4% of final NAV)</t>
-        </is>
+          <t>-43.2%</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>-13.6%</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>-38.1%</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>-16.7%</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>-53.7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>Regime</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>Months</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>bull</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>132</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>Regime</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
-        <is>
-          <t>Months</t>
-        </is>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>chop</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>58</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>bull</t>
+          <t>fear1</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>132</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>chop</t>
+          <t>euphoria</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>58</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>fear1</t>
+          <t>fear2</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>euphoria</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>fear2</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
         <v>1</v>
       </c>
     </row>
@@ -16770,8 +17034,8 @@
   <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Backtest: fully-invested apples-to-apples mode (no cash/no sells) vs B&H
</commit_message>
<xml_diff>
--- a/backtest.xlsx
+++ b/backtest.xlsx
@@ -454,7 +454,7 @@
     <col width="9" customWidth="1" min="18" max="18"/>
     <col width="9" customWidth="1" min="19" max="19"/>
     <col width="15" customWidth="1" min="20" max="20"/>
-    <col width="9" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="14" customWidth="1" min="23" max="23"/>
     <col width="10" customWidth="1" min="24" max="24"/>
@@ -3075,7 +3075,7 @@
         <v>6375.7</v>
       </c>
       <c r="R32" t="n">
-        <v>131676.4</v>
+        <v>131676.3</v>
       </c>
       <c r="S32" t="n">
         <v>0</v>
@@ -3312,7 +3312,7 @@
         <v>1744.2</v>
       </c>
       <c r="P35" t="n">
-        <v>207458.3</v>
+        <v>207458.2</v>
       </c>
       <c r="Q35" t="n">
         <v>6375.7</v>
@@ -3399,7 +3399,7 @@
         <v>6375.7</v>
       </c>
       <c r="R36" t="n">
-        <v>180876.6</v>
+        <v>180876.5</v>
       </c>
       <c r="S36" t="n">
         <v>0</v>
@@ -3486,10 +3486,10 @@
         <v>0</v>
       </c>
       <c r="T37" t="n">
-        <v>434751</v>
+        <v>434750</v>
       </c>
       <c r="U37" t="n">
-        <v>434751</v>
+        <v>434750</v>
       </c>
       <c r="V37" t="n">
         <v>360000</v>
@@ -3561,7 +3561,7 @@
         <v>6375.7</v>
       </c>
       <c r="R38" t="n">
-        <v>198183.3</v>
+        <v>198183.2</v>
       </c>
       <c r="S38" t="n">
         <v>0</v>
@@ -3744,7 +3744,7 @@
         <v>1.715</v>
       </c>
       <c r="Y40" t="n">
-        <v>503927</v>
+        <v>503926</v>
       </c>
     </row>
     <row r="41">
@@ -4041,7 +4041,7 @@
         <v>1744.2</v>
       </c>
       <c r="P44" t="n">
-        <v>274317.8</v>
+        <v>274317.7</v>
       </c>
       <c r="Q44" t="n">
         <v>6375.7</v>
@@ -4068,7 +4068,7 @@
         <v>1.957</v>
       </c>
       <c r="Y44" t="n">
-        <v>587994</v>
+        <v>587993</v>
       </c>
     </row>
     <row r="45">
@@ -4149,7 +4149,7 @@
         <v>2.141</v>
       </c>
       <c r="Y45" t="n">
-        <v>627129</v>
+        <v>627130</v>
       </c>
     </row>
     <row r="46">
@@ -4215,10 +4215,10 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>798005</v>
+        <v>798004</v>
       </c>
       <c r="U46" t="n">
-        <v>798005</v>
+        <v>798004</v>
       </c>
       <c r="V46" t="n">
         <v>450000</v>
@@ -4620,10 +4620,10 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>974913</v>
+        <v>974912</v>
       </c>
       <c r="U51" t="n">
-        <v>974913</v>
+        <v>974912</v>
       </c>
       <c r="V51" t="n">
         <v>500000</v>
@@ -4770,7 +4770,7 @@
         <v>1744.2</v>
       </c>
       <c r="P53" t="n">
-        <v>311064.9</v>
+        <v>311064.8</v>
       </c>
       <c r="Q53" t="n">
         <v>6375.7</v>
@@ -4959,7 +4959,7 @@
         <v>3.558</v>
       </c>
       <c r="Y55" t="n">
-        <v>876003</v>
+        <v>876002</v>
       </c>
     </row>
     <row r="56">
@@ -5013,7 +5013,7 @@
         <v>1744.2</v>
       </c>
       <c r="P56" t="n">
-        <v>320066.2</v>
+        <v>320066.1</v>
       </c>
       <c r="Q56" t="n">
         <v>6375.7</v>
@@ -5187,10 +5187,10 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>1607746</v>
+        <v>1607745</v>
       </c>
       <c r="U58" t="n">
-        <v>1607746</v>
+        <v>1607745</v>
       </c>
       <c r="V58" t="n">
         <v>570000</v>
@@ -5430,10 +5430,10 @@
         <v>0</v>
       </c>
       <c r="T61" t="n">
-        <v>1756344</v>
+        <v>1756343</v>
       </c>
       <c r="U61" t="n">
-        <v>1756344</v>
+        <v>1756343</v>
       </c>
       <c r="V61" t="n">
         <v>600000</v>
@@ -5526,7 +5526,7 @@
         <v>4.049</v>
       </c>
       <c r="Y62" t="n">
-        <v>1006577</v>
+        <v>1006576</v>
       </c>
     </row>
     <row r="63">
@@ -5607,7 +5607,7 @@
         <v>4.082</v>
       </c>
       <c r="Y63" t="n">
-        <v>1035916</v>
+        <v>1035917</v>
       </c>
     </row>
     <row r="64">
@@ -5688,7 +5688,7 @@
         <v>4.634</v>
       </c>
       <c r="Y64" t="n">
-        <v>1069199</v>
+        <v>1069198</v>
       </c>
     </row>
     <row r="65">
@@ -6255,7 +6255,7 @@
         <v>3.921</v>
       </c>
       <c r="Y71" t="n">
-        <v>1167297</v>
+        <v>1167298</v>
       </c>
     </row>
     <row r="72">
@@ -6336,7 +6336,7 @@
         <v>3.192</v>
       </c>
       <c r="Y72" t="n">
-        <v>1096623</v>
+        <v>1096622</v>
       </c>
     </row>
     <row r="73">
@@ -6645,10 +6645,10 @@
         <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>1726273</v>
+        <v>1726274</v>
       </c>
       <c r="U76" t="n">
-        <v>1726273</v>
+        <v>1726274</v>
       </c>
       <c r="V76" t="n">
         <v>750000</v>
@@ -6741,7 +6741,7 @@
         <v>3.694</v>
       </c>
       <c r="Y77" t="n">
-        <v>1189266</v>
+        <v>1189265</v>
       </c>
     </row>
     <row r="78">
@@ -6822,7 +6822,7 @@
         <v>4.553</v>
       </c>
       <c r="Y78" t="n">
-        <v>1284297</v>
+        <v>1284298</v>
       </c>
     </row>
     <row r="79">
@@ -6984,7 +6984,7 @@
         <v>5.255</v>
       </c>
       <c r="Y80" t="n">
-        <v>1346712</v>
+        <v>1346711</v>
       </c>
     </row>
     <row r="81">
@@ -7050,10 +7050,10 @@
         <v>0</v>
       </c>
       <c r="T81" t="n">
-        <v>2284299</v>
+        <v>2284298</v>
       </c>
       <c r="U81" t="n">
-        <v>2284299</v>
+        <v>2284298</v>
       </c>
       <c r="V81" t="n">
         <v>800000</v>
@@ -7065,7 +7065,7 @@
         <v>5.04</v>
       </c>
       <c r="Y81" t="n">
-        <v>1337077</v>
+        <v>1337078</v>
       </c>
     </row>
     <row r="82">
@@ -7293,10 +7293,10 @@
         <v>0</v>
       </c>
       <c r="T84" t="n">
-        <v>2968225</v>
+        <v>2968224</v>
       </c>
       <c r="U84" t="n">
-        <v>2968225</v>
+        <v>2968224</v>
       </c>
       <c r="V84" t="n">
         <v>830000</v>
@@ -7611,7 +7611,7 @@
         <v>7882.7</v>
       </c>
       <c r="R88" t="n">
-        <v>342207.6</v>
+        <v>342207.5</v>
       </c>
       <c r="S88" t="n">
         <v>0</v>
@@ -7632,7 +7632,7 @@
         <v>9.215999999999999</v>
       </c>
       <c r="Y88" t="n">
-        <v>1700222</v>
+        <v>1700221</v>
       </c>
     </row>
     <row r="89">
@@ -7698,10 +7698,10 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>3798192</v>
+        <v>3798193</v>
       </c>
       <c r="U89" t="n">
-        <v>3798192</v>
+        <v>3798193</v>
       </c>
       <c r="V89" t="n">
         <v>880000</v>
@@ -7713,7 +7713,7 @@
         <v>8.175000000000001</v>
       </c>
       <c r="Y89" t="n">
-        <v>1670801</v>
+        <v>1670802</v>
       </c>
     </row>
     <row r="90">
@@ -7794,7 +7794,7 @@
         <v>9.17</v>
       </c>
       <c r="Y90" t="n">
-        <v>1748649</v>
+        <v>1748648</v>
       </c>
     </row>
     <row r="91">
@@ -7854,7 +7854,7 @@
         <v>7882.7</v>
       </c>
       <c r="R91" t="n">
-        <v>344800.7</v>
+        <v>344800.6</v>
       </c>
       <c r="S91" t="n">
         <v>0</v>
@@ -7935,7 +7935,7 @@
         <v>7882.7</v>
       </c>
       <c r="R92" t="n">
-        <v>345482.5</v>
+        <v>345482.4</v>
       </c>
       <c r="S92" t="n">
         <v>0</v>
@@ -7956,7 +7956,7 @@
         <v>10.414</v>
       </c>
       <c r="Y92" t="n">
-        <v>1799588</v>
+        <v>1799589</v>
       </c>
     </row>
     <row r="93">
@@ -8022,10 +8022,10 @@
         <v>0</v>
       </c>
       <c r="T93" t="n">
-        <v>5877482</v>
+        <v>5877481</v>
       </c>
       <c r="U93" t="n">
-        <v>5877482</v>
+        <v>5877481</v>
       </c>
       <c r="V93" t="n">
         <v>920000</v>
@@ -8037,7 +8037,7 @@
         <v>12.545</v>
       </c>
       <c r="Y93" t="n">
-        <v>1892475</v>
+        <v>1892474</v>
       </c>
     </row>
     <row r="94">
@@ -8103,10 +8103,10 @@
         <v>0</v>
       </c>
       <c r="T94" t="n">
-        <v>5946258</v>
+        <v>5946259</v>
       </c>
       <c r="U94" t="n">
-        <v>5946258</v>
+        <v>5946259</v>
       </c>
       <c r="V94" t="n">
         <v>930000</v>
@@ -8184,10 +8184,10 @@
         <v>0</v>
       </c>
       <c r="T95" t="n">
-        <v>5809421</v>
+        <v>5809422</v>
       </c>
       <c r="U95" t="n">
-        <v>5809421</v>
+        <v>5809422</v>
       </c>
       <c r="V95" t="n">
         <v>940000</v>
@@ -8346,10 +8346,10 @@
         <v>0</v>
       </c>
       <c r="T97" t="n">
-        <v>6984218</v>
+        <v>6984217</v>
       </c>
       <c r="U97" t="n">
-        <v>6984218</v>
+        <v>6984217</v>
       </c>
       <c r="V97" t="n">
         <v>960000</v>
@@ -8427,10 +8427,10 @@
         <v>0</v>
       </c>
       <c r="T98" t="n">
-        <v>6277671</v>
+        <v>6277670</v>
       </c>
       <c r="U98" t="n">
-        <v>6277671</v>
+        <v>6277670</v>
       </c>
       <c r="V98" t="n">
         <v>970000</v>
@@ -8508,10 +8508,10 @@
         <v>0</v>
       </c>
       <c r="T99" t="n">
-        <v>5568498</v>
+        <v>5568499</v>
       </c>
       <c r="U99" t="n">
-        <v>5568498</v>
+        <v>5568499</v>
       </c>
       <c r="V99" t="n">
         <v>980000</v>
@@ -8589,10 +8589,10 @@
         <v>0</v>
       </c>
       <c r="T100" t="n">
-        <v>6966364</v>
+        <v>6966365</v>
       </c>
       <c r="U100" t="n">
-        <v>6966364</v>
+        <v>6966365</v>
       </c>
       <c r="V100" t="n">
         <v>990000</v>
@@ -8751,10 +8751,10 @@
         <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>7078886</v>
+        <v>7078887</v>
       </c>
       <c r="U102" t="n">
-        <v>7078886</v>
+        <v>7078887</v>
       </c>
       <c r="V102" t="n">
         <v>1010000</v>
@@ -8766,7 +8766,7 @@
         <v>14.9</v>
       </c>
       <c r="Y102" t="n">
-        <v>2304064</v>
+        <v>2304065</v>
       </c>
     </row>
     <row r="103">
@@ -8913,10 +8913,10 @@
         <v>0</v>
       </c>
       <c r="T104" t="n">
-        <v>7517180</v>
+        <v>7517179</v>
       </c>
       <c r="U104" t="n">
-        <v>7517180</v>
+        <v>7517179</v>
       </c>
       <c r="V104" t="n">
         <v>1030000</v>
@@ -9009,7 +9009,7 @@
         <v>11.231</v>
       </c>
       <c r="Y105" t="n">
-        <v>2249708</v>
+        <v>2249709</v>
       </c>
     </row>
     <row r="106">
@@ -9075,10 +9075,10 @@
         <v>0</v>
       </c>
       <c r="T106" t="n">
-        <v>5453669</v>
+        <v>5453668</v>
       </c>
       <c r="U106" t="n">
-        <v>5453669</v>
+        <v>5453668</v>
       </c>
       <c r="V106" t="n">
         <v>1050000</v>
@@ -9225,7 +9225,7 @@
         <v>2168.3</v>
       </c>
       <c r="P108" t="n">
-        <v>388478.9</v>
+        <v>388478.8</v>
       </c>
       <c r="Q108" t="n">
         <v>8118</v>
@@ -9318,10 +9318,10 @@
         <v>0</v>
       </c>
       <c r="T109" t="n">
-        <v>6004059</v>
+        <v>6004060</v>
       </c>
       <c r="U109" t="n">
-        <v>6004059</v>
+        <v>6004060</v>
       </c>
       <c r="V109" t="n">
         <v>1080000</v>
@@ -9414,7 +9414,7 @@
         <v>13.603</v>
       </c>
       <c r="Y110" t="n">
-        <v>2444585</v>
+        <v>2444586</v>
       </c>
     </row>
     <row r="111">
@@ -9474,7 +9474,7 @@
         <v>8118</v>
       </c>
       <c r="R111" t="n">
-        <v>354751.3</v>
+        <v>354751.2</v>
       </c>
       <c r="S111" t="n">
         <v>0</v>
@@ -9642,10 +9642,10 @@
         <v>0</v>
       </c>
       <c r="T113" t="n">
-        <v>7101971</v>
+        <v>7101969</v>
       </c>
       <c r="U113" t="n">
-        <v>7101971</v>
+        <v>7101969</v>
       </c>
       <c r="V113" t="n">
         <v>1120000</v>
@@ -9723,10 +9723,10 @@
         <v>0</v>
       </c>
       <c r="T114" t="n">
-        <v>7877043</v>
+        <v>7877044</v>
       </c>
       <c r="U114" t="n">
-        <v>7877043</v>
+        <v>7877044</v>
       </c>
       <c r="V114" t="n">
         <v>1130000</v>
@@ -9738,7 +9738,7 @@
         <v>16.261</v>
       </c>
       <c r="Y114" t="n">
-        <v>2647302</v>
+        <v>2647303</v>
       </c>
     </row>
     <row r="115">
@@ -9885,10 +9885,10 @@
         <v>0</v>
       </c>
       <c r="T116" t="n">
-        <v>7674558</v>
+        <v>7674557</v>
       </c>
       <c r="U116" t="n">
-        <v>7674558</v>
+        <v>7674557</v>
       </c>
       <c r="V116" t="n">
         <v>1150000</v>
@@ -10062,7 +10062,7 @@
         <v>19.97</v>
       </c>
       <c r="Y118" t="n">
-        <v>2889163</v>
+        <v>2889164</v>
       </c>
     </row>
     <row r="119">
@@ -10128,10 +10128,10 @@
         <v>0</v>
       </c>
       <c r="T119" t="n">
-        <v>11444855</v>
+        <v>11444853</v>
       </c>
       <c r="U119" t="n">
-        <v>11444855</v>
+        <v>11444853</v>
       </c>
       <c r="V119" t="n">
         <v>1180000</v>
@@ -10209,10 +10209,10 @@
         <v>0</v>
       </c>
       <c r="T120" t="n">
-        <v>11066393</v>
+        <v>11066394</v>
       </c>
       <c r="U120" t="n">
-        <v>11066393</v>
+        <v>11066394</v>
       </c>
       <c r="V120" t="n">
         <v>1190000</v>
@@ -10290,10 +10290,10 @@
         <v>0</v>
       </c>
       <c r="T121" t="n">
-        <v>9345549</v>
+        <v>9345551</v>
       </c>
       <c r="U121" t="n">
-        <v>9345549</v>
+        <v>9345551</v>
       </c>
       <c r="V121" t="n">
         <v>1200000</v>
@@ -10446,16 +10446,16 @@
         <v>8118</v>
       </c>
       <c r="R123" t="n">
-        <v>360538</v>
+        <v>360537.9</v>
       </c>
       <c r="S123" t="n">
         <v>0</v>
       </c>
       <c r="T123" t="n">
-        <v>7350995</v>
+        <v>7350994</v>
       </c>
       <c r="U123" t="n">
-        <v>7350995</v>
+        <v>7350994</v>
       </c>
       <c r="V123" t="n">
         <v>1220000</v>
@@ -10527,16 +10527,16 @@
         <v>8191.6</v>
       </c>
       <c r="R124" t="n">
-        <v>360538</v>
+        <v>360537.9</v>
       </c>
       <c r="S124" t="n">
         <v>0</v>
       </c>
       <c r="T124" t="n">
-        <v>8576082</v>
+        <v>8576081</v>
       </c>
       <c r="U124" t="n">
-        <v>8576082</v>
+        <v>8576081</v>
       </c>
       <c r="V124" t="n">
         <v>1230000</v>
@@ -10548,7 +10548,7 @@
         <v>17.49</v>
       </c>
       <c r="Y124" t="n">
-        <v>3367287</v>
+        <v>3367286</v>
       </c>
     </row>
     <row r="125">
@@ -10608,16 +10608,16 @@
         <v>8259.4</v>
       </c>
       <c r="R125" t="n">
-        <v>360538</v>
+        <v>360537.9</v>
       </c>
       <c r="S125" t="n">
         <v>0</v>
       </c>
       <c r="T125" t="n">
-        <v>10167703</v>
+        <v>10167702</v>
       </c>
       <c r="U125" t="n">
-        <v>10167703</v>
+        <v>10167702</v>
       </c>
       <c r="V125" t="n">
         <v>1240000</v>
@@ -10689,16 +10689,16 @@
         <v>8321.799999999999</v>
       </c>
       <c r="R126" t="n">
-        <v>360538</v>
+        <v>360537.9</v>
       </c>
       <c r="S126" t="n">
         <v>0</v>
       </c>
       <c r="T126" t="n">
-        <v>12195955</v>
+        <v>12195954</v>
       </c>
       <c r="U126" t="n">
-        <v>12195955</v>
+        <v>12195954</v>
       </c>
       <c r="V126" t="n">
         <v>1250000</v>
@@ -10710,7 +10710,7 @@
         <v>24.828</v>
       </c>
       <c r="Y126" t="n">
-        <v>3862621</v>
+        <v>3862622</v>
       </c>
     </row>
     <row r="127">
@@ -10743,10 +10743,10 @@
         <v>0</v>
       </c>
       <c r="I127" t="n">
-        <v>767294</v>
+        <v>0</v>
       </c>
       <c r="J127" t="n">
-        <v>1245048</v>
+        <v>0</v>
       </c>
       <c r="K127" t="n">
         <v>285.28</v>
@@ -10764,22 +10764,22 @@
         <v>2248.2</v>
       </c>
       <c r="P127" t="n">
-        <v>358456.2</v>
+        <v>398284.7</v>
       </c>
       <c r="Q127" t="n">
         <v>8380.9</v>
       </c>
       <c r="R127" t="n">
-        <v>288430.4</v>
+        <v>360537.9</v>
       </c>
       <c r="S127" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T127" t="n">
-        <v>13235309</v>
+        <v>15247650</v>
       </c>
       <c r="U127" t="n">
-        <v>15245638</v>
+        <v>15247650</v>
       </c>
       <c r="V127" t="n">
         <v>1260000</v>
@@ -10845,34 +10845,34 @@
         <v>2266.8</v>
       </c>
       <c r="P128" t="n">
-        <v>358456.2</v>
+        <v>398284.7</v>
       </c>
       <c r="Q128" t="n">
         <v>8440.4</v>
       </c>
       <c r="R128" t="n">
-        <v>288430.4</v>
+        <v>360537.9</v>
       </c>
       <c r="S128" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T128" t="n">
-        <v>11640572</v>
+        <v>13443231</v>
       </c>
       <c r="U128" t="n">
-        <v>13650901</v>
+        <v>13443231</v>
       </c>
       <c r="V128" t="n">
         <v>1270000</v>
       </c>
       <c r="W128" t="n">
-        <v>-10.53</v>
+        <v>-11.9</v>
       </c>
       <c r="X128" t="n">
-        <v>27.755</v>
+        <v>27.329</v>
       </c>
       <c r="Y128" t="n">
-        <v>4057143</v>
+        <v>4057142</v>
       </c>
     </row>
     <row r="129">
@@ -10926,34 +10926,34 @@
         <v>2286</v>
       </c>
       <c r="P129" t="n">
-        <v>358456.2</v>
+        <v>398284.7</v>
       </c>
       <c r="Q129" t="n">
         <v>8499.700000000001</v>
       </c>
       <c r="R129" t="n">
-        <v>288430.4</v>
+        <v>360537.9</v>
       </c>
       <c r="S129" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T129" t="n">
-        <v>10980389</v>
+        <v>12699329</v>
       </c>
       <c r="U129" t="n">
-        <v>12990718</v>
+        <v>12699329</v>
       </c>
       <c r="V129" t="n">
         <v>1280000</v>
       </c>
       <c r="W129" t="n">
-        <v>-4.91</v>
+        <v>-5.61</v>
       </c>
       <c r="X129" t="n">
-        <v>26.393</v>
+        <v>25.797</v>
       </c>
       <c r="Y129" t="n">
-        <v>3943595</v>
+        <v>3943596</v>
       </c>
     </row>
     <row r="130">
@@ -11007,31 +11007,31 @@
         <v>2303.2</v>
       </c>
       <c r="P130" t="n">
-        <v>358456.2</v>
+        <v>398284.7</v>
       </c>
       <c r="Q130" t="n">
         <v>8549.4</v>
       </c>
       <c r="R130" t="n">
-        <v>288430.4</v>
+        <v>360537.9</v>
       </c>
       <c r="S130" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T130" t="n">
-        <v>15859051</v>
+        <v>18502833</v>
       </c>
       <c r="U130" t="n">
-        <v>17869380</v>
+        <v>18502833</v>
       </c>
       <c r="V130" t="n">
         <v>1290000</v>
       </c>
       <c r="W130" t="n">
-        <v>37.48</v>
+        <v>45.62</v>
       </c>
       <c r="X130" t="n">
-        <v>36.284</v>
+        <v>37.565</v>
       </c>
       <c r="Y130" t="n">
         <v>4396283</v>
@@ -11088,34 +11088,34 @@
         <v>2319.6</v>
       </c>
       <c r="P131" t="n">
-        <v>358456.2</v>
+        <v>398284.7</v>
       </c>
       <c r="Q131" t="n">
         <v>8596.5</v>
       </c>
       <c r="R131" t="n">
-        <v>288430.4</v>
+        <v>360537.9</v>
       </c>
       <c r="S131" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T131" t="n">
-        <v>18095381</v>
+        <v>21134547</v>
       </c>
       <c r="U131" t="n">
-        <v>20105711</v>
+        <v>21134547</v>
       </c>
       <c r="V131" t="n">
         <v>1300000</v>
       </c>
       <c r="W131" t="n">
-        <v>12.46</v>
+        <v>14.17</v>
       </c>
       <c r="X131" t="n">
-        <v>40.805</v>
+        <v>42.888</v>
       </c>
       <c r="Y131" t="n">
-        <v>4621799</v>
+        <v>4621800</v>
       </c>
     </row>
     <row r="132">
@@ -11169,34 +11169,34 @@
         <v>2336</v>
       </c>
       <c r="P132" t="n">
-        <v>358456.2</v>
+        <v>398284.7</v>
       </c>
       <c r="Q132" t="n">
         <v>8642</v>
       </c>
       <c r="R132" t="n">
-        <v>288430.4</v>
+        <v>360537.9</v>
       </c>
       <c r="S132" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T132" t="n">
-        <v>18748462</v>
+        <v>21944520</v>
       </c>
       <c r="U132" t="n">
-        <v>20758792</v>
+        <v>21944520</v>
       </c>
       <c r="V132" t="n">
         <v>1310000</v>
       </c>
       <c r="W132" t="n">
-        <v>3.2</v>
+        <v>3.79</v>
       </c>
       <c r="X132" t="n">
-        <v>42.11</v>
+        <v>44.511</v>
       </c>
       <c r="Y132" t="n">
-        <v>4643869</v>
+        <v>4643868</v>
       </c>
     </row>
     <row r="133">
@@ -11250,34 +11250,34 @@
         <v>2352.4</v>
       </c>
       <c r="P133" t="n">
-        <v>358456.2</v>
+        <v>398284.7</v>
       </c>
       <c r="Q133" t="n">
         <v>8684.700000000001</v>
       </c>
       <c r="R133" t="n">
-        <v>288430.4</v>
+        <v>360537.9</v>
       </c>
       <c r="S133" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T133" t="n">
-        <v>20195911</v>
+        <v>23751399</v>
       </c>
       <c r="U133" t="n">
-        <v>22206241</v>
+        <v>23751399</v>
       </c>
       <c r="V133" t="n">
         <v>1320000</v>
       </c>
       <c r="W133" t="n">
-        <v>6.92</v>
+        <v>8.19</v>
       </c>
       <c r="X133" t="n">
-        <v>45.026</v>
+        <v>48.156</v>
       </c>
       <c r="Y133" t="n">
-        <v>4647660</v>
+        <v>4647659</v>
       </c>
     </row>
     <row r="134">
@@ -11331,31 +11331,31 @@
         <v>2368.5</v>
       </c>
       <c r="P134" t="n">
-        <v>358456.2</v>
+        <v>398284.7</v>
       </c>
       <c r="Q134" t="n">
         <v>8727</v>
       </c>
       <c r="R134" t="n">
-        <v>288430.4</v>
+        <v>360537.9</v>
       </c>
       <c r="S134" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T134" t="n">
-        <v>20268341</v>
+        <v>23809373</v>
       </c>
       <c r="U134" t="n">
-        <v>22278671</v>
+        <v>23809373</v>
       </c>
       <c r="V134" t="n">
         <v>1330000</v>
       </c>
       <c r="W134" t="n">
-        <v>0.28</v>
+        <v>0.2</v>
       </c>
       <c r="X134" t="n">
-        <v>45.153</v>
+        <v>48.253</v>
       </c>
       <c r="Y134" t="n">
         <v>4737438</v>
@@ -11412,31 +11412,31 @@
         <v>2368.5</v>
       </c>
       <c r="P135" t="n">
-        <v>358650.5</v>
+        <v>398479</v>
       </c>
       <c r="Q135" t="n">
         <v>8727</v>
       </c>
       <c r="R135" t="n">
-        <v>288569.9</v>
+        <v>360677.5</v>
       </c>
       <c r="S135" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T135" t="n">
-        <v>21356495</v>
+        <v>24961851</v>
       </c>
       <c r="U135" t="n">
-        <v>23366824</v>
+        <v>24961851</v>
       </c>
       <c r="V135" t="n">
         <v>1340000</v>
       </c>
       <c r="W135" t="n">
-        <v>4.84</v>
+        <v>4.8</v>
       </c>
       <c r="X135" t="n">
-        <v>47.338</v>
+        <v>50.569</v>
       </c>
       <c r="Y135" t="n">
         <v>5027403</v>
@@ -11493,31 +11493,31 @@
         <v>2368.5</v>
       </c>
       <c r="P136" t="n">
-        <v>358854.4</v>
+        <v>398682.9</v>
       </c>
       <c r="Q136" t="n">
         <v>8727</v>
       </c>
       <c r="R136" t="n">
-        <v>288702.7</v>
+        <v>360810.2</v>
       </c>
       <c r="S136" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T136" t="n">
-        <v>21475511</v>
+        <v>25164174</v>
       </c>
       <c r="U136" t="n">
-        <v>23485840</v>
+        <v>25164174</v>
       </c>
       <c r="V136" t="n">
         <v>1350000</v>
       </c>
       <c r="W136" t="n">
-        <v>0.47</v>
+        <v>0.77</v>
       </c>
       <c r="X136" t="n">
-        <v>47.559</v>
+        <v>50.958</v>
       </c>
       <c r="Y136" t="n">
         <v>4977002</v>
@@ -11574,34 +11574,34 @@
         <v>2368.5</v>
       </c>
       <c r="P137" t="n">
-        <v>359025.2</v>
+        <v>398853.7</v>
       </c>
       <c r="Q137" t="n">
         <v>8727</v>
       </c>
       <c r="R137" t="n">
-        <v>288818.2</v>
+        <v>360925.8</v>
       </c>
       <c r="S137" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T137" t="n">
-        <v>24908235</v>
+        <v>29189207</v>
       </c>
       <c r="U137" t="n">
-        <v>26918564</v>
+        <v>29189207</v>
       </c>
       <c r="V137" t="n">
         <v>1360000</v>
       </c>
       <c r="W137" t="n">
-        <v>14.57</v>
+        <v>15.96</v>
       </c>
       <c r="X137" t="n">
-        <v>54.49</v>
+        <v>59.089</v>
       </c>
       <c r="Y137" t="n">
-        <v>5298658</v>
+        <v>5298659</v>
       </c>
     </row>
     <row r="138">
@@ -11655,34 +11655,34 @@
         <v>2368.5</v>
       </c>
       <c r="P138" t="n">
-        <v>359182.8</v>
+        <v>399011.3</v>
       </c>
       <c r="Q138" t="n">
         <v>8727</v>
       </c>
       <c r="R138" t="n">
-        <v>288934.2</v>
+        <v>361041.8</v>
       </c>
       <c r="S138" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T138" t="n">
-        <v>25781200</v>
+        <v>30149064</v>
       </c>
       <c r="U138" t="n">
-        <v>27791530</v>
+        <v>30149064</v>
       </c>
       <c r="V138" t="n">
         <v>1370000</v>
       </c>
       <c r="W138" t="n">
-        <v>3.21</v>
+        <v>3.25</v>
       </c>
       <c r="X138" t="n">
-        <v>56.236</v>
+        <v>61.012</v>
       </c>
       <c r="Y138" t="n">
-        <v>5460239</v>
+        <v>5460241</v>
       </c>
     </row>
     <row r="139">
@@ -11736,31 +11736,31 @@
         <v>2368.5</v>
       </c>
       <c r="P139" t="n">
-        <v>359322.7</v>
+        <v>399151.2</v>
       </c>
       <c r="Q139" t="n">
         <v>8727</v>
       </c>
       <c r="R139" t="n">
-        <v>289044.8</v>
+        <v>361152.4</v>
       </c>
       <c r="S139" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T139" t="n">
-        <v>27901224</v>
+        <v>32579500</v>
       </c>
       <c r="U139" t="n">
-        <v>29911553</v>
+        <v>32579500</v>
       </c>
       <c r="V139" t="n">
         <v>1380000</v>
       </c>
       <c r="W139" t="n">
-        <v>7.59</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="X139" t="n">
-        <v>60.506</v>
+        <v>65.91</v>
       </c>
       <c r="Y139" t="n">
         <v>5700579</v>
@@ -11817,31 +11817,31 @@
         <v>2382.9</v>
       </c>
       <c r="P140" t="n">
-        <v>359322.7</v>
+        <v>399151.2</v>
       </c>
       <c r="Q140" t="n">
         <v>8767.1</v>
       </c>
       <c r="R140" t="n">
-        <v>289044.8</v>
+        <v>361152.4</v>
       </c>
       <c r="S140" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T140" t="n">
-        <v>23836146</v>
+        <v>27821991</v>
       </c>
       <c r="U140" t="n">
-        <v>25846475</v>
+        <v>27821991</v>
       </c>
       <c r="V140" t="n">
         <v>1390000</v>
       </c>
       <c r="W140" t="n">
-        <v>-13.62</v>
+        <v>-14.63</v>
       </c>
       <c r="X140" t="n">
-        <v>52.263</v>
+        <v>56.265</v>
       </c>
       <c r="Y140" t="n">
         <v>5386596</v>
@@ -11898,34 +11898,34 @@
         <v>2382.9</v>
       </c>
       <c r="P141" t="n">
-        <v>359457.6</v>
+        <v>399286</v>
       </c>
       <c r="Q141" t="n">
         <v>8767.1</v>
       </c>
       <c r="R141" t="n">
-        <v>289152.9</v>
+        <v>361260.5</v>
       </c>
       <c r="S141" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T141" t="n">
-        <v>28743957</v>
+        <v>33553109</v>
       </c>
       <c r="U141" t="n">
-        <v>30754286</v>
+        <v>33553109</v>
       </c>
       <c r="V141" t="n">
         <v>1400000</v>
       </c>
       <c r="W141" t="n">
-        <v>18.95</v>
+        <v>20.56</v>
       </c>
       <c r="X141" t="n">
-        <v>62.167</v>
+        <v>67.83499999999999</v>
       </c>
       <c r="Y141" t="n">
-        <v>5820188</v>
+        <v>5820189</v>
       </c>
     </row>
     <row r="142">
@@ -11979,34 +11979,34 @@
         <v>2395.9</v>
       </c>
       <c r="P142" t="n">
-        <v>359457.6</v>
+        <v>399286</v>
       </c>
       <c r="Q142" t="n">
         <v>8800.9</v>
       </c>
       <c r="R142" t="n">
-        <v>289152.9</v>
+        <v>361260.5</v>
       </c>
       <c r="S142" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T142" t="n">
-        <v>34394463</v>
+        <v>40473534</v>
       </c>
       <c r="U142" t="n">
-        <v>36404792</v>
+        <v>40473534</v>
       </c>
       <c r="V142" t="n">
         <v>1410000</v>
       </c>
       <c r="W142" t="n">
-        <v>18.34</v>
+        <v>20.6</v>
       </c>
       <c r="X142" t="n">
-        <v>73.568</v>
+        <v>81.806</v>
       </c>
       <c r="Y142" t="n">
-        <v>5946399</v>
+        <v>5946398</v>
       </c>
     </row>
     <row r="143">
@@ -12060,34 +12060,34 @@
         <v>2395.9</v>
       </c>
       <c r="P143" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q143" t="n">
         <v>8800.9</v>
       </c>
       <c r="R143" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S143" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T143" t="n">
-        <v>35624097</v>
+        <v>41964991</v>
       </c>
       <c r="U143" t="n">
-        <v>37634427</v>
+        <v>41964991</v>
       </c>
       <c r="V143" t="n">
         <v>1420000</v>
       </c>
       <c r="W143" t="n">
-        <v>3.35</v>
+        <v>3.66</v>
       </c>
       <c r="X143" t="n">
-        <v>76.033</v>
+        <v>84.8</v>
       </c>
       <c r="Y143" t="n">
-        <v>6024912</v>
+        <v>6024911</v>
       </c>
     </row>
     <row r="144">
@@ -12141,34 +12141,34 @@
         <v>2410.1</v>
       </c>
       <c r="P144" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q144" t="n">
         <v>8838.1</v>
       </c>
       <c r="R144" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S144" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T144" t="n">
-        <v>25169557</v>
+        <v>29465121</v>
       </c>
       <c r="U144" t="n">
-        <v>27179886</v>
+        <v>29465121</v>
       </c>
       <c r="V144" t="n">
         <v>1430000</v>
       </c>
       <c r="W144" t="n">
-        <v>-27.81</v>
+        <v>-29.81</v>
       </c>
       <c r="X144" t="n">
-        <v>54.891</v>
+        <v>59.521</v>
       </c>
       <c r="Y144" t="n">
-        <v>5507902</v>
+        <v>5507901</v>
       </c>
     </row>
     <row r="145">
@@ -12222,34 +12222,34 @@
         <v>2424.8</v>
       </c>
       <c r="P145" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q145" t="n">
         <v>8876.299999999999</v>
       </c>
       <c r="R145" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S145" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T145" t="n">
-        <v>22499081</v>
+        <v>26366601</v>
       </c>
       <c r="U145" t="n">
-        <v>24509410</v>
+        <v>26366601</v>
       </c>
       <c r="V145" t="n">
         <v>1440000</v>
       </c>
       <c r="W145" t="n">
-        <v>-9.859999999999999</v>
+        <v>-10.55</v>
       </c>
       <c r="X145" t="n">
-        <v>49.478</v>
+        <v>53.242</v>
       </c>
       <c r="Y145" t="n">
-        <v>5271360</v>
+        <v>5271359</v>
       </c>
     </row>
     <row r="146">
@@ -12303,31 +12303,31 @@
         <v>2439</v>
       </c>
       <c r="P146" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q146" t="n">
         <v>8914.299999999999</v>
       </c>
       <c r="R146" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S146" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T146" t="n">
-        <v>22912703</v>
+        <v>26733468</v>
       </c>
       <c r="U146" t="n">
-        <v>24923032</v>
+        <v>26733468</v>
       </c>
       <c r="V146" t="n">
         <v>1450000</v>
       </c>
       <c r="W146" t="n">
-        <v>1.65</v>
+        <v>1.35</v>
       </c>
       <c r="X146" t="n">
-        <v>50.293</v>
+        <v>53.962</v>
       </c>
       <c r="Y146" t="n">
         <v>5527411</v>
@@ -12384,34 +12384,34 @@
         <v>2455.3</v>
       </c>
       <c r="P147" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q147" t="n">
         <v>8958.799999999999</v>
       </c>
       <c r="R147" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S147" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T147" t="n">
-        <v>14270759</v>
+        <v>16522123</v>
       </c>
       <c r="U147" t="n">
-        <v>16281088</v>
+        <v>16522123</v>
       </c>
       <c r="V147" t="n">
         <v>1460000</v>
       </c>
       <c r="W147" t="n">
-        <v>-34.71</v>
+        <v>-38.23</v>
       </c>
       <c r="X147" t="n">
-        <v>32.834</v>
+        <v>33.33</v>
       </c>
       <c r="Y147" t="n">
-        <v>4785907</v>
+        <v>4785908</v>
       </c>
     </row>
     <row r="148">
@@ -12465,34 +12465,34 @@
         <v>2471.9</v>
       </c>
       <c r="P148" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q148" t="n">
         <v>9000.700000000001</v>
       </c>
       <c r="R148" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S148" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T148" t="n">
-        <v>14471120</v>
+        <v>16839658</v>
       </c>
       <c r="U148" t="n">
-        <v>16481449</v>
+        <v>16839658</v>
       </c>
       <c r="V148" t="n">
         <v>1470000</v>
       </c>
       <c r="W148" t="n">
-        <v>1.17</v>
+        <v>1.86</v>
       </c>
       <c r="X148" t="n">
-        <v>33.218</v>
+        <v>33.951</v>
       </c>
       <c r="Y148" t="n">
-        <v>4719966</v>
+        <v>4719965</v>
       </c>
     </row>
     <row r="149">
@@ -12546,31 +12546,31 @@
         <v>2490.2</v>
       </c>
       <c r="P149" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q149" t="n">
         <v>9051</v>
       </c>
       <c r="R149" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S149" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T149" t="n">
-        <v>9384857</v>
+        <v>10759377</v>
       </c>
       <c r="U149" t="n">
-        <v>11395187</v>
+        <v>10759377</v>
       </c>
       <c r="V149" t="n">
         <v>1480000</v>
       </c>
       <c r="W149" t="n">
-        <v>-30.92</v>
+        <v>-36.17</v>
       </c>
       <c r="X149" t="n">
-        <v>22.946</v>
+        <v>21.672</v>
       </c>
       <c r="Y149" t="n">
         <v>4309506</v>
@@ -12627,34 +12627,34 @@
         <v>2506.4</v>
       </c>
       <c r="P150" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q150" t="n">
         <v>9094.1</v>
       </c>
       <c r="R150" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S150" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T150" t="n">
-        <v>13127070</v>
+        <v>15151249</v>
       </c>
       <c r="U150" t="n">
-        <v>15137400</v>
+        <v>15151249</v>
       </c>
       <c r="V150" t="n">
         <v>1490000</v>
       </c>
       <c r="W150" t="n">
-        <v>32.75</v>
+        <v>40.73</v>
       </c>
       <c r="X150" t="n">
-        <v>30.462</v>
+        <v>30.498</v>
       </c>
       <c r="Y150" t="n">
-        <v>4860414</v>
+        <v>4860413</v>
       </c>
     </row>
     <row r="151">
@@ -12708,34 +12708,34 @@
         <v>2523.5</v>
       </c>
       <c r="P151" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q151" t="n">
         <v>9141.9</v>
       </c>
       <c r="R151" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S151" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T151" t="n">
-        <v>10416649</v>
+        <v>11929511</v>
       </c>
       <c r="U151" t="n">
-        <v>12426978</v>
+        <v>11929511</v>
       </c>
       <c r="V151" t="n">
         <v>1500000</v>
       </c>
       <c r="W151" t="n">
-        <v>-17.97</v>
+        <v>-21.33</v>
       </c>
       <c r="X151" t="n">
-        <v>24.988</v>
+        <v>23.993</v>
       </c>
       <c r="Y151" t="n">
-        <v>4620959</v>
+        <v>4620957</v>
       </c>
     </row>
     <row r="152">
@@ -12789,31 +12789,31 @@
         <v>2542.6</v>
       </c>
       <c r="P152" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q152" t="n">
         <v>9197.200000000001</v>
       </c>
       <c r="R152" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S152" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T152" t="n">
-        <v>7311772</v>
+        <v>8302176</v>
       </c>
       <c r="U152" t="n">
-        <v>9322101</v>
+        <v>8302176</v>
       </c>
       <c r="V152" t="n">
         <v>1510000</v>
       </c>
       <c r="W152" t="n">
-        <v>-25.07</v>
+        <v>-30.49</v>
       </c>
       <c r="X152" t="n">
-        <v>18.724</v>
+        <v>16.678</v>
       </c>
       <c r="Y152" t="n">
         <v>4144106</v>
@@ -12870,34 +12870,34 @@
         <v>2560.9</v>
       </c>
       <c r="P153" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q153" t="n">
         <v>9251.299999999999</v>
       </c>
       <c r="R153" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S153" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T153" t="n">
-        <v>7663587</v>
+        <v>8689211</v>
       </c>
       <c r="U153" t="n">
-        <v>9673916</v>
+        <v>8689211</v>
       </c>
       <c r="V153" t="n">
         <v>1520000</v>
       </c>
       <c r="W153" t="n">
-        <v>3.67</v>
+        <v>4.54</v>
       </c>
       <c r="X153" t="n">
-        <v>19.411</v>
+        <v>17.435</v>
       </c>
       <c r="Y153" t="n">
-        <v>4319854</v>
+        <v>4319853</v>
       </c>
     </row>
     <row r="154">
@@ -12951,31 +12951,31 @@
         <v>2578.3</v>
       </c>
       <c r="P154" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q154" t="n">
         <v>9296.299999999999</v>
       </c>
       <c r="R154" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S154" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T154" t="n">
-        <v>9716005</v>
+        <v>11135782</v>
       </c>
       <c r="U154" t="n">
-        <v>11726335</v>
+        <v>11135782</v>
       </c>
       <c r="V154" t="n">
         <v>1530000</v>
       </c>
       <c r="W154" t="n">
-        <v>21.11</v>
+        <v>28.04</v>
       </c>
       <c r="X154" t="n">
-        <v>23.509</v>
+        <v>22.324</v>
       </c>
       <c r="Y154" t="n">
         <v>4569342</v>
@@ -13032,34 +13032,34 @@
         <v>2597.5</v>
       </c>
       <c r="P155" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q155" t="n">
         <v>9346.200000000001</v>
       </c>
       <c r="R155" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S155" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T155" t="n">
-        <v>7337148</v>
+        <v>8350213</v>
       </c>
       <c r="U155" t="n">
-        <v>9347477</v>
+        <v>8350213</v>
       </c>
       <c r="V155" t="n">
         <v>1540000</v>
       </c>
       <c r="W155" t="n">
-        <v>-20.37</v>
+        <v>-25.1</v>
       </c>
       <c r="X155" t="n">
-        <v>18.72</v>
+        <v>16.72</v>
       </c>
       <c r="Y155" t="n">
-        <v>4167468</v>
+        <v>4167467</v>
       </c>
     </row>
     <row r="156">
@@ -13113,31 +13113,31 @@
         <v>2614.7</v>
       </c>
       <c r="P156" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q156" t="n">
         <v>9388.9</v>
       </c>
       <c r="R156" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S156" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T156" t="n">
-        <v>9917835</v>
+        <v>11380368</v>
       </c>
       <c r="U156" t="n">
-        <v>11928165</v>
+        <v>11380368</v>
       </c>
       <c r="V156" t="n">
         <v>1550000</v>
       </c>
       <c r="W156" t="n">
-        <v>27.5</v>
+        <v>36.17</v>
       </c>
       <c r="X156" t="n">
-        <v>23.868</v>
+        <v>22.767</v>
       </c>
       <c r="Y156" t="n">
         <v>4620998</v>
@@ -13194,34 +13194,34 @@
         <v>2632.1</v>
       </c>
       <c r="P157" t="n">
-        <v>359583.3</v>
+        <v>399411.8</v>
       </c>
       <c r="Q157" t="n">
         <v>9431.200000000001</v>
       </c>
       <c r="R157" t="n">
-        <v>289228.6</v>
+        <v>361336.1</v>
       </c>
       <c r="S157" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T157" t="n">
-        <v>9837910</v>
+        <v>11294702</v>
       </c>
       <c r="U157" t="n">
-        <v>11848239</v>
+        <v>11294702</v>
       </c>
       <c r="V157" t="n">
         <v>1560000</v>
       </c>
       <c r="W157" t="n">
-        <v>-0.75</v>
+        <v>-0.84</v>
       </c>
       <c r="X157" t="n">
-        <v>23.688</v>
+        <v>22.576</v>
       </c>
       <c r="Y157" t="n">
-        <v>4614363</v>
+        <v>4614362</v>
       </c>
     </row>
     <row r="158">
@@ -13275,31 +13275,31 @@
         <v>2632.1</v>
       </c>
       <c r="P158" t="n">
-        <v>359949.4</v>
+        <v>399777.8</v>
       </c>
       <c r="Q158" t="n">
         <v>9431.200000000001</v>
       </c>
       <c r="R158" t="n">
-        <v>289507.1</v>
+        <v>361614.7</v>
       </c>
       <c r="S158" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T158" t="n">
-        <v>12157915</v>
+        <v>13994542</v>
       </c>
       <c r="U158" t="n">
-        <v>14168244</v>
+        <v>13994542</v>
       </c>
       <c r="V158" t="n">
         <v>1570000</v>
       </c>
       <c r="W158" t="n">
-        <v>19.5</v>
+        <v>23.82</v>
       </c>
       <c r="X158" t="n">
-        <v>28.307</v>
+        <v>27.952</v>
       </c>
       <c r="Y158" t="n">
         <v>5062381</v>
@@ -13356,31 +13356,31 @@
         <v>2632.1</v>
       </c>
       <c r="P159" t="n">
-        <v>360315.6</v>
+        <v>400144</v>
       </c>
       <c r="Q159" t="n">
         <v>9431.200000000001</v>
       </c>
       <c r="R159" t="n">
-        <v>289865.3</v>
+        <v>361972.8</v>
       </c>
       <c r="S159" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T159" t="n">
-        <v>10941510</v>
+        <v>12490340</v>
       </c>
       <c r="U159" t="n">
-        <v>12951839</v>
+        <v>12490340</v>
       </c>
       <c r="V159" t="n">
         <v>1580000</v>
       </c>
       <c r="W159" t="n">
-        <v>-8.66</v>
+        <v>-10.82</v>
       </c>
       <c r="X159" t="n">
-        <v>25.856</v>
+        <v>24.928</v>
       </c>
       <c r="Y159" t="n">
         <v>5098083</v>
@@ -13437,31 +13437,31 @@
         <v>2632.1</v>
       </c>
       <c r="P160" t="n">
-        <v>360613.3</v>
+        <v>400441.7</v>
       </c>
       <c r="Q160" t="n">
         <v>9431.200000000001</v>
       </c>
       <c r="R160" t="n">
-        <v>290106.3</v>
+        <v>362213.8</v>
       </c>
       <c r="S160" t="n">
-        <v>2010329</v>
+        <v>0</v>
       </c>
       <c r="T160" t="n">
-        <v>14306486</v>
+        <v>16469316</v>
       </c>
       <c r="U160" t="n">
-        <v>16316816</v>
+        <v>16469316</v>
       </c>
       <c r="V160" t="n">
         <v>1590000</v>
       </c>
       <c r="W160" t="n">
-        <v>25.9</v>
+        <v>31.78</v>
       </c>
       <c r="X160" t="n">
-        <v>32.554</v>
+        <v>32.849</v>
       </c>
       <c r="Y160" t="n">
         <v>5509995</v>
@@ -13485,13 +13485,13 @@
         <v>10000</v>
       </c>
       <c r="E161" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="F161" t="n">
         <v>0</v>
       </c>
       <c r="G161" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="H161" t="n">
         <v>0</v>
@@ -13515,37 +13515,37 @@
         <v>24.37</v>
       </c>
       <c r="O161" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P161" t="n">
-        <v>360613.3</v>
+        <v>400441.7</v>
       </c>
       <c r="Q161" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R161" t="n">
-        <v>290106.3</v>
+        <v>362213.8</v>
       </c>
       <c r="S161" t="n">
-        <v>2020329</v>
+        <v>0</v>
       </c>
       <c r="T161" t="n">
-        <v>16604858</v>
+        <v>19163123</v>
       </c>
       <c r="U161" t="n">
-        <v>18625187</v>
+        <v>19163123</v>
       </c>
       <c r="V161" t="n">
         <v>1600000</v>
       </c>
       <c r="W161" t="n">
-        <v>14.09</v>
+        <v>16.3</v>
       </c>
       <c r="X161" t="n">
-        <v>37.14</v>
+        <v>38.202</v>
       </c>
       <c r="Y161" t="n">
-        <v>5867327</v>
+        <v>5867328</v>
       </c>
     </row>
     <row r="162">
@@ -13596,34 +13596,34 @@
         <v>27.88</v>
       </c>
       <c r="O162" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P162" t="n">
-        <v>360840.9</v>
+        <v>400669.3</v>
       </c>
       <c r="Q162" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R162" t="n">
-        <v>290285.4</v>
+        <v>362393</v>
       </c>
       <c r="S162" t="n">
-        <v>2020329</v>
+        <v>0</v>
       </c>
       <c r="T162" t="n">
-        <v>18501854</v>
+        <v>21397101</v>
       </c>
       <c r="U162" t="n">
-        <v>20522184</v>
+        <v>21397101</v>
       </c>
       <c r="V162" t="n">
         <v>1610000</v>
       </c>
       <c r="W162" t="n">
-        <v>10.13</v>
+        <v>11.61</v>
       </c>
       <c r="X162" t="n">
-        <v>40.903</v>
+        <v>42.635</v>
       </c>
       <c r="Y162" t="n">
         <v>6103802</v>
@@ -13677,34 +13677,34 @@
         <v>23.42</v>
       </c>
       <c r="O163" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P163" t="n">
-        <v>361083.9</v>
+        <v>400912.3</v>
       </c>
       <c r="Q163" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R163" t="n">
-        <v>290498.7</v>
+        <v>362606.3</v>
       </c>
       <c r="S163" t="n">
-        <v>2020329</v>
+        <v>0</v>
       </c>
       <c r="T163" t="n">
-        <v>16658182</v>
+        <v>19175820</v>
       </c>
       <c r="U163" t="n">
-        <v>18678511</v>
+        <v>19175820</v>
       </c>
       <c r="V163" t="n">
         <v>1620000</v>
       </c>
       <c r="W163" t="n">
-        <v>-9.029999999999999</v>
+        <v>-10.43</v>
       </c>
       <c r="X163" t="n">
-        <v>37.208</v>
+        <v>38.189</v>
       </c>
       <c r="Y163" t="n">
         <v>6023273</v>
@@ -13758,37 +13758,37 @@
         <v>18.55</v>
       </c>
       <c r="O164" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P164" t="n">
-        <v>361372.4</v>
+        <v>401200.8</v>
       </c>
       <c r="Q164" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R164" t="n">
-        <v>290767.9</v>
+        <v>362875.5</v>
       </c>
       <c r="S164" t="n">
-        <v>2020329</v>
+        <v>0</v>
       </c>
       <c r="T164" t="n">
-        <v>13929153</v>
+        <v>15966067</v>
       </c>
       <c r="U164" t="n">
-        <v>15949483</v>
+        <v>15966067</v>
       </c>
       <c r="V164" t="n">
         <v>1630000</v>
       </c>
       <c r="W164" t="n">
-        <v>-14.66</v>
+        <v>-16.79</v>
       </c>
       <c r="X164" t="n">
-        <v>31.752</v>
+        <v>31.777</v>
       </c>
       <c r="Y164" t="n">
-        <v>5727288</v>
+        <v>5727287</v>
       </c>
     </row>
     <row r="165">
@@ -13839,34 +13839,34 @@
         <v>14.65</v>
       </c>
       <c r="O165" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P165" t="n">
-        <v>361685.8</v>
+        <v>401514.3</v>
       </c>
       <c r="Q165" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R165" t="n">
-        <v>291108.9</v>
+        <v>363216.5</v>
       </c>
       <c r="S165" t="n">
-        <v>2020329</v>
+        <v>0</v>
       </c>
       <c r="T165" t="n">
-        <v>12230112</v>
+        <v>13930309</v>
       </c>
       <c r="U165" t="n">
-        <v>14250441</v>
+        <v>13930309</v>
       </c>
       <c r="V165" t="n">
         <v>1640000</v>
       </c>
       <c r="W165" t="n">
-        <v>-10.72</v>
+        <v>-12.81</v>
       </c>
       <c r="X165" t="n">
-        <v>28.35</v>
+        <v>27.705</v>
       </c>
       <c r="Y165" t="n">
         <v>5618982</v>
@@ -13920,37 +13920,37 @@
         <v>22.43</v>
       </c>
       <c r="O166" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P166" t="n">
-        <v>361920.1</v>
+        <v>401748.6</v>
       </c>
       <c r="Q166" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R166" t="n">
-        <v>291331.7</v>
+        <v>363439.2</v>
       </c>
       <c r="S166" t="n">
-        <v>2020329</v>
+        <v>0</v>
       </c>
       <c r="T166" t="n">
-        <v>16752395</v>
+        <v>19229261</v>
       </c>
       <c r="U166" t="n">
-        <v>18772725</v>
+        <v>19229261</v>
       </c>
       <c r="V166" t="n">
         <v>1650000</v>
       </c>
       <c r="W166" t="n">
-        <v>31.66</v>
+        <v>37.97</v>
       </c>
       <c r="X166" t="n">
-        <v>37.326</v>
+        <v>38.224</v>
       </c>
       <c r="Y166" t="n">
-        <v>6236879</v>
+        <v>6236880</v>
       </c>
     </row>
     <row r="167">
@@ -13983,10 +13983,10 @@
         <v>5000</v>
       </c>
       <c r="I167" t="n">
-        <v>895831</v>
+        <v>0</v>
       </c>
       <c r="J167" t="n">
-        <v>1802742</v>
+        <v>0</v>
       </c>
       <c r="K167" t="n">
         <v>404.54</v>
@@ -14001,34 +14001,34 @@
         <v>30.94</v>
       </c>
       <c r="O167" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P167" t="n">
-        <v>325929.9</v>
+        <v>401950.4</v>
       </c>
       <c r="Q167" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R167" t="n">
-        <v>233226.8</v>
+        <v>363600.7</v>
       </c>
       <c r="S167" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T167" t="n">
-        <v>17985074</v>
+        <v>23911804</v>
       </c>
       <c r="U167" t="n">
-        <v>22701278</v>
+        <v>23911804</v>
       </c>
       <c r="V167" t="n">
         <v>1660000</v>
       </c>
       <c r="W167" t="n">
-        <v>20.89</v>
+        <v>24.3</v>
       </c>
       <c r="X167" t="n">
-        <v>45.123</v>
+        <v>47.513</v>
       </c>
       <c r="Y167" t="n">
         <v>6595322</v>
@@ -14082,37 +14082,37 @@
         <v>31.63</v>
       </c>
       <c r="O168" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P168" t="n">
-        <v>326124.2</v>
+        <v>402144.7</v>
       </c>
       <c r="Q168" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R168" t="n">
-        <v>233384.7</v>
+        <v>363758.6</v>
       </c>
       <c r="S168" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T168" t="n">
-        <v>18586959</v>
+        <v>24676080</v>
       </c>
       <c r="U168" t="n">
-        <v>23303164</v>
+        <v>24676080</v>
       </c>
       <c r="V168" t="n">
         <v>1670000</v>
       </c>
       <c r="W168" t="n">
-        <v>2.61</v>
+        <v>3.15</v>
       </c>
       <c r="X168" t="n">
-        <v>46.3</v>
+        <v>49.011</v>
       </c>
       <c r="Y168" t="n">
-        <v>6725295</v>
+        <v>6725294</v>
       </c>
     </row>
     <row r="169">
@@ -14163,37 +14163,37 @@
         <v>42.21</v>
       </c>
       <c r="O169" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P169" t="n">
-        <v>326293.7</v>
+        <v>402314.2</v>
       </c>
       <c r="Q169" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R169" t="n">
-        <v>233503</v>
+        <v>363876.9</v>
       </c>
       <c r="S169" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T169" t="n">
-        <v>22597309</v>
+        <v>30353798</v>
       </c>
       <c r="U169" t="n">
-        <v>27313513</v>
+        <v>30353798</v>
       </c>
       <c r="V169" t="n">
         <v>1680000</v>
       </c>
       <c r="W169" t="n">
-        <v>17.17</v>
+        <v>22.97</v>
       </c>
       <c r="X169" t="n">
-        <v>54.248</v>
+        <v>60.269</v>
       </c>
       <c r="Y169" t="n">
-        <v>7090605</v>
+        <v>7090606</v>
       </c>
     </row>
     <row r="170">
@@ -14244,34 +14244,34 @@
         <v>45.89</v>
       </c>
       <c r="O170" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P170" t="n">
-        <v>326459.4</v>
+        <v>402479.8</v>
       </c>
       <c r="Q170" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R170" t="n">
-        <v>233611.9</v>
+        <v>363985.8</v>
       </c>
       <c r="S170" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T170" t="n">
-        <v>23828268</v>
+        <v>32116992</v>
       </c>
       <c r="U170" t="n">
-        <v>28544472</v>
+        <v>32116992</v>
       </c>
       <c r="V170" t="n">
         <v>1690000</v>
       </c>
       <c r="W170" t="n">
-        <v>4.47</v>
+        <v>5.78</v>
       </c>
       <c r="X170" t="n">
-        <v>56.673</v>
+        <v>63.75</v>
       </c>
       <c r="Y170" t="n">
         <v>7190999</v>
@@ -14325,37 +14325,37 @@
         <v>37.65</v>
       </c>
       <c r="O171" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P171" t="n">
-        <v>326652.6</v>
+        <v>402673.1</v>
       </c>
       <c r="Q171" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R171" t="n">
-        <v>233744.5</v>
+        <v>364118.5</v>
       </c>
       <c r="S171" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T171" t="n">
-        <v>20351215</v>
+        <v>27237243</v>
       </c>
       <c r="U171" t="n">
-        <v>25067419</v>
+        <v>27237243</v>
       </c>
       <c r="V171" t="n">
         <v>1700000</v>
       </c>
       <c r="W171" t="n">
-        <v>-12.22</v>
+        <v>-15.22</v>
       </c>
       <c r="X171" t="n">
-        <v>49.749</v>
+        <v>54.044</v>
       </c>
       <c r="Y171" t="n">
-        <v>6886470</v>
+        <v>6886471</v>
       </c>
     </row>
     <row r="172">
@@ -14406,37 +14406,37 @@
         <v>47.92</v>
       </c>
       <c r="O172" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P172" t="n">
-        <v>326815.7</v>
+        <v>402836.2</v>
       </c>
       <c r="Q172" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R172" t="n">
-        <v>233848.8</v>
+        <v>364222.7</v>
       </c>
       <c r="S172" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T172" t="n">
-        <v>24642707</v>
+        <v>33233013</v>
       </c>
       <c r="U172" t="n">
-        <v>29358911</v>
+        <v>33233013</v>
       </c>
       <c r="V172" t="n">
         <v>1710000</v>
       </c>
       <c r="W172" t="n">
-        <v>17.08</v>
+        <v>21.98</v>
       </c>
       <c r="X172" t="n">
-        <v>58.246</v>
+        <v>65.92100000000001</v>
       </c>
       <c r="Y172" t="n">
-        <v>7320103</v>
+        <v>7320104</v>
       </c>
     </row>
     <row r="173">
@@ -14487,34 +14487,34 @@
         <v>54.75</v>
       </c>
       <c r="O173" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P173" t="n">
-        <v>326953.3</v>
+        <v>402973.7</v>
       </c>
       <c r="Q173" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R173" t="n">
-        <v>233940</v>
+        <v>364313.9</v>
       </c>
       <c r="S173" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T173" t="n">
-        <v>28368036</v>
+        <v>38280840</v>
       </c>
       <c r="U173" t="n">
-        <v>33084240</v>
+        <v>38280840</v>
       </c>
       <c r="V173" t="n">
         <v>1720000</v>
       </c>
       <c r="W173" t="n">
-        <v>12.65</v>
+        <v>15.16</v>
       </c>
       <c r="X173" t="n">
-        <v>65.61799999999999</v>
+        <v>75.914</v>
       </c>
       <c r="Y173" t="n">
         <v>7803714</v>
@@ -14568,37 +14568,37 @@
         <v>43.9</v>
       </c>
       <c r="O174" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P174" t="n">
-        <v>327102</v>
+        <v>403122.5</v>
       </c>
       <c r="Q174" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R174" t="n">
-        <v>234053.8</v>
+        <v>364427.7</v>
       </c>
       <c r="S174" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T174" t="n">
-        <v>24799955</v>
+        <v>33090699</v>
       </c>
       <c r="U174" t="n">
-        <v>29516159</v>
+        <v>33090699</v>
       </c>
       <c r="V174" t="n">
         <v>1730000</v>
       </c>
       <c r="W174" t="n">
-        <v>-10.82</v>
+        <v>-13.58</v>
       </c>
       <c r="X174" t="n">
-        <v>58.521</v>
+        <v>65.602</v>
       </c>
       <c r="Y174" t="n">
-        <v>7682749</v>
+        <v>7682748</v>
       </c>
     </row>
     <row r="175">
@@ -14637,7 +14637,7 @@
         <v>0</v>
       </c>
       <c r="K175" t="n">
-        <v>471.85</v>
+        <v>471.84</v>
       </c>
       <c r="L175" t="n">
         <v>33.75</v>
@@ -14649,34 +14649,34 @@
         <v>38.36</v>
       </c>
       <c r="O175" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P175" t="n">
-        <v>327250</v>
+        <v>403270.5</v>
       </c>
       <c r="Q175" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R175" t="n">
-        <v>234184</v>
+        <v>364557.9</v>
       </c>
       <c r="S175" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T175" t="n">
-        <v>23547372</v>
+        <v>31128409</v>
       </c>
       <c r="U175" t="n">
-        <v>28263576</v>
+        <v>31128409</v>
       </c>
       <c r="V175" t="n">
         <v>1740000</v>
       </c>
       <c r="W175" t="n">
-        <v>-4.28</v>
+        <v>-5.96</v>
       </c>
       <c r="X175" t="n">
-        <v>56.018</v>
+        <v>61.692</v>
       </c>
       <c r="Y175" t="n">
         <v>7777546</v>
@@ -14730,34 +14730,34 @@
         <v>36.34</v>
       </c>
       <c r="O176" t="n">
-        <v>2632.1</v>
+        <v>2645.8</v>
       </c>
       <c r="P176" t="n">
-        <v>327389.7</v>
+        <v>403410.1</v>
       </c>
       <c r="Q176" t="n">
-        <v>9431.200000000001</v>
+        <v>9464.4</v>
       </c>
       <c r="R176" t="n">
-        <v>234321.5</v>
+        <v>364695.4</v>
       </c>
       <c r="S176" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T176" t="n">
-        <v>23797032</v>
+        <v>31268446</v>
       </c>
       <c r="U176" t="n">
-        <v>28513236</v>
+        <v>31268446</v>
       </c>
       <c r="V176" t="n">
         <v>1750000</v>
       </c>
       <c r="W176" t="n">
-        <v>0.85</v>
+        <v>0.42</v>
       </c>
       <c r="X176" t="n">
-        <v>56.493</v>
+        <v>61.949</v>
       </c>
       <c r="Y176" t="n">
         <v>7991432</v>
@@ -14811,37 +14811,37 @@
         <v>29.81</v>
       </c>
       <c r="O177" t="n">
-        <v>2642.5</v>
+        <v>2656.2</v>
       </c>
       <c r="P177" t="n">
-        <v>327389.7</v>
+        <v>403410.1</v>
       </c>
       <c r="Q177" t="n">
-        <v>9452</v>
+        <v>9485.299999999999</v>
       </c>
       <c r="R177" t="n">
-        <v>234321.5</v>
+        <v>364695.4</v>
       </c>
       <c r="S177" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T177" t="n">
-        <v>21739846</v>
+        <v>28245894</v>
       </c>
       <c r="U177" t="n">
-        <v>26456050</v>
+        <v>28245894</v>
       </c>
       <c r="V177" t="n">
         <v>1760000</v>
       </c>
       <c r="W177" t="n">
-        <v>-7.25</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="X177" t="n">
-        <v>52.397</v>
+        <v>55.941</v>
       </c>
       <c r="Y177" t="n">
-        <v>7932325</v>
+        <v>7932326</v>
       </c>
     </row>
     <row r="178">
@@ -14892,37 +14892,37 @@
         <v>27.8</v>
       </c>
       <c r="O178" t="n">
-        <v>2642.5</v>
+        <v>2656.2</v>
       </c>
       <c r="P178" t="n">
-        <v>327516.4</v>
+        <v>403536.8</v>
       </c>
       <c r="Q178" t="n">
-        <v>9452</v>
+        <v>9485.299999999999</v>
       </c>
       <c r="R178" t="n">
-        <v>234501.2</v>
+        <v>364875.1</v>
       </c>
       <c r="S178" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T178" t="n">
-        <v>23037207</v>
+        <v>29673043</v>
       </c>
       <c r="U178" t="n">
-        <v>27753411</v>
+        <v>29673043</v>
       </c>
       <c r="V178" t="n">
         <v>1770000</v>
       </c>
       <c r="W178" t="n">
-        <v>4.87</v>
+        <v>5.02</v>
       </c>
       <c r="X178" t="n">
-        <v>54.947</v>
+        <v>58.748</v>
       </c>
       <c r="Y178" t="n">
-        <v>8366761</v>
+        <v>8366760</v>
       </c>
     </row>
     <row r="179">
@@ -14973,34 +14973,34 @@
         <v>27.13</v>
       </c>
       <c r="O179" t="n">
-        <v>2642.5</v>
+        <v>2656.2</v>
       </c>
       <c r="P179" t="n">
-        <v>327643.9</v>
+        <v>403664.3</v>
       </c>
       <c r="Q179" t="n">
-        <v>9452</v>
+        <v>9485.299999999999</v>
       </c>
       <c r="R179" t="n">
-        <v>234685.3</v>
+        <v>365059.2</v>
       </c>
       <c r="S179" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T179" t="n">
-        <v>22827093</v>
+        <v>29357461</v>
       </c>
       <c r="U179" t="n">
-        <v>27543297</v>
+        <v>29357461</v>
       </c>
       <c r="V179" t="n">
         <v>1780000</v>
       </c>
       <c r="W179" t="n">
-        <v>-0.79</v>
+        <v>-1.1</v>
       </c>
       <c r="X179" t="n">
-        <v>54.511</v>
+        <v>58.103</v>
       </c>
       <c r="Y179" t="n">
         <v>8414738</v>
@@ -15054,37 +15054,37 @@
         <v>26.84</v>
       </c>
       <c r="O180" t="n">
-        <v>2642.5</v>
+        <v>2656.2</v>
       </c>
       <c r="P180" t="n">
-        <v>327765.8</v>
+        <v>403786.3</v>
       </c>
       <c r="Q180" t="n">
-        <v>9452</v>
+        <v>9485.299999999999</v>
       </c>
       <c r="R180" t="n">
-        <v>234871.4</v>
+        <v>365245.3</v>
       </c>
       <c r="S180" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T180" t="n">
-        <v>23394493</v>
+        <v>30022609</v>
       </c>
       <c r="U180" t="n">
-        <v>28110697</v>
+        <v>30022609</v>
       </c>
       <c r="V180" t="n">
         <v>1790000</v>
       </c>
       <c r="W180" t="n">
-        <v>2.02</v>
+        <v>2.23</v>
       </c>
       <c r="X180" t="n">
-        <v>55.614</v>
+        <v>59.4</v>
       </c>
       <c r="Y180" t="n">
-        <v>8606773</v>
+        <v>8606772</v>
       </c>
     </row>
     <row r="181">
@@ -15135,37 +15135,37 @@
         <v>22.58</v>
       </c>
       <c r="O181" t="n">
-        <v>2642.5</v>
+        <v>2656.2</v>
       </c>
       <c r="P181" t="n">
-        <v>327900.5</v>
+        <v>403921</v>
       </c>
       <c r="Q181" t="n">
-        <v>9452</v>
+        <v>9485.299999999999</v>
       </c>
       <c r="R181" t="n">
-        <v>235092.6</v>
+        <v>365466.5</v>
       </c>
       <c r="S181" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T181" t="n">
-        <v>20998469</v>
+        <v>26776824</v>
       </c>
       <c r="U181" t="n">
-        <v>25714673</v>
+        <v>26776824</v>
       </c>
       <c r="V181" t="n">
         <v>1800000</v>
       </c>
       <c r="W181" t="n">
-        <v>-8.56</v>
+        <v>-10.84</v>
       </c>
       <c r="X181" t="n">
-        <v>50.854</v>
+        <v>52.958</v>
       </c>
       <c r="Y181" t="n">
-        <v>8384082</v>
+        <v>8384081</v>
       </c>
     </row>
     <row r="182">
@@ -15216,34 +15216,34 @@
         <v>15.9</v>
       </c>
       <c r="O182" t="n">
-        <v>2653.2</v>
+        <v>2666.9</v>
       </c>
       <c r="P182" t="n">
-        <v>327900.5</v>
+        <v>403921</v>
       </c>
       <c r="Q182" t="n">
-        <v>9475.700000000001</v>
+        <v>9509</v>
       </c>
       <c r="R182" t="n">
-        <v>235092.6</v>
+        <v>365466.5</v>
       </c>
       <c r="S182" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T182" t="n">
-        <v>16301702</v>
+        <v>20550300</v>
       </c>
       <c r="U182" t="n">
-        <v>21017906</v>
+        <v>20550300</v>
       </c>
       <c r="V182" t="n">
         <v>1810000</v>
       </c>
       <c r="W182" t="n">
-        <v>-18.3</v>
+        <v>-23.29</v>
       </c>
       <c r="X182" t="n">
-        <v>41.546</v>
+        <v>40.624</v>
       </c>
       <c r="Y182" t="n">
         <v>7758040</v>
@@ -15297,34 +15297,34 @@
         <v>12.12</v>
       </c>
       <c r="O183" t="n">
-        <v>2663.7</v>
+        <v>2677.5</v>
       </c>
       <c r="P183" t="n">
-        <v>327900.5</v>
+        <v>403921</v>
       </c>
       <c r="Q183" t="n">
-        <v>9499.4</v>
+        <v>9532.700000000001</v>
       </c>
       <c r="R183" t="n">
-        <v>235092.6</v>
+        <v>365466.5</v>
       </c>
       <c r="S183" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T183" t="n">
-        <v>15045252</v>
+        <v>18710170</v>
       </c>
       <c r="U183" t="n">
-        <v>19761456</v>
+        <v>18710170</v>
       </c>
       <c r="V183" t="n">
         <v>1820000</v>
       </c>
       <c r="W183" t="n">
-        <v>-6.03</v>
+        <v>-9</v>
       </c>
       <c r="X183" t="n">
-        <v>39.043</v>
+        <v>36.967</v>
       </c>
       <c r="Y183" t="n">
         <v>7876396</v>
@@ -15378,34 +15378,34 @@
         <v>16.11</v>
       </c>
       <c r="O184" t="n">
-        <v>2673.4</v>
+        <v>2687.2</v>
       </c>
       <c r="P184" t="n">
-        <v>327900.5</v>
+        <v>403921</v>
       </c>
       <c r="Q184" t="n">
-        <v>9520.299999999999</v>
+        <v>9553.6</v>
       </c>
       <c r="R184" t="n">
-        <v>235092.6</v>
+        <v>365466.5</v>
       </c>
       <c r="S184" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T184" t="n">
-        <v>18841732</v>
+        <v>23599915</v>
       </c>
       <c r="U184" t="n">
-        <v>23557936</v>
+        <v>23599915</v>
       </c>
       <c r="V184" t="n">
         <v>1830000</v>
       </c>
       <c r="W184" t="n">
-        <v>19.16</v>
+        <v>26.08</v>
       </c>
       <c r="X184" t="n">
-        <v>46.523</v>
+        <v>46.608</v>
       </c>
       <c r="Y184" t="n">
         <v>8609304</v>
@@ -15459,34 +15459,34 @@
         <v>25.1</v>
       </c>
       <c r="O185" t="n">
-        <v>2673.4</v>
+        <v>2687.2</v>
       </c>
       <c r="P185" t="n">
-        <v>328021.4</v>
+        <v>404041.9</v>
       </c>
       <c r="Q185" t="n">
-        <v>9520.299999999999</v>
+        <v>9553.6</v>
       </c>
       <c r="R185" t="n">
-        <v>235291.5</v>
+        <v>365665.4</v>
       </c>
       <c r="S185" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T185" t="n">
-        <v>23578764</v>
+        <v>30010014</v>
       </c>
       <c r="U185" t="n">
-        <v>28294968</v>
+        <v>30010014</v>
       </c>
       <c r="V185" t="n">
         <v>1840000</v>
       </c>
       <c r="W185" t="n">
-        <v>20.07</v>
+        <v>27.12</v>
       </c>
       <c r="X185" t="n">
-        <v>55.859</v>
+        <v>59.248</v>
       </c>
       <c r="Y185" t="n">
         <v>9169070</v>
@@ -15540,37 +15540,37 @@
         <v>24.97</v>
       </c>
       <c r="O186" t="n">
-        <v>2673.4</v>
+        <v>2687.2</v>
       </c>
       <c r="P186" t="n">
-        <v>328135.1</v>
+        <v>404155.6</v>
       </c>
       <c r="Q186" t="n">
-        <v>9520.299999999999</v>
+        <v>9553.6</v>
       </c>
       <c r="R186" t="n">
-        <v>235491.6</v>
+        <v>365865.5</v>
       </c>
       <c r="S186" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T186" t="n">
-        <v>24538684</v>
+        <v>31150711</v>
       </c>
       <c r="U186" t="n">
-        <v>29254888</v>
+        <v>31150711</v>
       </c>
       <c r="V186" t="n">
         <v>1850000</v>
       </c>
       <c r="W186" t="n">
-        <v>3.36</v>
+        <v>3.77</v>
       </c>
       <c r="X186" t="n">
-        <v>57.734</v>
+        <v>61.48</v>
       </c>
       <c r="Y186" t="n">
-        <v>9401289</v>
+        <v>9401290</v>
       </c>
     </row>
     <row r="187">
@@ -15621,37 +15621,37 @@
         <v>26.03</v>
       </c>
       <c r="O187" t="n">
-        <v>2673.4</v>
+        <v>2687.2</v>
       </c>
       <c r="P187" t="n">
-        <v>328247.4</v>
+        <v>404267.8</v>
       </c>
       <c r="Q187" t="n">
-        <v>9520.299999999999</v>
+        <v>9553.6</v>
       </c>
       <c r="R187" t="n">
-        <v>235683.4</v>
+        <v>366057.3</v>
       </c>
       <c r="S187" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T187" t="n">
-        <v>25014801</v>
+        <v>31808639</v>
       </c>
       <c r="U187" t="n">
-        <v>29731005</v>
+        <v>31808639</v>
       </c>
       <c r="V187" t="n">
         <v>1860000</v>
       </c>
       <c r="W187" t="n">
-        <v>1.59</v>
+        <v>2.08</v>
       </c>
       <c r="X187" t="n">
-        <v>58.654</v>
+        <v>62.759</v>
       </c>
       <c r="Y187" t="n">
-        <v>9500965</v>
+        <v>9500966</v>
       </c>
     </row>
     <row r="188">
@@ -15702,34 +15702,34 @@
         <v>34.84</v>
       </c>
       <c r="O188" t="n">
-        <v>2673.4</v>
+        <v>2687.2</v>
       </c>
       <c r="P188" t="n">
-        <v>328344.3</v>
+        <v>404364.8</v>
       </c>
       <c r="Q188" t="n">
-        <v>9520.299999999999</v>
+        <v>9553.6</v>
       </c>
       <c r="R188" t="n">
-        <v>235826.8</v>
+        <v>366200.7</v>
       </c>
       <c r="S188" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T188" t="n">
-        <v>29835459</v>
+        <v>38314372</v>
       </c>
       <c r="U188" t="n">
-        <v>34551663</v>
+        <v>38314372</v>
       </c>
       <c r="V188" t="n">
         <v>1870000</v>
       </c>
       <c r="W188" t="n">
-        <v>16.18</v>
+        <v>20.42</v>
       </c>
       <c r="X188" t="n">
-        <v>68.14400000000001</v>
+        <v>75.575</v>
       </c>
       <c r="Y188" t="n">
         <v>10021748</v>
@@ -15783,34 +15783,34 @@
         <v>47.78</v>
       </c>
       <c r="O189" t="n">
-        <v>2673.4</v>
+        <v>2687.2</v>
       </c>
       <c r="P189" t="n">
-        <v>328430.2</v>
+        <v>404450.6</v>
       </c>
       <c r="Q189" t="n">
-        <v>9520.299999999999</v>
+        <v>9553.6</v>
       </c>
       <c r="R189" t="n">
-        <v>235931.3</v>
+        <v>366305.2</v>
       </c>
       <c r="S189" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T189" t="n">
-        <v>35501261</v>
+        <v>46173491</v>
       </c>
       <c r="U189" t="n">
-        <v>40217466</v>
+        <v>46173491</v>
       </c>
       <c r="V189" t="n">
         <v>1880000</v>
       </c>
       <c r="W189" t="n">
-        <v>16.37</v>
+        <v>20.49</v>
       </c>
       <c r="X189" t="n">
-        <v>79.29900000000001</v>
+        <v>91.057</v>
       </c>
       <c r="Y189" t="n">
         <v>10510816</v>
@@ -15864,34 +15864,34 @@
         <v>41.26</v>
       </c>
       <c r="O190" t="n">
-        <v>2673.4</v>
+        <v>2687.2</v>
       </c>
       <c r="P190" t="n">
-        <v>328522</v>
+        <v>404542.5</v>
       </c>
       <c r="Q190" t="n">
-        <v>9520.299999999999</v>
+        <v>9553.6</v>
       </c>
       <c r="R190" t="n">
-        <v>236052.4</v>
+        <v>366426.3</v>
       </c>
       <c r="S190" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T190" t="n">
-        <v>32594288</v>
+        <v>42126524</v>
       </c>
       <c r="U190" t="n">
-        <v>37310492</v>
+        <v>42126524</v>
       </c>
       <c r="V190" t="n">
         <v>1890000</v>
       </c>
       <c r="W190" t="n">
-        <v>-7.25</v>
+        <v>-8.789999999999999</v>
       </c>
       <c r="X190" t="n">
-        <v>73.548</v>
+        <v>83.057</v>
       </c>
       <c r="Y190" t="n">
         <v>10356729</v>
@@ -15945,34 +15945,34 @@
         <v>42.03</v>
       </c>
       <c r="O191" t="n">
-        <v>2673.4</v>
+        <v>2687.2</v>
       </c>
       <c r="P191" t="n">
-        <v>328616.9</v>
+        <v>404637.4</v>
       </c>
       <c r="Q191" t="n">
-        <v>9520.299999999999</v>
+        <v>9553.6</v>
       </c>
       <c r="R191" t="n">
-        <v>236171.2</v>
+        <v>366545.2</v>
       </c>
       <c r="S191" t="n">
-        <v>4716204</v>
+        <v>0</v>
       </c>
       <c r="T191" t="n">
-        <v>32291157</v>
+        <v>41792364</v>
       </c>
       <c r="U191" t="n">
-        <v>37007361</v>
+        <v>41792364</v>
       </c>
       <c r="V191" t="n">
         <v>1900000</v>
       </c>
       <c r="W191" t="n">
-        <v>-0.84</v>
+        <v>-0.82</v>
       </c>
       <c r="X191" t="n">
-        <v>72.93000000000001</v>
+        <v>82.378</v>
       </c>
       <c r="Y191" t="n">
         <v>10297336</v>
@@ -16008,10 +16008,10 @@
         <v>5000</v>
       </c>
       <c r="I192" t="n">
-        <v>1771602</v>
+        <v>0</v>
       </c>
       <c r="J192" t="n">
-        <v>2918604</v>
+        <v>0</v>
       </c>
       <c r="K192" t="n">
         <v>621.09</v>
@@ -16026,34 +16026,34 @@
         <v>61.79</v>
       </c>
       <c r="O192" t="n">
-        <v>2673.4</v>
+        <v>2687.2</v>
       </c>
       <c r="P192" t="n">
-        <v>295847.9</v>
+        <v>404730.1</v>
       </c>
       <c r="Q192" t="n">
-        <v>9520.299999999999</v>
+        <v>9553.6</v>
       </c>
       <c r="R192" t="n">
-        <v>189017.8</v>
+        <v>366626</v>
       </c>
       <c r="S192" t="n">
-        <v>9401721</v>
+        <v>0</v>
       </c>
       <c r="T192" t="n">
-        <v>33130320</v>
+        <v>49996612</v>
       </c>
       <c r="U192" t="n">
-        <v>42532041</v>
+        <v>49996612</v>
       </c>
       <c r="V192" t="n">
         <v>1910000</v>
       </c>
       <c r="W192" t="n">
-        <v>14.91</v>
+        <v>19.61</v>
       </c>
       <c r="X192" t="n">
-        <v>83.807</v>
+        <v>98.53</v>
       </c>
       <c r="Y192" t="n">
         <v>10434050</v>
@@ -16107,34 +16107,34 @@
         <v>62.77</v>
       </c>
       <c r="O193" t="n">
-        <v>2673.4</v>
+        <v>2687.2</v>
       </c>
       <c r="P193" t="n">
-        <v>295948.9</v>
+        <v>404831.1</v>
       </c>
       <c r="Q193" t="n">
-        <v>9520.299999999999</v>
+        <v>9553.6</v>
       </c>
       <c r="R193" t="n">
-        <v>189097.4</v>
+        <v>366705.6</v>
       </c>
       <c r="S193" t="n">
-        <v>9401721</v>
+        <v>0</v>
       </c>
       <c r="T193" t="n">
-        <v>31991112</v>
+        <v>48544370</v>
       </c>
       <c r="U193" t="n">
-        <v>41392833</v>
+        <v>48544370</v>
       </c>
       <c r="V193" t="n">
         <v>1920000</v>
       </c>
       <c r="W193" t="n">
-        <v>-2.7</v>
+        <v>-2.92</v>
       </c>
       <c r="X193" t="n">
-        <v>81.54300000000001</v>
+        <v>95.648</v>
       </c>
       <c r="Y193" t="n">
         <v>10199409</v>
@@ -16188,34 +16188,34 @@
         <v>47.91</v>
       </c>
       <c r="O194" t="n">
-        <v>2682.1</v>
+        <v>2695.8</v>
       </c>
       <c r="P194" t="n">
-        <v>295948.9</v>
+        <v>404831.1</v>
       </c>
       <c r="Q194" t="n">
-        <v>9533.299999999999</v>
+        <v>9566.6</v>
       </c>
       <c r="R194" t="n">
-        <v>189097.4</v>
+        <v>366705.6</v>
       </c>
       <c r="S194" t="n">
-        <v>9401721</v>
+        <v>0</v>
       </c>
       <c r="T194" t="n">
-        <v>26597931</v>
+        <v>39666028</v>
       </c>
       <c r="U194" t="n">
-        <v>35999652</v>
+        <v>39666028</v>
       </c>
       <c r="V194" t="n">
         <v>1930000</v>
       </c>
       <c r="W194" t="n">
-        <v>-13.05</v>
+        <v>-18.31</v>
       </c>
       <c r="X194" t="n">
-        <v>70.899</v>
+        <v>78.13500000000001</v>
       </c>
       <c r="Y194" t="n">
         <v>9715926</v>
@@ -16269,34 +16269,34 @@
         <v>126.98</v>
       </c>
       <c r="O195" t="n">
-        <v>2682.1</v>
+        <v>2695.8</v>
       </c>
       <c r="P195" t="n">
-        <v>296027.6</v>
+        <v>404909.7</v>
       </c>
       <c r="Q195" t="n">
-        <v>9533.299999999999</v>
+        <v>9566.6</v>
       </c>
       <c r="R195" t="n">
-        <v>189136.7</v>
+        <v>366744.9</v>
       </c>
       <c r="S195" t="n">
-        <v>9401721</v>
+        <v>0</v>
       </c>
       <c r="T195" t="n">
-        <v>49447838</v>
+        <v>78944923</v>
       </c>
       <c r="U195" t="n">
-        <v>58849559</v>
+        <v>78944923</v>
       </c>
       <c r="V195" t="n">
         <v>1940000</v>
       </c>
       <c r="W195" t="n">
-        <v>63.44</v>
+        <v>99</v>
       </c>
       <c r="X195" t="n">
-        <v>115.88</v>
+        <v>155.489</v>
       </c>
       <c r="Y195" t="n">
         <v>11250353</v>
@@ -16320,22 +16320,22 @@
         <v>10000</v>
       </c>
       <c r="E196" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="F196" t="n">
         <v>0</v>
       </c>
       <c r="G196" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="H196" t="n">
         <v>0</v>
       </c>
       <c r="I196" t="n">
-        <v>2503209</v>
+        <v>0</v>
       </c>
       <c r="J196" t="n">
-        <v>8486187</v>
+        <v>0</v>
       </c>
       <c r="K196" t="n">
         <v>738.3099999999999</v>
@@ -16350,34 +16350,34 @@
         <v>224.34</v>
       </c>
       <c r="O196" t="n">
-        <v>2682.1</v>
+        <v>2702.6</v>
       </c>
       <c r="P196" t="n">
-        <v>266424.8</v>
+        <v>404909.7</v>
       </c>
       <c r="Q196" t="n">
-        <v>9533.299999999999</v>
+        <v>9574.9</v>
       </c>
       <c r="R196" t="n">
-        <v>151309.4</v>
+        <v>366744.9</v>
       </c>
       <c r="S196" t="n">
-        <v>20390127</v>
+        <v>0</v>
       </c>
       <c r="T196" t="n">
-        <v>64163636</v>
+        <v>124244775</v>
       </c>
       <c r="U196" t="n">
-        <v>84553763</v>
+        <v>124244775</v>
       </c>
       <c r="V196" t="n">
         <v>1950000</v>
       </c>
       <c r="W196" t="n">
-        <v>43.68</v>
+        <v>57.37</v>
       </c>
       <c r="X196" t="n">
-        <v>166.496</v>
+        <v>244.691</v>
       </c>
       <c r="Y196" t="n">
         <v>12449335</v>
@@ -16413,10 +16413,10 @@
         <v>0</v>
       </c>
       <c r="I197" t="n">
-        <v>1946233</v>
+        <v>0</v>
       </c>
       <c r="J197" t="n">
-        <v>5524003</v>
+        <v>0</v>
       </c>
       <c r="K197" t="n">
         <v>705.0599999999999</v>
@@ -16431,34 +16431,34 @@
         <v>182.54</v>
       </c>
       <c r="O197" t="n">
-        <v>2689.2</v>
+        <v>2709.7</v>
       </c>
       <c r="P197" t="n">
-        <v>239782.3</v>
+        <v>404909.7</v>
       </c>
       <c r="Q197" t="n">
-        <v>9542.1</v>
+        <v>9583.700000000001</v>
       </c>
       <c r="R197" t="n">
-        <v>121047.5</v>
+        <v>366744.9</v>
       </c>
       <c r="S197" t="n">
-        <v>27852894</v>
+        <v>0</v>
       </c>
       <c r="T197" t="n">
-        <v>46944174</v>
+        <v>103894486</v>
       </c>
       <c r="U197" t="n">
-        <v>74797068</v>
+        <v>103894486</v>
       </c>
       <c r="V197" t="n">
         <v>1960000</v>
       </c>
       <c r="W197" t="n">
-        <v>-11.54</v>
+        <v>-16.39</v>
       </c>
       <c r="X197" t="n">
-        <v>147.279</v>
+        <v>204.593</v>
       </c>
       <c r="Y197" t="n">
         <v>11898665</v>
@@ -16582,7 +16582,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$74,797,068</t>
+          <t>$103,894,486</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -16592,17 +16592,17 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>$101,660,685</t>
+          <t>$101,660,684</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>$34,886,610</t>
+          <t>$34,886,609</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>$205,415,389</t>
+          <t>$205,415,386</t>
         </is>
       </c>
     </row>
@@ -16614,7 +16614,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$72,837,068</t>
+          <t>$101,934,486</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -16624,17 +16624,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>$99,700,685</t>
+          <t>$99,700,684</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>$32,926,610</t>
+          <t>$32,926,609</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>$203,455,389</t>
+          <t>$203,455,386</t>
         </is>
       </c>
     </row>
@@ -16646,7 +16646,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>38.16x</t>
+          <t>53.01x</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -16678,7 +16678,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>36.0%/yr</t>
+          <t>38.7%/yr</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -16710,7 +16710,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>38.3%/yr</t>
+          <t>41.8%/yr</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -16742,7 +16742,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0.86</t>
+          <t>0.84</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -16806,7 +16806,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0.94</t>
+          <t>0.98</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -16838,7 +16838,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>-75.4%</t>
+          <t>-80.3%</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -16902,7 +16902,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>63.4%</t>
+          <t>99.0%</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -17031,7 +17031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17053,142 +17053,154 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Contributions</t>
+          <t>Mode</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Flat $10,000/month DCA, identical for strategy and benchmark.</t>
+          <t>APPLES-TO-APPLES: always fully invested — no cash, no profit-taking sells — so it is directly comparable to fully-invested Buy &amp; Hold.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fear II reserve</t>
+          <t>Contributions</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cash saved in euphoria + profit-taking trims is deployed into TQQQ/SOXL during Fear II.</t>
+          <t>Flat $10,000/month DCA, identical for strategy and every benchmark.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Euphoria</t>
+          <t>Allocation</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Euphoria months route the contribution to cash (pause), not the market.</t>
+          <t>Each month the full contribution buys the regime's target ETFs: bull/fear1/fear2 -&gt; TQQQ+SOXL; chop -&gt; QQQ+SMH.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Profit-taking</t>
+          <t>Euphoria</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Live evaluate(): CAUTION trims 20% SOXL + 10% TQQQ; EXTREME trims 50%/50%. Proceeds to cash.</t>
+          <t>Euphoria deploys into the defensive unleveraged sleeve (QQQ+SMH) instead of holding cash — stays fully invested.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Benchmark</t>
+          <t>Profit-taking</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Buy &amp; Hold = same $/month into 100% QQQ, never sold.</t>
+          <t>Disabled in this comparison (the alert is still shown for context but triggers no sells).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Investment Sharpe</t>
+          <t>Benchmark</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Annualized Sharpe of monthly time-weighted returns, EQUAL-weighted (pure strategy skill).</t>
+          <t>Buy &amp; Hold = same $/month into 100% of one ETF, never sold.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Contribution Sharpe</t>
+          <t>Investment Sharpe</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Same monthly returns but CAPITAL-weighted by dollars deployed — the 'growth of the asset' view.</t>
+          <t>Annualized Sharpe of monthly time-weighted returns, EQUAL-weighted (pure strategy skill).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TWR vs IRR</t>
+          <t>Contribution Sharpe</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TWR = cash-flow-neutral strategy return. IRR = money-weighted, reflects contribution timing.</t>
+          <t>Same monthly returns but CAPITAL-weighted by dollars deployed — the 'growth of the asset' view.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Max drawdown</t>
+          <t>TWR vs IRR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Computed on the time-weighted return index (contribution-neutral), so it's the true investment drawdown.</t>
+          <t>TWR = cash-flow-neutral strategy return. IRR = money-weighted, reflects contribution timing.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Risk-free</t>
+          <t>Max drawdown</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0% (cash earns 0 in this model). Sharpe = excess over this.</t>
+          <t>Computed on the time-weighted return index (contribution-neutral), so it's the true investment drawdown.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Transaction cost</t>
+          <t>Risk-free</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0.1% per trade (slippage).</t>
+          <t>0% (cash earns 0 in this model). Sharpe = excess over this.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Transaction cost</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0.1% per trade (slippage).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>P/E signal</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>QQQ P/E is unavailable historically, so the profit-taking monitor runs on its other 6 signals (incl. CAPE).</t>
         </is>

</xml_diff>

<commit_message>
Backtest: add portfolio composition (% allocation) stacked-area chart
</commit_message>
<xml_diff>
--- a/backtest.xlsx
+++ b/backtest.xlsx
@@ -2676,10 +2676,10 @@
         <v>0</v>
       </c>
       <c r="T27" t="n">
-        <v>313159</v>
+        <v>313160</v>
       </c>
       <c r="U27" t="n">
-        <v>313159</v>
+        <v>313160</v>
       </c>
       <c r="V27" t="n">
         <v>260000</v>
@@ -3009,7 +3009,7 @@
         <v>300000</v>
       </c>
       <c r="W31" t="n">
-        <v>7.93</v>
+        <v>7.94</v>
       </c>
       <c r="X31" t="n">
         <v>1.357</v>
@@ -3312,7 +3312,7 @@
         <v>1744.2</v>
       </c>
       <c r="P35" t="n">
-        <v>207458.2</v>
+        <v>207458.3</v>
       </c>
       <c r="Q35" t="n">
         <v>6375.7</v>
@@ -3486,10 +3486,10 @@
         <v>0</v>
       </c>
       <c r="T37" t="n">
-        <v>434750</v>
+        <v>434751</v>
       </c>
       <c r="U37" t="n">
-        <v>434750</v>
+        <v>434751</v>
       </c>
       <c r="V37" t="n">
         <v>360000</v>
@@ -3561,7 +3561,7 @@
         <v>6375.7</v>
       </c>
       <c r="R38" t="n">
-        <v>198183.2</v>
+        <v>198183.3</v>
       </c>
       <c r="S38" t="n">
         <v>0</v>
@@ -3987,7 +3987,7 @@
         <v>1.721</v>
       </c>
       <c r="Y43" t="n">
-        <v>551360</v>
+        <v>551361</v>
       </c>
     </row>
     <row r="44">
@@ -4215,10 +4215,10 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>798004</v>
+        <v>798005</v>
       </c>
       <c r="U46" t="n">
-        <v>798004</v>
+        <v>798005</v>
       </c>
       <c r="V46" t="n">
         <v>450000</v>
@@ -4635,7 +4635,7 @@
         <v>2.608</v>
       </c>
       <c r="Y51" t="n">
-        <v>728449</v>
+        <v>728448</v>
       </c>
     </row>
     <row r="52">
@@ -4959,7 +4959,7 @@
         <v>3.558</v>
       </c>
       <c r="Y55" t="n">
-        <v>876002</v>
+        <v>876003</v>
       </c>
     </row>
     <row r="56">
@@ -5268,10 +5268,10 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>1561240</v>
+        <v>1561239</v>
       </c>
       <c r="U59" t="n">
-        <v>1561240</v>
+        <v>1561239</v>
       </c>
       <c r="V59" t="n">
         <v>580000</v>
@@ -5526,7 +5526,7 @@
         <v>4.049</v>
       </c>
       <c r="Y62" t="n">
-        <v>1006576</v>
+        <v>1006577</v>
       </c>
     </row>
     <row r="63">
@@ -5607,7 +5607,7 @@
         <v>4.082</v>
       </c>
       <c r="Y63" t="n">
-        <v>1035917</v>
+        <v>1035916</v>
       </c>
     </row>
     <row r="64">
@@ -5688,7 +5688,7 @@
         <v>4.634</v>
       </c>
       <c r="Y64" t="n">
-        <v>1069198</v>
+        <v>1069199</v>
       </c>
     </row>
     <row r="65">
@@ -6645,10 +6645,10 @@
         <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>1726274</v>
+        <v>1726273</v>
       </c>
       <c r="U76" t="n">
-        <v>1726274</v>
+        <v>1726273</v>
       </c>
       <c r="V76" t="n">
         <v>750000</v>
@@ -6660,7 +6660,7 @@
         <v>3.902</v>
       </c>
       <c r="Y76" t="n">
-        <v>1206766</v>
+        <v>1206765</v>
       </c>
     </row>
     <row r="77">
@@ -6822,7 +6822,7 @@
         <v>4.553</v>
       </c>
       <c r="Y78" t="n">
-        <v>1284298</v>
+        <v>1284297</v>
       </c>
     </row>
     <row r="79">
@@ -6969,10 +6969,10 @@
         <v>0</v>
       </c>
       <c r="T80" t="n">
-        <v>2371549</v>
+        <v>2371550</v>
       </c>
       <c r="U80" t="n">
-        <v>2371549</v>
+        <v>2371550</v>
       </c>
       <c r="V80" t="n">
         <v>790000</v>
@@ -6984,7 +6984,7 @@
         <v>5.255</v>
       </c>
       <c r="Y80" t="n">
-        <v>1346711</v>
+        <v>1346712</v>
       </c>
     </row>
     <row r="81">
@@ -7065,7 +7065,7 @@
         <v>5.04</v>
       </c>
       <c r="Y81" t="n">
-        <v>1337078</v>
+        <v>1337077</v>
       </c>
     </row>
     <row r="82">
@@ -7146,7 +7146,7 @@
         <v>5.53</v>
       </c>
       <c r="Y82" t="n">
-        <v>1352896</v>
+        <v>1352897</v>
       </c>
     </row>
     <row r="83">
@@ -7470,7 +7470,7 @@
         <v>7.683</v>
       </c>
       <c r="Y86" t="n">
-        <v>1573918</v>
+        <v>1573917</v>
       </c>
     </row>
     <row r="87">
@@ -7611,7 +7611,7 @@
         <v>7882.7</v>
       </c>
       <c r="R88" t="n">
-        <v>342207.5</v>
+        <v>342207.6</v>
       </c>
       <c r="S88" t="n">
         <v>0</v>
@@ -7632,7 +7632,7 @@
         <v>9.215999999999999</v>
       </c>
       <c r="Y88" t="n">
-        <v>1700221</v>
+        <v>1700222</v>
       </c>
     </row>
     <row r="89">
@@ -7698,10 +7698,10 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>3798193</v>
+        <v>3798192</v>
       </c>
       <c r="U89" t="n">
-        <v>3798193</v>
+        <v>3798192</v>
       </c>
       <c r="V89" t="n">
         <v>880000</v>
@@ -7713,7 +7713,7 @@
         <v>8.175000000000001</v>
       </c>
       <c r="Y89" t="n">
-        <v>1670802</v>
+        <v>1670801</v>
       </c>
     </row>
     <row r="90">
@@ -7794,7 +7794,7 @@
         <v>9.17</v>
       </c>
       <c r="Y90" t="n">
-        <v>1748648</v>
+        <v>1748647</v>
       </c>
     </row>
     <row r="91">
@@ -7854,16 +7854,16 @@
         <v>7882.7</v>
       </c>
       <c r="R91" t="n">
-        <v>344800.6</v>
+        <v>344800.7</v>
       </c>
       <c r="S91" t="n">
         <v>0</v>
       </c>
       <c r="T91" t="n">
-        <v>4529336</v>
+        <v>4529337</v>
       </c>
       <c r="U91" t="n">
-        <v>4529336</v>
+        <v>4529337</v>
       </c>
       <c r="V91" t="n">
         <v>900000</v>
@@ -7935,7 +7935,7 @@
         <v>7882.7</v>
       </c>
       <c r="R92" t="n">
-        <v>345482.4</v>
+        <v>345482.5</v>
       </c>
       <c r="S92" t="n">
         <v>0</v>
@@ -8022,10 +8022,10 @@
         <v>0</v>
       </c>
       <c r="T93" t="n">
-        <v>5877481</v>
+        <v>5877482</v>
       </c>
       <c r="U93" t="n">
-        <v>5877481</v>
+        <v>5877482</v>
       </c>
       <c r="V93" t="n">
         <v>920000</v>
@@ -8037,7 +8037,7 @@
         <v>12.545</v>
       </c>
       <c r="Y93" t="n">
-        <v>1892474</v>
+        <v>1892475</v>
       </c>
     </row>
     <row r="94">
@@ -8103,10 +8103,10 @@
         <v>0</v>
       </c>
       <c r="T94" t="n">
-        <v>5946259</v>
+        <v>5946258</v>
       </c>
       <c r="U94" t="n">
-        <v>5946259</v>
+        <v>5946258</v>
       </c>
       <c r="V94" t="n">
         <v>930000</v>
@@ -8184,10 +8184,10 @@
         <v>0</v>
       </c>
       <c r="T95" t="n">
-        <v>5809422</v>
+        <v>5809421</v>
       </c>
       <c r="U95" t="n">
-        <v>5809422</v>
+        <v>5809421</v>
       </c>
       <c r="V95" t="n">
         <v>940000</v>
@@ -8199,7 +8199,7 @@
         <v>12.358</v>
       </c>
       <c r="Y95" t="n">
-        <v>1961468</v>
+        <v>1961469</v>
       </c>
     </row>
     <row r="96">
@@ -8280,7 +8280,7 @@
         <v>15.409</v>
       </c>
       <c r="Y96" t="n">
-        <v>2143225</v>
+        <v>2143226</v>
       </c>
     </row>
     <row r="97">
@@ -8361,7 +8361,7 @@
         <v>14.815</v>
       </c>
       <c r="Y97" t="n">
-        <v>2125508</v>
+        <v>2125507</v>
       </c>
     </row>
     <row r="98">
@@ -8427,10 +8427,10 @@
         <v>0</v>
       </c>
       <c r="T98" t="n">
-        <v>6277670</v>
+        <v>6277672</v>
       </c>
       <c r="U98" t="n">
-        <v>6277670</v>
+        <v>6277672</v>
       </c>
       <c r="V98" t="n">
         <v>970000</v>
@@ -8508,10 +8508,10 @@
         <v>0</v>
       </c>
       <c r="T99" t="n">
-        <v>5568499</v>
+        <v>5568498</v>
       </c>
       <c r="U99" t="n">
-        <v>5568499</v>
+        <v>5568498</v>
       </c>
       <c r="V99" t="n">
         <v>980000</v>
@@ -8685,7 +8685,7 @@
         <v>13.697</v>
       </c>
       <c r="Y101" t="n">
-        <v>2231668</v>
+        <v>2231669</v>
       </c>
     </row>
     <row r="102">
@@ -8913,10 +8913,10 @@
         <v>0</v>
       </c>
       <c r="T104" t="n">
-        <v>7517179</v>
+        <v>7517180</v>
       </c>
       <c r="U104" t="n">
-        <v>7517179</v>
+        <v>7517180</v>
       </c>
       <c r="V104" t="n">
         <v>1030000</v>
@@ -9075,10 +9075,10 @@
         <v>0</v>
       </c>
       <c r="T106" t="n">
-        <v>5453668</v>
+        <v>5453669</v>
       </c>
       <c r="U106" t="n">
-        <v>5453668</v>
+        <v>5453669</v>
       </c>
       <c r="V106" t="n">
         <v>1050000</v>
@@ -9090,7 +9090,7 @@
         <v>11.407</v>
       </c>
       <c r="Y106" t="n">
-        <v>2253737</v>
+        <v>2253736</v>
       </c>
     </row>
     <row r="107">
@@ -9156,10 +9156,10 @@
         <v>0</v>
       </c>
       <c r="T107" t="n">
-        <v>4252567</v>
+        <v>4252568</v>
       </c>
       <c r="U107" t="n">
-        <v>4252567</v>
+        <v>4252568</v>
       </c>
       <c r="V107" t="n">
         <v>1060000</v>
@@ -9225,7 +9225,7 @@
         <v>2168.3</v>
       </c>
       <c r="P108" t="n">
-        <v>388478.8</v>
+        <v>388478.9</v>
       </c>
       <c r="Q108" t="n">
         <v>8118</v>
@@ -9252,7 +9252,7 @@
         <v>11.061</v>
       </c>
       <c r="Y108" t="n">
-        <v>2264918</v>
+        <v>2264917</v>
       </c>
     </row>
     <row r="109">
@@ -9414,7 +9414,7 @@
         <v>13.603</v>
       </c>
       <c r="Y110" t="n">
-        <v>2444586</v>
+        <v>2444585</v>
       </c>
     </row>
     <row r="111">
@@ -9474,16 +9474,16 @@
         <v>8118</v>
       </c>
       <c r="R111" t="n">
-        <v>354751.2</v>
+        <v>354751.3</v>
       </c>
       <c r="S111" t="n">
         <v>0</v>
       </c>
       <c r="T111" t="n">
-        <v>8210213</v>
+        <v>8210212</v>
       </c>
       <c r="U111" t="n">
-        <v>8210213</v>
+        <v>8210212</v>
       </c>
       <c r="V111" t="n">
         <v>1100000</v>
@@ -9642,10 +9642,10 @@
         <v>0</v>
       </c>
       <c r="T113" t="n">
-        <v>7101969</v>
+        <v>7101970</v>
       </c>
       <c r="U113" t="n">
-        <v>7101969</v>
+        <v>7101970</v>
       </c>
       <c r="V113" t="n">
         <v>1120000</v>
@@ -9657,7 +9657,7 @@
         <v>14.679</v>
       </c>
       <c r="Y113" t="n">
-        <v>2577141</v>
+        <v>2577142</v>
       </c>
     </row>
     <row r="114">
@@ -9723,10 +9723,10 @@
         <v>0</v>
       </c>
       <c r="T114" t="n">
-        <v>7877044</v>
+        <v>7877042</v>
       </c>
       <c r="U114" t="n">
-        <v>7877044</v>
+        <v>7877042</v>
       </c>
       <c r="V114" t="n">
         <v>1130000</v>
@@ -9738,7 +9738,7 @@
         <v>16.261</v>
       </c>
       <c r="Y114" t="n">
-        <v>2647303</v>
+        <v>2647302</v>
       </c>
     </row>
     <row r="115">
@@ -9804,10 +9804,10 @@
         <v>0</v>
       </c>
       <c r="T115" t="n">
-        <v>7231597</v>
+        <v>7231596</v>
       </c>
       <c r="U115" t="n">
-        <v>7231597</v>
+        <v>7231596</v>
       </c>
       <c r="V115" t="n">
         <v>1140000</v>
@@ -9819,7 +9819,7 @@
         <v>14.907</v>
       </c>
       <c r="Y115" t="n">
-        <v>2607006</v>
+        <v>2607007</v>
       </c>
     </row>
     <row r="116">
@@ -9885,10 +9885,10 @@
         <v>0</v>
       </c>
       <c r="T116" t="n">
-        <v>7674557</v>
+        <v>7674558</v>
       </c>
       <c r="U116" t="n">
-        <v>7674557</v>
+        <v>7674558</v>
       </c>
       <c r="V116" t="n">
         <v>1150000</v>
@@ -9966,10 +9966,10 @@
         <v>0</v>
       </c>
       <c r="T117" t="n">
-        <v>8740737</v>
+        <v>8740736</v>
       </c>
       <c r="U117" t="n">
-        <v>8740737</v>
+        <v>8740736</v>
       </c>
       <c r="V117" t="n">
         <v>1160000</v>
@@ -9981,7 +9981,7 @@
         <v>17.974</v>
       </c>
       <c r="Y117" t="n">
-        <v>2766589</v>
+        <v>2766590</v>
       </c>
     </row>
     <row r="118">
@@ -10047,10 +10047,10 @@
         <v>0</v>
       </c>
       <c r="T118" t="n">
-        <v>9720973</v>
+        <v>9720972</v>
       </c>
       <c r="U118" t="n">
-        <v>9720973</v>
+        <v>9720972</v>
       </c>
       <c r="V118" t="n">
         <v>1170000</v>
@@ -10128,10 +10128,10 @@
         <v>0</v>
       </c>
       <c r="T119" t="n">
-        <v>11444853</v>
+        <v>11444851</v>
       </c>
       <c r="U119" t="n">
-        <v>11444853</v>
+        <v>11444851</v>
       </c>
       <c r="V119" t="n">
         <v>1180000</v>
@@ -10290,10 +10290,10 @@
         <v>0</v>
       </c>
       <c r="T121" t="n">
-        <v>9345551</v>
+        <v>9345549</v>
       </c>
       <c r="U121" t="n">
-        <v>9345551</v>
+        <v>9345549</v>
       </c>
       <c r="V121" t="n">
         <v>1200000</v>
@@ -10446,16 +10446,16 @@
         <v>8118</v>
       </c>
       <c r="R123" t="n">
-        <v>360537.9</v>
+        <v>360538</v>
       </c>
       <c r="S123" t="n">
         <v>0</v>
       </c>
       <c r="T123" t="n">
-        <v>7350994</v>
+        <v>7350995</v>
       </c>
       <c r="U123" t="n">
-        <v>7350994</v>
+        <v>7350995</v>
       </c>
       <c r="V123" t="n">
         <v>1220000</v>
@@ -10527,7 +10527,7 @@
         <v>8191.6</v>
       </c>
       <c r="R124" t="n">
-        <v>360537.9</v>
+        <v>360538</v>
       </c>
       <c r="S124" t="n">
         <v>0</v>
@@ -10548,7 +10548,7 @@
         <v>17.49</v>
       </c>
       <c r="Y124" t="n">
-        <v>3367286</v>
+        <v>3367287</v>
       </c>
     </row>
     <row r="125">
@@ -10608,7 +10608,7 @@
         <v>8259.4</v>
       </c>
       <c r="R125" t="n">
-        <v>360537.9</v>
+        <v>360538</v>
       </c>
       <c r="S125" t="n">
         <v>0</v>
@@ -10689,7 +10689,7 @@
         <v>8321.799999999999</v>
       </c>
       <c r="R126" t="n">
-        <v>360537.9</v>
+        <v>360538</v>
       </c>
       <c r="S126" t="n">
         <v>0</v>
@@ -10770,16 +10770,16 @@
         <v>8380.9</v>
       </c>
       <c r="R127" t="n">
-        <v>360537.9</v>
+        <v>360538</v>
       </c>
       <c r="S127" t="n">
         <v>0</v>
       </c>
       <c r="T127" t="n">
-        <v>15247650</v>
+        <v>15247651</v>
       </c>
       <c r="U127" t="n">
-        <v>15247650</v>
+        <v>15247651</v>
       </c>
       <c r="V127" t="n">
         <v>1260000</v>
@@ -10791,7 +10791,7 @@
         <v>31.02</v>
       </c>
       <c r="Y127" t="n">
-        <v>4295365</v>
+        <v>4295364</v>
       </c>
     </row>
     <row r="128">
@@ -10851,16 +10851,16 @@
         <v>8440.4</v>
       </c>
       <c r="R128" t="n">
-        <v>360537.9</v>
+        <v>360538</v>
       </c>
       <c r="S128" t="n">
         <v>0</v>
       </c>
       <c r="T128" t="n">
-        <v>13443231</v>
+        <v>13443232</v>
       </c>
       <c r="U128" t="n">
-        <v>13443231</v>
+        <v>13443232</v>
       </c>
       <c r="V128" t="n">
         <v>1270000</v>
@@ -10872,7 +10872,7 @@
         <v>27.329</v>
       </c>
       <c r="Y128" t="n">
-        <v>4057142</v>
+        <v>4057141</v>
       </c>
     </row>
     <row r="129">
@@ -10932,16 +10932,16 @@
         <v>8499.700000000001</v>
       </c>
       <c r="R129" t="n">
-        <v>360537.9</v>
+        <v>360538</v>
       </c>
       <c r="S129" t="n">
         <v>0</v>
       </c>
       <c r="T129" t="n">
-        <v>12699329</v>
+        <v>12699328</v>
       </c>
       <c r="U129" t="n">
-        <v>12699329</v>
+        <v>12699328</v>
       </c>
       <c r="V129" t="n">
         <v>1280000</v>
@@ -10953,7 +10953,7 @@
         <v>25.797</v>
       </c>
       <c r="Y129" t="n">
-        <v>3943596</v>
+        <v>3943594</v>
       </c>
     </row>
     <row r="130">
@@ -11013,16 +11013,16 @@
         <v>8549.4</v>
       </c>
       <c r="R130" t="n">
-        <v>360537.9</v>
+        <v>360538</v>
       </c>
       <c r="S130" t="n">
         <v>0</v>
       </c>
       <c r="T130" t="n">
-        <v>18502833</v>
+        <v>18502837</v>
       </c>
       <c r="U130" t="n">
-        <v>18502833</v>
+        <v>18502837</v>
       </c>
       <c r="V130" t="n">
         <v>1290000</v>
@@ -11034,7 +11034,7 @@
         <v>37.565</v>
       </c>
       <c r="Y130" t="n">
-        <v>4396283</v>
+        <v>4396284</v>
       </c>
     </row>
     <row r="131">
@@ -11094,16 +11094,16 @@
         <v>8596.5</v>
       </c>
       <c r="R131" t="n">
-        <v>360537.9</v>
+        <v>360538</v>
       </c>
       <c r="S131" t="n">
         <v>0</v>
       </c>
       <c r="T131" t="n">
-        <v>21134547</v>
+        <v>21134549</v>
       </c>
       <c r="U131" t="n">
-        <v>21134547</v>
+        <v>21134549</v>
       </c>
       <c r="V131" t="n">
         <v>1300000</v>
@@ -11115,7 +11115,7 @@
         <v>42.888</v>
       </c>
       <c r="Y131" t="n">
-        <v>4621800</v>
+        <v>4621799</v>
       </c>
     </row>
     <row r="132">
@@ -11175,16 +11175,16 @@
         <v>8642</v>
       </c>
       <c r="R132" t="n">
-        <v>360537.9</v>
+        <v>360538</v>
       </c>
       <c r="S132" t="n">
         <v>0</v>
       </c>
       <c r="T132" t="n">
-        <v>21944520</v>
+        <v>21944519</v>
       </c>
       <c r="U132" t="n">
-        <v>21944520</v>
+        <v>21944519</v>
       </c>
       <c r="V132" t="n">
         <v>1310000</v>
@@ -11196,7 +11196,7 @@
         <v>44.511</v>
       </c>
       <c r="Y132" t="n">
-        <v>4643868</v>
+        <v>4643869</v>
       </c>
     </row>
     <row r="133">
@@ -11256,16 +11256,16 @@
         <v>8684.700000000001</v>
       </c>
       <c r="R133" t="n">
-        <v>360537.9</v>
+        <v>360538</v>
       </c>
       <c r="S133" t="n">
         <v>0</v>
       </c>
       <c r="T133" t="n">
-        <v>23751399</v>
+        <v>23751398</v>
       </c>
       <c r="U133" t="n">
-        <v>23751399</v>
+        <v>23751398</v>
       </c>
       <c r="V133" t="n">
         <v>1320000</v>
@@ -11277,7 +11277,7 @@
         <v>48.156</v>
       </c>
       <c r="Y133" t="n">
-        <v>4647659</v>
+        <v>4647658</v>
       </c>
     </row>
     <row r="134">
@@ -11337,16 +11337,16 @@
         <v>8727</v>
       </c>
       <c r="R134" t="n">
-        <v>360537.9</v>
+        <v>360538</v>
       </c>
       <c r="S134" t="n">
         <v>0</v>
       </c>
       <c r="T134" t="n">
-        <v>23809373</v>
+        <v>23809377</v>
       </c>
       <c r="U134" t="n">
-        <v>23809373</v>
+        <v>23809377</v>
       </c>
       <c r="V134" t="n">
         <v>1330000</v>
@@ -11424,10 +11424,10 @@
         <v>0</v>
       </c>
       <c r="T135" t="n">
-        <v>24961851</v>
+        <v>24961850</v>
       </c>
       <c r="U135" t="n">
-        <v>24961851</v>
+        <v>24961850</v>
       </c>
       <c r="V135" t="n">
         <v>1340000</v>
@@ -11439,7 +11439,7 @@
         <v>50.569</v>
       </c>
       <c r="Y135" t="n">
-        <v>5027403</v>
+        <v>5027402</v>
       </c>
     </row>
     <row r="136">
@@ -11505,10 +11505,10 @@
         <v>0</v>
       </c>
       <c r="T136" t="n">
-        <v>25164174</v>
+        <v>25164171</v>
       </c>
       <c r="U136" t="n">
-        <v>25164174</v>
+        <v>25164171</v>
       </c>
       <c r="V136" t="n">
         <v>1350000</v>
@@ -11520,7 +11520,7 @@
         <v>50.958</v>
       </c>
       <c r="Y136" t="n">
-        <v>4977002</v>
+        <v>4977003</v>
       </c>
     </row>
     <row r="137">
@@ -11586,10 +11586,10 @@
         <v>0</v>
       </c>
       <c r="T137" t="n">
-        <v>29189207</v>
+        <v>29189210</v>
       </c>
       <c r="U137" t="n">
-        <v>29189207</v>
+        <v>29189210</v>
       </c>
       <c r="V137" t="n">
         <v>1360000</v>
@@ -11601,7 +11601,7 @@
         <v>59.089</v>
       </c>
       <c r="Y137" t="n">
-        <v>5298659</v>
+        <v>5298658</v>
       </c>
     </row>
     <row r="138">
@@ -11667,10 +11667,10 @@
         <v>0</v>
       </c>
       <c r="T138" t="n">
-        <v>30149064</v>
+        <v>30149070</v>
       </c>
       <c r="U138" t="n">
-        <v>30149064</v>
+        <v>30149070</v>
       </c>
       <c r="V138" t="n">
         <v>1370000</v>
@@ -11682,7 +11682,7 @@
         <v>61.012</v>
       </c>
       <c r="Y138" t="n">
-        <v>5460241</v>
+        <v>5460240</v>
       </c>
     </row>
     <row r="139">
@@ -11748,10 +11748,10 @@
         <v>0</v>
       </c>
       <c r="T139" t="n">
-        <v>32579500</v>
+        <v>32579498</v>
       </c>
       <c r="U139" t="n">
-        <v>32579500</v>
+        <v>32579498</v>
       </c>
       <c r="V139" t="n">
         <v>1380000</v>
@@ -11763,7 +11763,7 @@
         <v>65.91</v>
       </c>
       <c r="Y139" t="n">
-        <v>5700579</v>
+        <v>5700580</v>
       </c>
     </row>
     <row r="140">
@@ -11829,10 +11829,10 @@
         <v>0</v>
       </c>
       <c r="T140" t="n">
-        <v>27821991</v>
+        <v>27821993</v>
       </c>
       <c r="U140" t="n">
-        <v>27821991</v>
+        <v>27821993</v>
       </c>
       <c r="V140" t="n">
         <v>1390000</v>
@@ -11844,7 +11844,7 @@
         <v>56.265</v>
       </c>
       <c r="Y140" t="n">
-        <v>5386596</v>
+        <v>5386597</v>
       </c>
     </row>
     <row r="141">
@@ -11910,10 +11910,10 @@
         <v>0</v>
       </c>
       <c r="T141" t="n">
-        <v>33553109</v>
+        <v>33553104</v>
       </c>
       <c r="U141" t="n">
-        <v>33553109</v>
+        <v>33553104</v>
       </c>
       <c r="V141" t="n">
         <v>1400000</v>
@@ -11991,10 +11991,10 @@
         <v>0</v>
       </c>
       <c r="T142" t="n">
-        <v>40473534</v>
+        <v>40473531</v>
       </c>
       <c r="U142" t="n">
-        <v>40473534</v>
+        <v>40473531</v>
       </c>
       <c r="V142" t="n">
         <v>1410000</v>
@@ -12006,7 +12006,7 @@
         <v>81.806</v>
       </c>
       <c r="Y142" t="n">
-        <v>5946398</v>
+        <v>5946399</v>
       </c>
     </row>
     <row r="143">
@@ -12072,10 +12072,10 @@
         <v>0</v>
       </c>
       <c r="T143" t="n">
-        <v>41964991</v>
+        <v>41964996</v>
       </c>
       <c r="U143" t="n">
-        <v>41964991</v>
+        <v>41964996</v>
       </c>
       <c r="V143" t="n">
         <v>1420000</v>
@@ -12087,7 +12087,7 @@
         <v>84.8</v>
       </c>
       <c r="Y143" t="n">
-        <v>6024911</v>
+        <v>6024912</v>
       </c>
     </row>
     <row r="144">
@@ -12153,10 +12153,10 @@
         <v>0</v>
       </c>
       <c r="T144" t="n">
-        <v>29465121</v>
+        <v>29465118</v>
       </c>
       <c r="U144" t="n">
-        <v>29465121</v>
+        <v>29465118</v>
       </c>
       <c r="V144" t="n">
         <v>1430000</v>
@@ -12168,7 +12168,7 @@
         <v>59.521</v>
       </c>
       <c r="Y144" t="n">
-        <v>5507901</v>
+        <v>5507902</v>
       </c>
     </row>
     <row r="145">
@@ -12234,10 +12234,10 @@
         <v>0</v>
       </c>
       <c r="T145" t="n">
-        <v>26366601</v>
+        <v>26366603</v>
       </c>
       <c r="U145" t="n">
-        <v>26366601</v>
+        <v>26366603</v>
       </c>
       <c r="V145" t="n">
         <v>1440000</v>
@@ -12249,7 +12249,7 @@
         <v>53.242</v>
       </c>
       <c r="Y145" t="n">
-        <v>5271359</v>
+        <v>5271360</v>
       </c>
     </row>
     <row r="146">
@@ -12315,10 +12315,10 @@
         <v>0</v>
       </c>
       <c r="T146" t="n">
-        <v>26733468</v>
+        <v>26733470</v>
       </c>
       <c r="U146" t="n">
-        <v>26733468</v>
+        <v>26733470</v>
       </c>
       <c r="V146" t="n">
         <v>1450000</v>
@@ -12396,10 +12396,10 @@
         <v>0</v>
       </c>
       <c r="T147" t="n">
-        <v>16522123</v>
+        <v>16522122</v>
       </c>
       <c r="U147" t="n">
-        <v>16522123</v>
+        <v>16522122</v>
       </c>
       <c r="V147" t="n">
         <v>1460000</v>
@@ -12477,10 +12477,10 @@
         <v>0</v>
       </c>
       <c r="T148" t="n">
-        <v>16839658</v>
+        <v>16839659</v>
       </c>
       <c r="U148" t="n">
-        <v>16839658</v>
+        <v>16839659</v>
       </c>
       <c r="V148" t="n">
         <v>1470000</v>
@@ -12492,7 +12492,7 @@
         <v>33.951</v>
       </c>
       <c r="Y148" t="n">
-        <v>4719965</v>
+        <v>4719964</v>
       </c>
     </row>
     <row r="149">
@@ -12558,10 +12558,10 @@
         <v>0</v>
       </c>
       <c r="T149" t="n">
-        <v>10759377</v>
+        <v>10759378</v>
       </c>
       <c r="U149" t="n">
-        <v>10759377</v>
+        <v>10759378</v>
       </c>
       <c r="V149" t="n">
         <v>1480000</v>
@@ -12639,10 +12639,10 @@
         <v>0</v>
       </c>
       <c r="T150" t="n">
-        <v>15151249</v>
+        <v>15151251</v>
       </c>
       <c r="U150" t="n">
-        <v>15151249</v>
+        <v>15151251</v>
       </c>
       <c r="V150" t="n">
         <v>1490000</v>
@@ -12735,7 +12735,7 @@
         <v>23.993</v>
       </c>
       <c r="Y151" t="n">
-        <v>4620957</v>
+        <v>4620958</v>
       </c>
     </row>
     <row r="152">
@@ -12801,10 +12801,10 @@
         <v>0</v>
       </c>
       <c r="T152" t="n">
-        <v>8302176</v>
+        <v>8302175</v>
       </c>
       <c r="U152" t="n">
-        <v>8302176</v>
+        <v>8302175</v>
       </c>
       <c r="V152" t="n">
         <v>1510000</v>
@@ -12882,10 +12882,10 @@
         <v>0</v>
       </c>
       <c r="T153" t="n">
-        <v>8689211</v>
+        <v>8689212</v>
       </c>
       <c r="U153" t="n">
-        <v>8689211</v>
+        <v>8689212</v>
       </c>
       <c r="V153" t="n">
         <v>1520000</v>
@@ -12978,7 +12978,7 @@
         <v>22.324</v>
       </c>
       <c r="Y154" t="n">
-        <v>4569342</v>
+        <v>4569341</v>
       </c>
     </row>
     <row r="155">
@@ -13059,7 +13059,7 @@
         <v>16.72</v>
       </c>
       <c r="Y155" t="n">
-        <v>4167467</v>
+        <v>4167468</v>
       </c>
     </row>
     <row r="156">
@@ -13206,10 +13206,10 @@
         <v>0</v>
       </c>
       <c r="T157" t="n">
-        <v>11294702</v>
+        <v>11294701</v>
       </c>
       <c r="U157" t="n">
-        <v>11294702</v>
+        <v>11294701</v>
       </c>
       <c r="V157" t="n">
         <v>1560000</v>
@@ -13221,7 +13221,7 @@
         <v>22.576</v>
       </c>
       <c r="Y157" t="n">
-        <v>4614362</v>
+        <v>4614363</v>
       </c>
     </row>
     <row r="158">
@@ -13275,7 +13275,7 @@
         <v>2632.1</v>
       </c>
       <c r="P158" t="n">
-        <v>399777.8</v>
+        <v>399777.9</v>
       </c>
       <c r="Q158" t="n">
         <v>9431.200000000001</v>
@@ -13302,7 +13302,7 @@
         <v>27.952</v>
       </c>
       <c r="Y158" t="n">
-        <v>5062381</v>
+        <v>5062382</v>
       </c>
     </row>
     <row r="159">
@@ -13356,13 +13356,13 @@
         <v>2632.1</v>
       </c>
       <c r="P159" t="n">
-        <v>400144</v>
+        <v>400144.1</v>
       </c>
       <c r="Q159" t="n">
         <v>9431.200000000001</v>
       </c>
       <c r="R159" t="n">
-        <v>361972.8</v>
+        <v>361972.9</v>
       </c>
       <c r="S159" t="n">
         <v>0</v>
@@ -13383,7 +13383,7 @@
         <v>24.928</v>
       </c>
       <c r="Y159" t="n">
-        <v>5098083</v>
+        <v>5098082</v>
       </c>
     </row>
     <row r="160">
@@ -13443,16 +13443,16 @@
         <v>9431.200000000001</v>
       </c>
       <c r="R160" t="n">
-        <v>362213.8</v>
+        <v>362213.9</v>
       </c>
       <c r="S160" t="n">
         <v>0</v>
       </c>
       <c r="T160" t="n">
-        <v>16469316</v>
+        <v>16469314</v>
       </c>
       <c r="U160" t="n">
-        <v>16469316</v>
+        <v>16469314</v>
       </c>
       <c r="V160" t="n">
         <v>1590000</v>
@@ -13464,7 +13464,7 @@
         <v>32.849</v>
       </c>
       <c r="Y160" t="n">
-        <v>5509995</v>
+        <v>5509996</v>
       </c>
     </row>
     <row r="161">
@@ -13524,16 +13524,16 @@
         <v>9464.4</v>
       </c>
       <c r="R161" t="n">
-        <v>362213.8</v>
+        <v>362213.9</v>
       </c>
       <c r="S161" t="n">
         <v>0</v>
       </c>
       <c r="T161" t="n">
-        <v>19163123</v>
+        <v>19163121</v>
       </c>
       <c r="U161" t="n">
-        <v>19163123</v>
+        <v>19163121</v>
       </c>
       <c r="V161" t="n">
         <v>1600000</v>
@@ -13611,10 +13611,10 @@
         <v>0</v>
       </c>
       <c r="T162" t="n">
-        <v>21397101</v>
+        <v>21397100</v>
       </c>
       <c r="U162" t="n">
-        <v>21397101</v>
+        <v>21397100</v>
       </c>
       <c r="V162" t="n">
         <v>1610000</v>
@@ -13626,7 +13626,7 @@
         <v>42.635</v>
       </c>
       <c r="Y162" t="n">
-        <v>6103802</v>
+        <v>6103801</v>
       </c>
     </row>
     <row r="163">
@@ -13707,7 +13707,7 @@
         <v>38.189</v>
       </c>
       <c r="Y163" t="n">
-        <v>6023273</v>
+        <v>6023272</v>
       </c>
     </row>
     <row r="164">
@@ -13773,10 +13773,10 @@
         <v>0</v>
       </c>
       <c r="T164" t="n">
-        <v>15966067</v>
+        <v>15966070</v>
       </c>
       <c r="U164" t="n">
-        <v>15966067</v>
+        <v>15966070</v>
       </c>
       <c r="V164" t="n">
         <v>1630000</v>
@@ -13788,7 +13788,7 @@
         <v>31.777</v>
       </c>
       <c r="Y164" t="n">
-        <v>5727287</v>
+        <v>5727288</v>
       </c>
     </row>
     <row r="165">
@@ -13935,10 +13935,10 @@
         <v>0</v>
       </c>
       <c r="T166" t="n">
-        <v>19229261</v>
+        <v>19229262</v>
       </c>
       <c r="U166" t="n">
-        <v>19229261</v>
+        <v>19229262</v>
       </c>
       <c r="V166" t="n">
         <v>1650000</v>
@@ -14016,10 +14016,10 @@
         <v>0</v>
       </c>
       <c r="T167" t="n">
-        <v>23911804</v>
+        <v>23911803</v>
       </c>
       <c r="U167" t="n">
-        <v>23911804</v>
+        <v>23911803</v>
       </c>
       <c r="V167" t="n">
         <v>1660000</v>
@@ -14097,10 +14097,10 @@
         <v>0</v>
       </c>
       <c r="T168" t="n">
-        <v>24676080</v>
+        <v>24676081</v>
       </c>
       <c r="U168" t="n">
-        <v>24676080</v>
+        <v>24676081</v>
       </c>
       <c r="V168" t="n">
         <v>1670000</v>
@@ -14178,10 +14178,10 @@
         <v>0</v>
       </c>
       <c r="T169" t="n">
-        <v>30353798</v>
+        <v>30353797</v>
       </c>
       <c r="U169" t="n">
-        <v>30353798</v>
+        <v>30353797</v>
       </c>
       <c r="V169" t="n">
         <v>1680000</v>
@@ -14193,7 +14193,7 @@
         <v>60.269</v>
       </c>
       <c r="Y169" t="n">
-        <v>7090606</v>
+        <v>7090605</v>
       </c>
     </row>
     <row r="170">
@@ -14259,10 +14259,10 @@
         <v>0</v>
       </c>
       <c r="T170" t="n">
-        <v>32116992</v>
+        <v>32116991</v>
       </c>
       <c r="U170" t="n">
-        <v>32116992</v>
+        <v>32116991</v>
       </c>
       <c r="V170" t="n">
         <v>1690000</v>
@@ -14340,10 +14340,10 @@
         <v>0</v>
       </c>
       <c r="T171" t="n">
-        <v>27237243</v>
+        <v>27237245</v>
       </c>
       <c r="U171" t="n">
-        <v>27237243</v>
+        <v>27237245</v>
       </c>
       <c r="V171" t="n">
         <v>1700000</v>
@@ -14421,10 +14421,10 @@
         <v>0</v>
       </c>
       <c r="T172" t="n">
-        <v>33233013</v>
+        <v>33233014</v>
       </c>
       <c r="U172" t="n">
-        <v>33233013</v>
+        <v>33233014</v>
       </c>
       <c r="V172" t="n">
         <v>1710000</v>
@@ -14502,10 +14502,10 @@
         <v>0</v>
       </c>
       <c r="T173" t="n">
-        <v>38280840</v>
+        <v>38280841</v>
       </c>
       <c r="U173" t="n">
-        <v>38280840</v>
+        <v>38280841</v>
       </c>
       <c r="V173" t="n">
         <v>1720000</v>
@@ -14517,7 +14517,7 @@
         <v>75.914</v>
       </c>
       <c r="Y173" t="n">
-        <v>7803714</v>
+        <v>7803713</v>
       </c>
     </row>
     <row r="174">
@@ -14598,7 +14598,7 @@
         <v>65.602</v>
       </c>
       <c r="Y174" t="n">
-        <v>7682748</v>
+        <v>7682749</v>
       </c>
     </row>
     <row r="175">
@@ -14664,10 +14664,10 @@
         <v>0</v>
       </c>
       <c r="T175" t="n">
-        <v>31128409</v>
+        <v>31128408</v>
       </c>
       <c r="U175" t="n">
-        <v>31128409</v>
+        <v>31128408</v>
       </c>
       <c r="V175" t="n">
         <v>1740000</v>
@@ -14745,10 +14745,10 @@
         <v>0</v>
       </c>
       <c r="T176" t="n">
-        <v>31268446</v>
+        <v>31268445</v>
       </c>
       <c r="U176" t="n">
-        <v>31268446</v>
+        <v>31268445</v>
       </c>
       <c r="V176" t="n">
         <v>1750000</v>
@@ -14826,10 +14826,10 @@
         <v>0</v>
       </c>
       <c r="T177" t="n">
-        <v>28245894</v>
+        <v>28245895</v>
       </c>
       <c r="U177" t="n">
-        <v>28245894</v>
+        <v>28245895</v>
       </c>
       <c r="V177" t="n">
         <v>1760000</v>
@@ -14895,7 +14895,7 @@
         <v>2656.2</v>
       </c>
       <c r="P178" t="n">
-        <v>403536.8</v>
+        <v>403536.9</v>
       </c>
       <c r="Q178" t="n">
         <v>9485.299999999999</v>
@@ -14907,10 +14907,10 @@
         <v>0</v>
       </c>
       <c r="T178" t="n">
-        <v>29673043</v>
+        <v>29673045</v>
       </c>
       <c r="U178" t="n">
-        <v>29673043</v>
+        <v>29673045</v>
       </c>
       <c r="V178" t="n">
         <v>1770000</v>
@@ -14922,7 +14922,7 @@
         <v>58.748</v>
       </c>
       <c r="Y178" t="n">
-        <v>8366760</v>
+        <v>8366761</v>
       </c>
     </row>
     <row r="179">
@@ -14976,7 +14976,7 @@
         <v>2656.2</v>
       </c>
       <c r="P179" t="n">
-        <v>403664.3</v>
+        <v>403664.4</v>
       </c>
       <c r="Q179" t="n">
         <v>9485.299999999999</v>
@@ -14988,10 +14988,10 @@
         <v>0</v>
       </c>
       <c r="T179" t="n">
-        <v>29357461</v>
+        <v>29357463</v>
       </c>
       <c r="U179" t="n">
-        <v>29357461</v>
+        <v>29357463</v>
       </c>
       <c r="V179" t="n">
         <v>1780000</v>
@@ -15003,7 +15003,7 @@
         <v>58.103</v>
       </c>
       <c r="Y179" t="n">
-        <v>8414738</v>
+        <v>8414739</v>
       </c>
     </row>
     <row r="180">
@@ -15069,10 +15069,10 @@
         <v>0</v>
       </c>
       <c r="T180" t="n">
-        <v>30022609</v>
+        <v>30022612</v>
       </c>
       <c r="U180" t="n">
-        <v>30022609</v>
+        <v>30022612</v>
       </c>
       <c r="V180" t="n">
         <v>1790000</v>
@@ -15084,7 +15084,7 @@
         <v>59.4</v>
       </c>
       <c r="Y180" t="n">
-        <v>8606772</v>
+        <v>8606774</v>
       </c>
     </row>
     <row r="181">
@@ -15165,7 +15165,7 @@
         <v>52.958</v>
       </c>
       <c r="Y181" t="n">
-        <v>8384081</v>
+        <v>8384082</v>
       </c>
     </row>
     <row r="182">
@@ -15393,10 +15393,10 @@
         <v>0</v>
       </c>
       <c r="T184" t="n">
-        <v>23599915</v>
+        <v>23599916</v>
       </c>
       <c r="U184" t="n">
-        <v>23599915</v>
+        <v>23599916</v>
       </c>
       <c r="V184" t="n">
         <v>1830000</v>
@@ -15468,16 +15468,16 @@
         <v>9553.6</v>
       </c>
       <c r="R185" t="n">
-        <v>365665.4</v>
+        <v>365665.5</v>
       </c>
       <c r="S185" t="n">
         <v>0</v>
       </c>
       <c r="T185" t="n">
-        <v>30010014</v>
+        <v>30010015</v>
       </c>
       <c r="U185" t="n">
-        <v>30010014</v>
+        <v>30010015</v>
       </c>
       <c r="V185" t="n">
         <v>1840000</v>
@@ -15489,7 +15489,7 @@
         <v>59.248</v>
       </c>
       <c r="Y185" t="n">
-        <v>9169070</v>
+        <v>9169071</v>
       </c>
     </row>
     <row r="186">
@@ -15555,10 +15555,10 @@
         <v>0</v>
       </c>
       <c r="T186" t="n">
-        <v>31150711</v>
+        <v>31150712</v>
       </c>
       <c r="U186" t="n">
-        <v>31150711</v>
+        <v>31150712</v>
       </c>
       <c r="V186" t="n">
         <v>1850000</v>
@@ -15570,7 +15570,7 @@
         <v>61.48</v>
       </c>
       <c r="Y186" t="n">
-        <v>9401290</v>
+        <v>9401289</v>
       </c>
     </row>
     <row r="187">
@@ -15624,7 +15624,7 @@
         <v>2687.2</v>
       </c>
       <c r="P187" t="n">
-        <v>404267.8</v>
+        <v>404267.9</v>
       </c>
       <c r="Q187" t="n">
         <v>9553.6</v>
@@ -15651,7 +15651,7 @@
         <v>62.759</v>
       </c>
       <c r="Y187" t="n">
-        <v>9500966</v>
+        <v>9500965</v>
       </c>
     </row>
     <row r="188">
@@ -15792,16 +15792,16 @@
         <v>9553.6</v>
       </c>
       <c r="R189" t="n">
-        <v>366305.2</v>
+        <v>366305.3</v>
       </c>
       <c r="S189" t="n">
         <v>0</v>
       </c>
       <c r="T189" t="n">
-        <v>46173491</v>
+        <v>46173493</v>
       </c>
       <c r="U189" t="n">
-        <v>46173491</v>
+        <v>46173493</v>
       </c>
       <c r="V189" t="n">
         <v>1880000</v>
@@ -15813,7 +15813,7 @@
         <v>91.057</v>
       </c>
       <c r="Y189" t="n">
-        <v>10510816</v>
+        <v>10510817</v>
       </c>
     </row>
     <row r="190">
@@ -15879,10 +15879,10 @@
         <v>0</v>
       </c>
       <c r="T190" t="n">
-        <v>42126524</v>
+        <v>42126525</v>
       </c>
       <c r="U190" t="n">
-        <v>42126524</v>
+        <v>42126525</v>
       </c>
       <c r="V190" t="n">
         <v>1890000</v>
@@ -15894,7 +15894,7 @@
         <v>83.057</v>
       </c>
       <c r="Y190" t="n">
-        <v>10356729</v>
+        <v>10356728</v>
       </c>
     </row>
     <row r="191">
@@ -16041,10 +16041,10 @@
         <v>0</v>
       </c>
       <c r="T192" t="n">
-        <v>49996612</v>
+        <v>49996613</v>
       </c>
       <c r="U192" t="n">
-        <v>49996612</v>
+        <v>49996613</v>
       </c>
       <c r="V192" t="n">
         <v>1910000</v>
@@ -16122,10 +16122,10 @@
         <v>0</v>
       </c>
       <c r="T193" t="n">
-        <v>48544370</v>
+        <v>48544371</v>
       </c>
       <c r="U193" t="n">
-        <v>48544370</v>
+        <v>48544371</v>
       </c>
       <c r="V193" t="n">
         <v>1920000</v>
@@ -16203,10 +16203,10 @@
         <v>0</v>
       </c>
       <c r="T194" t="n">
-        <v>39666028</v>
+        <v>39666029</v>
       </c>
       <c r="U194" t="n">
-        <v>39666028</v>
+        <v>39666029</v>
       </c>
       <c r="V194" t="n">
         <v>1930000</v>
@@ -16284,10 +16284,10 @@
         <v>0</v>
       </c>
       <c r="T195" t="n">
-        <v>78944923</v>
+        <v>78944925</v>
       </c>
       <c r="U195" t="n">
-        <v>78944923</v>
+        <v>78944925</v>
       </c>
       <c r="V195" t="n">
         <v>1940000</v>
@@ -16365,10 +16365,10 @@
         <v>0</v>
       </c>
       <c r="T196" t="n">
-        <v>124244775</v>
+        <v>124244778</v>
       </c>
       <c r="U196" t="n">
-        <v>124244775</v>
+        <v>124244778</v>
       </c>
       <c r="V196" t="n">
         <v>1950000</v>
@@ -16446,10 +16446,10 @@
         <v>0</v>
       </c>
       <c r="T197" t="n">
-        <v>103894486</v>
+        <v>103894489</v>
       </c>
       <c r="U197" t="n">
-        <v>103894486</v>
+        <v>103894489</v>
       </c>
       <c r="V197" t="n">
         <v>1960000</v>
@@ -16461,7 +16461,7 @@
         <v>204.593</v>
       </c>
       <c r="Y197" t="n">
-        <v>11898665</v>
+        <v>11898666</v>
       </c>
     </row>
   </sheetData>
@@ -16582,12 +16582,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$103,894,486</t>
+          <t>$103,894,489</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>$11,898,665</t>
+          <t>$11,898,666</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -16597,12 +16597,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>$34,886,609</t>
+          <t>$34,886,610</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>$205,415,386</t>
+          <t>$205,415,393</t>
         </is>
       </c>
     </row>
@@ -16614,12 +16614,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$101,934,486</t>
+          <t>$101,934,489</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>$9,938,665</t>
+          <t>$9,938,666</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -16629,12 +16629,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>$32,926,609</t>
+          <t>$32,926,610</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>$203,455,386</t>
+          <t>$203,455,393</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Backtest: add 'Adaptive + cash' variant (annual Dec 25% cap) — halves drawdown
</commit_message>
<xml_diff>
--- a/backtest.xlsx
+++ b/backtest.xlsx
@@ -2502,7 +2502,7 @@
         <v>1653.3</v>
       </c>
       <c r="P25" t="n">
-        <v>124473.5</v>
+        <v>124473.4</v>
       </c>
       <c r="Q25" t="n">
         <v>5997.1</v>
@@ -2676,10 +2676,10 @@
         <v>0</v>
       </c>
       <c r="T27" t="n">
-        <v>313160</v>
+        <v>313159</v>
       </c>
       <c r="U27" t="n">
-        <v>313160</v>
+        <v>313159</v>
       </c>
       <c r="V27" t="n">
         <v>260000</v>
@@ -3009,7 +3009,7 @@
         <v>300000</v>
       </c>
       <c r="W31" t="n">
-        <v>7.94</v>
+        <v>7.93</v>
       </c>
       <c r="X31" t="n">
         <v>1.357</v>
@@ -3177,7 +3177,7 @@
         <v>1.216</v>
       </c>
       <c r="Y33" t="n">
-        <v>377066</v>
+        <v>377065</v>
       </c>
     </row>
     <row r="34">
@@ -4041,7 +4041,7 @@
         <v>1744.2</v>
       </c>
       <c r="P44" t="n">
-        <v>274317.7</v>
+        <v>274317.8</v>
       </c>
       <c r="Q44" t="n">
         <v>6375.7</v>
@@ -4554,7 +4554,7 @@
         <v>2.704</v>
       </c>
       <c r="Y50" t="n">
-        <v>720760</v>
+        <v>720761</v>
       </c>
     </row>
     <row r="51">
@@ -4878,7 +4878,7 @@
         <v>3.097</v>
       </c>
       <c r="Y54" t="n">
-        <v>824699</v>
+        <v>824700</v>
       </c>
     </row>
     <row r="55">
@@ -4959,7 +4959,7 @@
         <v>3.558</v>
       </c>
       <c r="Y55" t="n">
-        <v>876003</v>
+        <v>876002</v>
       </c>
     </row>
     <row r="56">
@@ -5187,10 +5187,10 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>1607745</v>
+        <v>1607746</v>
       </c>
       <c r="U58" t="n">
-        <v>1607745</v>
+        <v>1607746</v>
       </c>
       <c r="V58" t="n">
         <v>570000</v>
@@ -6645,10 +6645,10 @@
         <v>0</v>
       </c>
       <c r="T76" t="n">
-        <v>1726273</v>
+        <v>1726274</v>
       </c>
       <c r="U76" t="n">
-        <v>1726273</v>
+        <v>1726274</v>
       </c>
       <c r="V76" t="n">
         <v>750000</v>
@@ -6660,7 +6660,7 @@
         <v>3.902</v>
       </c>
       <c r="Y76" t="n">
-        <v>1206765</v>
+        <v>1206766</v>
       </c>
     </row>
     <row r="77">
@@ -7146,7 +7146,7 @@
         <v>5.53</v>
       </c>
       <c r="Y82" t="n">
-        <v>1352897</v>
+        <v>1352896</v>
       </c>
     </row>
     <row r="83">
@@ -7293,10 +7293,10 @@
         <v>0</v>
       </c>
       <c r="T84" t="n">
-        <v>2968224</v>
+        <v>2968225</v>
       </c>
       <c r="U84" t="n">
-        <v>2968224</v>
+        <v>2968225</v>
       </c>
       <c r="V84" t="n">
         <v>830000</v>
@@ -7389,7 +7389,7 @@
         <v>7.072</v>
       </c>
       <c r="Y85" t="n">
-        <v>1532859</v>
+        <v>1532858</v>
       </c>
     </row>
     <row r="86">
@@ -7470,7 +7470,7 @@
         <v>7.683</v>
       </c>
       <c r="Y86" t="n">
-        <v>1573917</v>
+        <v>1573918</v>
       </c>
     </row>
     <row r="87">
@@ -7611,7 +7611,7 @@
         <v>7882.7</v>
       </c>
       <c r="R88" t="n">
-        <v>342207.6</v>
+        <v>342207.5</v>
       </c>
       <c r="S88" t="n">
         <v>0</v>
@@ -7794,7 +7794,7 @@
         <v>9.17</v>
       </c>
       <c r="Y90" t="n">
-        <v>1748647</v>
+        <v>1748648</v>
       </c>
     </row>
     <row r="91">
@@ -7860,10 +7860,10 @@
         <v>0</v>
       </c>
       <c r="T91" t="n">
-        <v>4529337</v>
+        <v>4529336</v>
       </c>
       <c r="U91" t="n">
-        <v>4529337</v>
+        <v>4529336</v>
       </c>
       <c r="V91" t="n">
         <v>900000</v>
@@ -7941,10 +7941,10 @@
         <v>0</v>
       </c>
       <c r="T92" t="n">
-        <v>4870742</v>
+        <v>4870741</v>
       </c>
       <c r="U92" t="n">
-        <v>4870742</v>
+        <v>4870741</v>
       </c>
       <c r="V92" t="n">
         <v>910000</v>
@@ -7956,7 +7956,7 @@
         <v>10.414</v>
       </c>
       <c r="Y92" t="n">
-        <v>1799589</v>
+        <v>1799588</v>
       </c>
     </row>
     <row r="93">
@@ -8199,7 +8199,7 @@
         <v>12.358</v>
       </c>
       <c r="Y95" t="n">
-        <v>1961469</v>
+        <v>1961468</v>
       </c>
     </row>
     <row r="96">
@@ -8265,10 +8265,10 @@
         <v>0</v>
       </c>
       <c r="T96" t="n">
-        <v>7254016</v>
+        <v>7254015</v>
       </c>
       <c r="U96" t="n">
-        <v>7254016</v>
+        <v>7254015</v>
       </c>
       <c r="V96" t="n">
         <v>950000</v>
@@ -8280,7 +8280,7 @@
         <v>15.409</v>
       </c>
       <c r="Y96" t="n">
-        <v>2143226</v>
+        <v>2143225</v>
       </c>
     </row>
     <row r="97">
@@ -8361,7 +8361,7 @@
         <v>14.815</v>
       </c>
       <c r="Y97" t="n">
-        <v>2125507</v>
+        <v>2125508</v>
       </c>
     </row>
     <row r="98">
@@ -8508,10 +8508,10 @@
         <v>0</v>
       </c>
       <c r="T99" t="n">
-        <v>5568498</v>
+        <v>5568499</v>
       </c>
       <c r="U99" t="n">
-        <v>5568498</v>
+        <v>5568499</v>
       </c>
       <c r="V99" t="n">
         <v>980000</v>
@@ -8589,10 +8589,10 @@
         <v>0</v>
       </c>
       <c r="T100" t="n">
-        <v>6966365</v>
+        <v>6966364</v>
       </c>
       <c r="U100" t="n">
-        <v>6966365</v>
+        <v>6966364</v>
       </c>
       <c r="V100" t="n">
         <v>990000</v>
@@ -8685,7 +8685,7 @@
         <v>13.697</v>
       </c>
       <c r="Y101" t="n">
-        <v>2231669</v>
+        <v>2231668</v>
       </c>
     </row>
     <row r="102">
@@ -8832,10 +8832,10 @@
         <v>0</v>
       </c>
       <c r="T103" t="n">
-        <v>7860869</v>
+        <v>7860870</v>
       </c>
       <c r="U103" t="n">
-        <v>7860869</v>
+        <v>7860870</v>
       </c>
       <c r="V103" t="n">
         <v>1020000</v>
@@ -8913,10 +8913,10 @@
         <v>0</v>
       </c>
       <c r="T104" t="n">
-        <v>7517180</v>
+        <v>7517179</v>
       </c>
       <c r="U104" t="n">
-        <v>7517180</v>
+        <v>7517179</v>
       </c>
       <c r="V104" t="n">
         <v>1030000</v>
@@ -8994,10 +8994,10 @@
         <v>0</v>
       </c>
       <c r="T105" t="n">
-        <v>5359631</v>
+        <v>5359632</v>
       </c>
       <c r="U105" t="n">
-        <v>5359631</v>
+        <v>5359632</v>
       </c>
       <c r="V105" t="n">
         <v>1040000</v>
@@ -9156,10 +9156,10 @@
         <v>0</v>
       </c>
       <c r="T107" t="n">
-        <v>4252568</v>
+        <v>4252567</v>
       </c>
       <c r="U107" t="n">
-        <v>4252568</v>
+        <v>4252567</v>
       </c>
       <c r="V107" t="n">
         <v>1060000</v>
@@ -9252,7 +9252,7 @@
         <v>11.061</v>
       </c>
       <c r="Y108" t="n">
-        <v>2264917</v>
+        <v>2264918</v>
       </c>
     </row>
     <row r="109">
@@ -9399,10 +9399,10 @@
         <v>0</v>
       </c>
       <c r="T110" t="n">
-        <v>6552312</v>
+        <v>6552313</v>
       </c>
       <c r="U110" t="n">
-        <v>6552312</v>
+        <v>6552313</v>
       </c>
       <c r="V110" t="n">
         <v>1090000</v>
@@ -9414,7 +9414,7 @@
         <v>13.603</v>
       </c>
       <c r="Y110" t="n">
-        <v>2444585</v>
+        <v>2444586</v>
       </c>
     </row>
     <row r="111">
@@ -9480,10 +9480,10 @@
         <v>0</v>
       </c>
       <c r="T111" t="n">
-        <v>8210212</v>
+        <v>8210213</v>
       </c>
       <c r="U111" t="n">
-        <v>8210212</v>
+        <v>8210213</v>
       </c>
       <c r="V111" t="n">
         <v>1100000</v>
@@ -9495,7 +9495,7 @@
         <v>17.025</v>
       </c>
       <c r="Y111" t="n">
-        <v>2589010</v>
+        <v>2589009</v>
       </c>
     </row>
     <row r="112">
@@ -9576,7 +9576,7 @@
         <v>11.4</v>
       </c>
       <c r="Y112" t="n">
-        <v>2386049</v>
+        <v>2386050</v>
       </c>
     </row>
     <row r="113">
@@ -9642,10 +9642,10 @@
         <v>0</v>
       </c>
       <c r="T113" t="n">
-        <v>7101970</v>
+        <v>7101969</v>
       </c>
       <c r="U113" t="n">
-        <v>7101970</v>
+        <v>7101969</v>
       </c>
       <c r="V113" t="n">
         <v>1120000</v>
@@ -9738,7 +9738,7 @@
         <v>16.261</v>
       </c>
       <c r="Y114" t="n">
-        <v>2647302</v>
+        <v>2647303</v>
       </c>
     </row>
     <row r="115">
@@ -9900,7 +9900,7 @@
         <v>15.8</v>
       </c>
       <c r="Y116" t="n">
-        <v>2640925</v>
+        <v>2640926</v>
       </c>
     </row>
     <row r="117">
@@ -9966,10 +9966,10 @@
         <v>0</v>
       </c>
       <c r="T117" t="n">
-        <v>8740736</v>
+        <v>8740734</v>
       </c>
       <c r="U117" t="n">
-        <v>8740736</v>
+        <v>8740734</v>
       </c>
       <c r="V117" t="n">
         <v>1160000</v>
@@ -9981,7 +9981,7 @@
         <v>17.974</v>
       </c>
       <c r="Y117" t="n">
-        <v>2766590</v>
+        <v>2766589</v>
       </c>
     </row>
     <row r="118">
@@ -10047,10 +10047,10 @@
         <v>0</v>
       </c>
       <c r="T118" t="n">
-        <v>9720972</v>
+        <v>9720973</v>
       </c>
       <c r="U118" t="n">
-        <v>9720972</v>
+        <v>9720973</v>
       </c>
       <c r="V118" t="n">
         <v>1170000</v>
@@ -10128,10 +10128,10 @@
         <v>0</v>
       </c>
       <c r="T119" t="n">
-        <v>11444851</v>
+        <v>11444852</v>
       </c>
       <c r="U119" t="n">
-        <v>11444851</v>
+        <v>11444852</v>
       </c>
       <c r="V119" t="n">
         <v>1180000</v>
@@ -10224,7 +10224,7 @@
         <v>22.693</v>
       </c>
       <c r="Y120" t="n">
-        <v>3112928</v>
+        <v>3112927</v>
       </c>
     </row>
     <row r="121">
@@ -10290,10 +10290,10 @@
         <v>0</v>
       </c>
       <c r="T121" t="n">
-        <v>9345549</v>
+        <v>9345550</v>
       </c>
       <c r="U121" t="n">
-        <v>9345549</v>
+        <v>9345550</v>
       </c>
       <c r="V121" t="n">
         <v>1200000</v>
@@ -10305,7 +10305,7 @@
         <v>19.144</v>
       </c>
       <c r="Y121" t="n">
-        <v>2934355</v>
+        <v>2934354</v>
       </c>
     </row>
     <row r="122">
@@ -10614,10 +10614,10 @@
         <v>0</v>
       </c>
       <c r="T125" t="n">
-        <v>10167702</v>
+        <v>10167703</v>
       </c>
       <c r="U125" t="n">
-        <v>10167702</v>
+        <v>10167703</v>
       </c>
       <c r="V125" t="n">
         <v>1240000</v>
@@ -10695,10 +10695,10 @@
         <v>0</v>
       </c>
       <c r="T126" t="n">
-        <v>12195954</v>
+        <v>12195955</v>
       </c>
       <c r="U126" t="n">
-        <v>12195954</v>
+        <v>12195955</v>
       </c>
       <c r="V126" t="n">
         <v>1250000</v>
@@ -10710,7 +10710,7 @@
         <v>24.828</v>
       </c>
       <c r="Y126" t="n">
-        <v>3862622</v>
+        <v>3862620</v>
       </c>
     </row>
     <row r="127">
@@ -10776,10 +10776,10 @@
         <v>0</v>
       </c>
       <c r="T127" t="n">
-        <v>15247651</v>
+        <v>15247650</v>
       </c>
       <c r="U127" t="n">
-        <v>15247651</v>
+        <v>15247650</v>
       </c>
       <c r="V127" t="n">
         <v>1260000</v>
@@ -10791,7 +10791,7 @@
         <v>31.02</v>
       </c>
       <c r="Y127" t="n">
-        <v>4295364</v>
+        <v>4295365</v>
       </c>
     </row>
     <row r="128">
@@ -10857,10 +10857,10 @@
         <v>0</v>
       </c>
       <c r="T128" t="n">
-        <v>13443232</v>
+        <v>13443231</v>
       </c>
       <c r="U128" t="n">
-        <v>13443232</v>
+        <v>13443231</v>
       </c>
       <c r="V128" t="n">
         <v>1270000</v>
@@ -10872,7 +10872,7 @@
         <v>27.329</v>
       </c>
       <c r="Y128" t="n">
-        <v>4057141</v>
+        <v>4057142</v>
       </c>
     </row>
     <row r="129">
@@ -10953,7 +10953,7 @@
         <v>25.797</v>
       </c>
       <c r="Y129" t="n">
-        <v>3943594</v>
+        <v>3943595</v>
       </c>
     </row>
     <row r="130">
@@ -11019,10 +11019,10 @@
         <v>0</v>
       </c>
       <c r="T130" t="n">
-        <v>18502837</v>
+        <v>18502833</v>
       </c>
       <c r="U130" t="n">
-        <v>18502837</v>
+        <v>18502833</v>
       </c>
       <c r="V130" t="n">
         <v>1290000</v>
@@ -11034,7 +11034,7 @@
         <v>37.565</v>
       </c>
       <c r="Y130" t="n">
-        <v>4396284</v>
+        <v>4396285</v>
       </c>
     </row>
     <row r="131">
@@ -11115,7 +11115,7 @@
         <v>42.888</v>
       </c>
       <c r="Y131" t="n">
-        <v>4621799</v>
+        <v>4621798</v>
       </c>
     </row>
     <row r="132">
@@ -11181,10 +11181,10 @@
         <v>0</v>
       </c>
       <c r="T132" t="n">
-        <v>21944519</v>
+        <v>21944520</v>
       </c>
       <c r="U132" t="n">
-        <v>21944519</v>
+        <v>21944520</v>
       </c>
       <c r="V132" t="n">
         <v>1310000</v>
@@ -11262,10 +11262,10 @@
         <v>0</v>
       </c>
       <c r="T133" t="n">
-        <v>23751398</v>
+        <v>23751399</v>
       </c>
       <c r="U133" t="n">
-        <v>23751398</v>
+        <v>23751399</v>
       </c>
       <c r="V133" t="n">
         <v>1320000</v>
@@ -11277,7 +11277,7 @@
         <v>48.156</v>
       </c>
       <c r="Y133" t="n">
-        <v>4647658</v>
+        <v>4647659</v>
       </c>
     </row>
     <row r="134">
@@ -11343,10 +11343,10 @@
         <v>0</v>
       </c>
       <c r="T134" t="n">
-        <v>23809377</v>
+        <v>23809374</v>
       </c>
       <c r="U134" t="n">
-        <v>23809377</v>
+        <v>23809374</v>
       </c>
       <c r="V134" t="n">
         <v>1330000</v>
@@ -11358,7 +11358,7 @@
         <v>48.253</v>
       </c>
       <c r="Y134" t="n">
-        <v>4737438</v>
+        <v>4737439</v>
       </c>
     </row>
     <row r="135">
@@ -11424,10 +11424,10 @@
         <v>0</v>
       </c>
       <c r="T135" t="n">
-        <v>24961850</v>
+        <v>24961851</v>
       </c>
       <c r="U135" t="n">
-        <v>24961850</v>
+        <v>24961851</v>
       </c>
       <c r="V135" t="n">
         <v>1340000</v>
@@ -11520,7 +11520,7 @@
         <v>50.958</v>
       </c>
       <c r="Y136" t="n">
-        <v>4977003</v>
+        <v>4977001</v>
       </c>
     </row>
     <row r="137">
@@ -11586,10 +11586,10 @@
         <v>0</v>
       </c>
       <c r="T137" t="n">
-        <v>29189210</v>
+        <v>29189209</v>
       </c>
       <c r="U137" t="n">
-        <v>29189210</v>
+        <v>29189209</v>
       </c>
       <c r="V137" t="n">
         <v>1360000</v>
@@ -11601,7 +11601,7 @@
         <v>59.089</v>
       </c>
       <c r="Y137" t="n">
-        <v>5298658</v>
+        <v>5298659</v>
       </c>
     </row>
     <row r="138">
@@ -11667,10 +11667,10 @@
         <v>0</v>
       </c>
       <c r="T138" t="n">
-        <v>30149070</v>
+        <v>30149069</v>
       </c>
       <c r="U138" t="n">
-        <v>30149070</v>
+        <v>30149069</v>
       </c>
       <c r="V138" t="n">
         <v>1370000</v>
@@ -11829,10 +11829,10 @@
         <v>0</v>
       </c>
       <c r="T140" t="n">
-        <v>27821993</v>
+        <v>27821990</v>
       </c>
       <c r="U140" t="n">
-        <v>27821993</v>
+        <v>27821990</v>
       </c>
       <c r="V140" t="n">
         <v>1390000</v>
@@ -11844,7 +11844,7 @@
         <v>56.265</v>
       </c>
       <c r="Y140" t="n">
-        <v>5386597</v>
+        <v>5386596</v>
       </c>
     </row>
     <row r="141">
@@ -11910,10 +11910,10 @@
         <v>0</v>
       </c>
       <c r="T141" t="n">
-        <v>33553104</v>
+        <v>33553107</v>
       </c>
       <c r="U141" t="n">
-        <v>33553104</v>
+        <v>33553107</v>
       </c>
       <c r="V141" t="n">
         <v>1400000</v>
@@ -11925,7 +11925,7 @@
         <v>67.83499999999999</v>
       </c>
       <c r="Y141" t="n">
-        <v>5820189</v>
+        <v>5820190</v>
       </c>
     </row>
     <row r="142">
@@ -11991,10 +11991,10 @@
         <v>0</v>
       </c>
       <c r="T142" t="n">
-        <v>40473531</v>
+        <v>40473532</v>
       </c>
       <c r="U142" t="n">
-        <v>40473531</v>
+        <v>40473532</v>
       </c>
       <c r="V142" t="n">
         <v>1410000</v>
@@ -12072,10 +12072,10 @@
         <v>0</v>
       </c>
       <c r="T143" t="n">
-        <v>41964996</v>
+        <v>41964989</v>
       </c>
       <c r="U143" t="n">
-        <v>41964996</v>
+        <v>41964989</v>
       </c>
       <c r="V143" t="n">
         <v>1420000</v>
@@ -12087,7 +12087,7 @@
         <v>84.8</v>
       </c>
       <c r="Y143" t="n">
-        <v>6024912</v>
+        <v>6024911</v>
       </c>
     </row>
     <row r="144">
@@ -12153,10 +12153,10 @@
         <v>0</v>
       </c>
       <c r="T144" t="n">
-        <v>29465118</v>
+        <v>29465119</v>
       </c>
       <c r="U144" t="n">
-        <v>29465118</v>
+        <v>29465119</v>
       </c>
       <c r="V144" t="n">
         <v>1430000</v>
@@ -12234,10 +12234,10 @@
         <v>0</v>
       </c>
       <c r="T145" t="n">
-        <v>26366603</v>
+        <v>26366606</v>
       </c>
       <c r="U145" t="n">
-        <v>26366603</v>
+        <v>26366606</v>
       </c>
       <c r="V145" t="n">
         <v>1440000</v>
@@ -12249,7 +12249,7 @@
         <v>53.242</v>
       </c>
       <c r="Y145" t="n">
-        <v>5271360</v>
+        <v>5271359</v>
       </c>
     </row>
     <row r="146">
@@ -12315,10 +12315,10 @@
         <v>0</v>
       </c>
       <c r="T146" t="n">
-        <v>26733470</v>
+        <v>26733466</v>
       </c>
       <c r="U146" t="n">
-        <v>26733470</v>
+        <v>26733466</v>
       </c>
       <c r="V146" t="n">
         <v>1450000</v>
@@ -12396,10 +12396,10 @@
         <v>0</v>
       </c>
       <c r="T147" t="n">
-        <v>16522122</v>
+        <v>16522120</v>
       </c>
       <c r="U147" t="n">
-        <v>16522122</v>
+        <v>16522120</v>
       </c>
       <c r="V147" t="n">
         <v>1460000</v>
@@ -12411,7 +12411,7 @@
         <v>33.33</v>
       </c>
       <c r="Y147" t="n">
-        <v>4785908</v>
+        <v>4785907</v>
       </c>
     </row>
     <row r="148">
@@ -12477,10 +12477,10 @@
         <v>0</v>
       </c>
       <c r="T148" t="n">
-        <v>16839659</v>
+        <v>16839657</v>
       </c>
       <c r="U148" t="n">
-        <v>16839659</v>
+        <v>16839657</v>
       </c>
       <c r="V148" t="n">
         <v>1470000</v>
@@ -12492,7 +12492,7 @@
         <v>33.951</v>
       </c>
       <c r="Y148" t="n">
-        <v>4719964</v>
+        <v>4719965</v>
       </c>
     </row>
     <row r="149">
@@ -12639,10 +12639,10 @@
         <v>0</v>
       </c>
       <c r="T150" t="n">
-        <v>15151251</v>
+        <v>15151252</v>
       </c>
       <c r="U150" t="n">
-        <v>15151251</v>
+        <v>15151252</v>
       </c>
       <c r="V150" t="n">
         <v>1490000</v>
@@ -12654,7 +12654,7 @@
         <v>30.498</v>
       </c>
       <c r="Y150" t="n">
-        <v>4860413</v>
+        <v>4860414</v>
       </c>
     </row>
     <row r="151">
@@ -12720,10 +12720,10 @@
         <v>0</v>
       </c>
       <c r="T151" t="n">
-        <v>11929511</v>
+        <v>11929512</v>
       </c>
       <c r="U151" t="n">
-        <v>11929511</v>
+        <v>11929512</v>
       </c>
       <c r="V151" t="n">
         <v>1500000</v>
@@ -12816,7 +12816,7 @@
         <v>16.678</v>
       </c>
       <c r="Y152" t="n">
-        <v>4144106</v>
+        <v>4144105</v>
       </c>
     </row>
     <row r="153">
@@ -12882,10 +12882,10 @@
         <v>0</v>
       </c>
       <c r="T153" t="n">
-        <v>8689212</v>
+        <v>8689213</v>
       </c>
       <c r="U153" t="n">
-        <v>8689212</v>
+        <v>8689213</v>
       </c>
       <c r="V153" t="n">
         <v>1520000</v>
@@ -12978,7 +12978,7 @@
         <v>22.324</v>
       </c>
       <c r="Y154" t="n">
-        <v>4569341</v>
+        <v>4569342</v>
       </c>
     </row>
     <row r="155">
@@ -13140,7 +13140,7 @@
         <v>22.767</v>
       </c>
       <c r="Y156" t="n">
-        <v>4620998</v>
+        <v>4620997</v>
       </c>
     </row>
     <row r="157">
@@ -13206,10 +13206,10 @@
         <v>0</v>
       </c>
       <c r="T157" t="n">
-        <v>11294701</v>
+        <v>11294702</v>
       </c>
       <c r="U157" t="n">
-        <v>11294701</v>
+        <v>11294702</v>
       </c>
       <c r="V157" t="n">
         <v>1560000</v>
@@ -13221,7 +13221,7 @@
         <v>22.576</v>
       </c>
       <c r="Y157" t="n">
-        <v>4614363</v>
+        <v>4614362</v>
       </c>
     </row>
     <row r="158">
@@ -13287,10 +13287,10 @@
         <v>0</v>
       </c>
       <c r="T158" t="n">
-        <v>13994542</v>
+        <v>13994543</v>
       </c>
       <c r="U158" t="n">
-        <v>13994542</v>
+        <v>13994543</v>
       </c>
       <c r="V158" t="n">
         <v>1570000</v>
@@ -13302,7 +13302,7 @@
         <v>27.952</v>
       </c>
       <c r="Y158" t="n">
-        <v>5062382</v>
+        <v>5062380</v>
       </c>
     </row>
     <row r="159">
@@ -13443,7 +13443,7 @@
         <v>9431.200000000001</v>
       </c>
       <c r="R160" t="n">
-        <v>362213.9</v>
+        <v>362213.8</v>
       </c>
       <c r="S160" t="n">
         <v>0</v>
@@ -13524,7 +13524,7 @@
         <v>9464.4</v>
       </c>
       <c r="R161" t="n">
-        <v>362213.9</v>
+        <v>362213.8</v>
       </c>
       <c r="S161" t="n">
         <v>0</v>
@@ -13611,10 +13611,10 @@
         <v>0</v>
       </c>
       <c r="T162" t="n">
-        <v>21397100</v>
+        <v>21397102</v>
       </c>
       <c r="U162" t="n">
-        <v>21397100</v>
+        <v>21397102</v>
       </c>
       <c r="V162" t="n">
         <v>1610000</v>
@@ -13626,7 +13626,7 @@
         <v>42.635</v>
       </c>
       <c r="Y162" t="n">
-        <v>6103801</v>
+        <v>6103803</v>
       </c>
     </row>
     <row r="163">
@@ -13773,10 +13773,10 @@
         <v>0</v>
       </c>
       <c r="T164" t="n">
-        <v>15966070</v>
+        <v>15966068</v>
       </c>
       <c r="U164" t="n">
-        <v>15966070</v>
+        <v>15966068</v>
       </c>
       <c r="V164" t="n">
         <v>1630000</v>
@@ -13788,7 +13788,7 @@
         <v>31.777</v>
       </c>
       <c r="Y164" t="n">
-        <v>5727288</v>
+        <v>5727289</v>
       </c>
     </row>
     <row r="165">
@@ -13854,10 +13854,10 @@
         <v>0</v>
       </c>
       <c r="T165" t="n">
-        <v>13930309</v>
+        <v>13930308</v>
       </c>
       <c r="U165" t="n">
-        <v>13930309</v>
+        <v>13930308</v>
       </c>
       <c r="V165" t="n">
         <v>1640000</v>
@@ -13935,10 +13935,10 @@
         <v>0</v>
       </c>
       <c r="T166" t="n">
-        <v>19229262</v>
+        <v>19229260</v>
       </c>
       <c r="U166" t="n">
-        <v>19229262</v>
+        <v>19229260</v>
       </c>
       <c r="V166" t="n">
         <v>1650000</v>
@@ -13950,7 +13950,7 @@
         <v>38.224</v>
       </c>
       <c r="Y166" t="n">
-        <v>6236880</v>
+        <v>6236879</v>
       </c>
     </row>
     <row r="167">
@@ -14016,10 +14016,10 @@
         <v>0</v>
       </c>
       <c r="T167" t="n">
-        <v>23911803</v>
+        <v>23911805</v>
       </c>
       <c r="U167" t="n">
-        <v>23911803</v>
+        <v>23911805</v>
       </c>
       <c r="V167" t="n">
         <v>1660000</v>
@@ -14112,7 +14112,7 @@
         <v>49.011</v>
       </c>
       <c r="Y168" t="n">
-        <v>6725294</v>
+        <v>6725295</v>
       </c>
     </row>
     <row r="169">
@@ -14178,10 +14178,10 @@
         <v>0</v>
       </c>
       <c r="T169" t="n">
-        <v>30353797</v>
+        <v>30353798</v>
       </c>
       <c r="U169" t="n">
-        <v>30353797</v>
+        <v>30353798</v>
       </c>
       <c r="V169" t="n">
         <v>1680000</v>
@@ -14259,10 +14259,10 @@
         <v>0</v>
       </c>
       <c r="T170" t="n">
-        <v>32116991</v>
+        <v>32116992</v>
       </c>
       <c r="U170" t="n">
-        <v>32116991</v>
+        <v>32116992</v>
       </c>
       <c r="V170" t="n">
         <v>1690000</v>
@@ -14340,10 +14340,10 @@
         <v>0</v>
       </c>
       <c r="T171" t="n">
-        <v>27237245</v>
+        <v>27237246</v>
       </c>
       <c r="U171" t="n">
-        <v>27237245</v>
+        <v>27237246</v>
       </c>
       <c r="V171" t="n">
         <v>1700000</v>
@@ -14355,7 +14355,7 @@
         <v>54.044</v>
       </c>
       <c r="Y171" t="n">
-        <v>6886471</v>
+        <v>6886470</v>
       </c>
     </row>
     <row r="172">
@@ -14421,10 +14421,10 @@
         <v>0</v>
       </c>
       <c r="T172" t="n">
-        <v>33233014</v>
+        <v>33233012</v>
       </c>
       <c r="U172" t="n">
-        <v>33233014</v>
+        <v>33233012</v>
       </c>
       <c r="V172" t="n">
         <v>1710000</v>
@@ -14502,10 +14502,10 @@
         <v>0</v>
       </c>
       <c r="T173" t="n">
-        <v>38280841</v>
+        <v>38280842</v>
       </c>
       <c r="U173" t="n">
-        <v>38280841</v>
+        <v>38280842</v>
       </c>
       <c r="V173" t="n">
         <v>1720000</v>
@@ -14583,10 +14583,10 @@
         <v>0</v>
       </c>
       <c r="T174" t="n">
-        <v>33090699</v>
+        <v>33090702</v>
       </c>
       <c r="U174" t="n">
-        <v>33090699</v>
+        <v>33090702</v>
       </c>
       <c r="V174" t="n">
         <v>1730000</v>
@@ -14637,7 +14637,7 @@
         <v>0</v>
       </c>
       <c r="K175" t="n">
-        <v>471.84</v>
+        <v>471.85</v>
       </c>
       <c r="L175" t="n">
         <v>33.75</v>
@@ -14745,10 +14745,10 @@
         <v>0</v>
       </c>
       <c r="T176" t="n">
-        <v>31268445</v>
+        <v>31268446</v>
       </c>
       <c r="U176" t="n">
-        <v>31268445</v>
+        <v>31268446</v>
       </c>
       <c r="V176" t="n">
         <v>1750000</v>
@@ -14826,10 +14826,10 @@
         <v>0</v>
       </c>
       <c r="T177" t="n">
-        <v>28245895</v>
+        <v>28245894</v>
       </c>
       <c r="U177" t="n">
-        <v>28245895</v>
+        <v>28245894</v>
       </c>
       <c r="V177" t="n">
         <v>1760000</v>
@@ -14841,7 +14841,7 @@
         <v>55.941</v>
       </c>
       <c r="Y177" t="n">
-        <v>7932326</v>
+        <v>7932325</v>
       </c>
     </row>
     <row r="178">
@@ -14895,7 +14895,7 @@
         <v>2656.2</v>
       </c>
       <c r="P178" t="n">
-        <v>403536.9</v>
+        <v>403536.8</v>
       </c>
       <c r="Q178" t="n">
         <v>9485.299999999999</v>
@@ -14907,10 +14907,10 @@
         <v>0</v>
       </c>
       <c r="T178" t="n">
-        <v>29673045</v>
+        <v>29673046</v>
       </c>
       <c r="U178" t="n">
-        <v>29673045</v>
+        <v>29673046</v>
       </c>
       <c r="V178" t="n">
         <v>1770000</v>
@@ -15069,10 +15069,10 @@
         <v>0</v>
       </c>
       <c r="T180" t="n">
-        <v>30022612</v>
+        <v>30022610</v>
       </c>
       <c r="U180" t="n">
-        <v>30022612</v>
+        <v>30022610</v>
       </c>
       <c r="V180" t="n">
         <v>1790000</v>
@@ -15084,7 +15084,7 @@
         <v>59.4</v>
       </c>
       <c r="Y180" t="n">
-        <v>8606774</v>
+        <v>8606773</v>
       </c>
     </row>
     <row r="181">
@@ -15165,7 +15165,7 @@
         <v>52.958</v>
       </c>
       <c r="Y181" t="n">
-        <v>8384082</v>
+        <v>8384081</v>
       </c>
     </row>
     <row r="182">
@@ -15231,10 +15231,10 @@
         <v>0</v>
       </c>
       <c r="T182" t="n">
-        <v>20550300</v>
+        <v>20550299</v>
       </c>
       <c r="U182" t="n">
-        <v>20550300</v>
+        <v>20550299</v>
       </c>
       <c r="V182" t="n">
         <v>1810000</v>
@@ -15246,7 +15246,7 @@
         <v>40.624</v>
       </c>
       <c r="Y182" t="n">
-        <v>7758040</v>
+        <v>7758039</v>
       </c>
     </row>
     <row r="183">
@@ -15393,10 +15393,10 @@
         <v>0</v>
       </c>
       <c r="T184" t="n">
-        <v>23599916</v>
+        <v>23599915</v>
       </c>
       <c r="U184" t="n">
-        <v>23599916</v>
+        <v>23599915</v>
       </c>
       <c r="V184" t="n">
         <v>1830000</v>
@@ -15408,7 +15408,7 @@
         <v>46.608</v>
       </c>
       <c r="Y184" t="n">
-        <v>8609304</v>
+        <v>8609305</v>
       </c>
     </row>
     <row r="185">
@@ -15489,7 +15489,7 @@
         <v>59.248</v>
       </c>
       <c r="Y185" t="n">
-        <v>9169071</v>
+        <v>9169069</v>
       </c>
     </row>
     <row r="186">
@@ -15570,7 +15570,7 @@
         <v>61.48</v>
       </c>
       <c r="Y186" t="n">
-        <v>9401289</v>
+        <v>9401290</v>
       </c>
     </row>
     <row r="187">
@@ -15636,10 +15636,10 @@
         <v>0</v>
       </c>
       <c r="T187" t="n">
-        <v>31808639</v>
+        <v>31808641</v>
       </c>
       <c r="U187" t="n">
-        <v>31808639</v>
+        <v>31808641</v>
       </c>
       <c r="V187" t="n">
         <v>1860000</v>
@@ -15651,7 +15651,7 @@
         <v>62.759</v>
       </c>
       <c r="Y187" t="n">
-        <v>9500965</v>
+        <v>9500966</v>
       </c>
     </row>
     <row r="188">
@@ -15798,10 +15798,10 @@
         <v>0</v>
       </c>
       <c r="T189" t="n">
-        <v>46173493</v>
+        <v>46173492</v>
       </c>
       <c r="U189" t="n">
-        <v>46173493</v>
+        <v>46173492</v>
       </c>
       <c r="V189" t="n">
         <v>1880000</v>
@@ -16461,7 +16461,7 @@
         <v>204.593</v>
       </c>
       <c r="Y197" t="n">
-        <v>11898666</v>
+        <v>11898665</v>
       </c>
     </row>
   </sheetData>
@@ -16587,12 +16587,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>$11,898,666</t>
+          <t>$11,898,665</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>$101,660,684</t>
+          <t>$101,660,686</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -16602,7 +16602,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>$205,415,393</t>
+          <t>$205,415,389</t>
         </is>
       </c>
     </row>
@@ -16619,12 +16619,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>$9,938,666</t>
+          <t>$9,938,665</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>$99,700,684</t>
+          <t>$99,700,686</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -16634,7 +16634,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>$203,455,393</t>
+          <t>$203,455,389</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Backtest-temp: add fully-invested 25% cap variant (equal-weight rebalance)
</commit_message>
<xml_diff>
--- a/backtest.xlsx
+++ b/backtest.xlsx
@@ -1773,7 +1773,7 @@
         <v>1059.3</v>
       </c>
       <c r="P16" t="n">
-        <v>85514.10000000001</v>
+        <v>85514</v>
       </c>
       <c r="Q16" t="n">
         <v>3734.9</v>
@@ -2502,7 +2502,7 @@
         <v>1653.3</v>
       </c>
       <c r="P25" t="n">
-        <v>124473.4</v>
+        <v>124473.5</v>
       </c>
       <c r="Q25" t="n">
         <v>5997.1</v>
@@ -3177,7 +3177,7 @@
         <v>1.216</v>
       </c>
       <c r="Y33" t="n">
-        <v>377065</v>
+        <v>377066</v>
       </c>
     </row>
     <row r="34">
@@ -3486,10 +3486,10 @@
         <v>0</v>
       </c>
       <c r="T37" t="n">
-        <v>434751</v>
+        <v>434750</v>
       </c>
       <c r="U37" t="n">
-        <v>434751</v>
+        <v>434750</v>
       </c>
       <c r="V37" t="n">
         <v>360000</v>
@@ -3987,7 +3987,7 @@
         <v>1.721</v>
       </c>
       <c r="Y43" t="n">
-        <v>551361</v>
+        <v>551360</v>
       </c>
     </row>
     <row r="44">
@@ -4554,7 +4554,7 @@
         <v>2.704</v>
       </c>
       <c r="Y50" t="n">
-        <v>720761</v>
+        <v>720760</v>
       </c>
     </row>
     <row r="51">
@@ -4770,7 +4770,7 @@
         <v>1744.2</v>
       </c>
       <c r="P53" t="n">
-        <v>311064.8</v>
+        <v>311064.9</v>
       </c>
       <c r="Q53" t="n">
         <v>6375.7</v>
@@ -4878,7 +4878,7 @@
         <v>3.097</v>
       </c>
       <c r="Y54" t="n">
-        <v>824700</v>
+        <v>824699</v>
       </c>
     </row>
     <row r="55">
@@ -4959,7 +4959,7 @@
         <v>3.558</v>
       </c>
       <c r="Y55" t="n">
-        <v>876002</v>
+        <v>876003</v>
       </c>
     </row>
     <row r="56">
@@ -5013,7 +5013,7 @@
         <v>1744.2</v>
       </c>
       <c r="P56" t="n">
-        <v>320066.1</v>
+        <v>320066.2</v>
       </c>
       <c r="Q56" t="n">
         <v>6375.7</v>
@@ -5268,10 +5268,10 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>1561239</v>
+        <v>1561240</v>
       </c>
       <c r="U59" t="n">
-        <v>1561239</v>
+        <v>1561240</v>
       </c>
       <c r="V59" t="n">
         <v>580000</v>
@@ -5592,10 +5592,10 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>1661896</v>
+        <v>1661897</v>
       </c>
       <c r="U63" t="n">
-        <v>1661896</v>
+        <v>1661897</v>
       </c>
       <c r="V63" t="n">
         <v>620000</v>
@@ -5607,7 +5607,7 @@
         <v>4.082</v>
       </c>
       <c r="Y63" t="n">
-        <v>1035916</v>
+        <v>1035917</v>
       </c>
     </row>
     <row r="64">
@@ -5673,10 +5673,10 @@
         <v>0</v>
       </c>
       <c r="T64" t="n">
-        <v>1896444</v>
+        <v>1896443</v>
       </c>
       <c r="U64" t="n">
-        <v>1896444</v>
+        <v>1896443</v>
       </c>
       <c r="V64" t="n">
         <v>630000</v>
@@ -5931,7 +5931,7 @@
         <v>3.326</v>
       </c>
       <c r="Y67" t="n">
-        <v>1044793</v>
+        <v>1044792</v>
       </c>
     </row>
     <row r="68">
@@ -6228,7 +6228,7 @@
         <v>1950.3</v>
       </c>
       <c r="P71" t="n">
-        <v>345701.7</v>
+        <v>345701.8</v>
       </c>
       <c r="Q71" t="n">
         <v>7245.6</v>
@@ -6309,7 +6309,7 @@
         <v>2002</v>
       </c>
       <c r="P72" t="n">
-        <v>345701.7</v>
+        <v>345701.8</v>
       </c>
       <c r="Q72" t="n">
         <v>7466.2</v>
@@ -6390,7 +6390,7 @@
         <v>2054.4</v>
       </c>
       <c r="P73" t="n">
-        <v>345701.7</v>
+        <v>345701.8</v>
       </c>
       <c r="Q73" t="n">
         <v>7683.6</v>
@@ -6417,7 +6417,7 @@
         <v>3.133</v>
       </c>
       <c r="Y73" t="n">
-        <v>1089447</v>
+        <v>1089446</v>
       </c>
     </row>
     <row r="74">
@@ -6471,7 +6471,7 @@
         <v>2103.5</v>
       </c>
       <c r="P74" t="n">
-        <v>345701.7</v>
+        <v>345701.8</v>
       </c>
       <c r="Q74" t="n">
         <v>7882.7</v>
@@ -6660,7 +6660,7 @@
         <v>3.902</v>
       </c>
       <c r="Y76" t="n">
-        <v>1206766</v>
+        <v>1206765</v>
       </c>
     </row>
     <row r="77">
@@ -7131,10 +7131,10 @@
         <v>0</v>
       </c>
       <c r="T82" t="n">
-        <v>2516508</v>
+        <v>2516509</v>
       </c>
       <c r="U82" t="n">
-        <v>2516508</v>
+        <v>2516509</v>
       </c>
       <c r="V82" t="n">
         <v>810000</v>
@@ -7293,10 +7293,10 @@
         <v>0</v>
       </c>
       <c r="T84" t="n">
-        <v>2968225</v>
+        <v>2968224</v>
       </c>
       <c r="U84" t="n">
-        <v>2968225</v>
+        <v>2968224</v>
       </c>
       <c r="V84" t="n">
         <v>830000</v>
@@ -7389,7 +7389,7 @@
         <v>7.072</v>
       </c>
       <c r="Y85" t="n">
-        <v>1532858</v>
+        <v>1532859</v>
       </c>
     </row>
     <row r="86">
@@ -7611,7 +7611,7 @@
         <v>7882.7</v>
       </c>
       <c r="R88" t="n">
-        <v>342207.5</v>
+        <v>342207.6</v>
       </c>
       <c r="S88" t="n">
         <v>0</v>
@@ -7698,10 +7698,10 @@
         <v>0</v>
       </c>
       <c r="T89" t="n">
-        <v>3798192</v>
+        <v>3798193</v>
       </c>
       <c r="U89" t="n">
-        <v>3798192</v>
+        <v>3798193</v>
       </c>
       <c r="V89" t="n">
         <v>880000</v>
@@ -7941,10 +7941,10 @@
         <v>0</v>
       </c>
       <c r="T92" t="n">
-        <v>4870741</v>
+        <v>4870742</v>
       </c>
       <c r="U92" t="n">
-        <v>4870741</v>
+        <v>4870742</v>
       </c>
       <c r="V92" t="n">
         <v>910000</v>
@@ -7956,7 +7956,7 @@
         <v>10.414</v>
       </c>
       <c r="Y92" t="n">
-        <v>1799588</v>
+        <v>1799589</v>
       </c>
     </row>
     <row r="93">
@@ -8022,10 +8022,10 @@
         <v>0</v>
       </c>
       <c r="T93" t="n">
-        <v>5877482</v>
+        <v>5877481</v>
       </c>
       <c r="U93" t="n">
-        <v>5877482</v>
+        <v>5877481</v>
       </c>
       <c r="V93" t="n">
         <v>920000</v>
@@ -8118,7 +8118,7 @@
         <v>12.671</v>
       </c>
       <c r="Y94" t="n">
-        <v>1939779</v>
+        <v>1939780</v>
       </c>
     </row>
     <row r="95">
@@ -8199,7 +8199,7 @@
         <v>12.358</v>
       </c>
       <c r="Y95" t="n">
-        <v>1961468</v>
+        <v>1961469</v>
       </c>
     </row>
     <row r="96">
@@ -8265,10 +8265,10 @@
         <v>0</v>
       </c>
       <c r="T96" t="n">
-        <v>7254015</v>
+        <v>7254016</v>
       </c>
       <c r="U96" t="n">
-        <v>7254015</v>
+        <v>7254016</v>
       </c>
       <c r="V96" t="n">
         <v>950000</v>
@@ -8427,10 +8427,10 @@
         <v>0</v>
       </c>
       <c r="T98" t="n">
-        <v>6277672</v>
+        <v>6277671</v>
       </c>
       <c r="U98" t="n">
-        <v>6277672</v>
+        <v>6277671</v>
       </c>
       <c r="V98" t="n">
         <v>970000</v>
@@ -8508,10 +8508,10 @@
         <v>0</v>
       </c>
       <c r="T99" t="n">
-        <v>5568499</v>
+        <v>5568498</v>
       </c>
       <c r="U99" t="n">
-        <v>5568499</v>
+        <v>5568498</v>
       </c>
       <c r="V99" t="n">
         <v>980000</v>
@@ -8523,7 +8523,7 @@
         <v>11.772</v>
       </c>
       <c r="Y99" t="n">
-        <v>2069156</v>
+        <v>2069155</v>
       </c>
     </row>
     <row r="100">
@@ -8604,7 +8604,7 @@
         <v>14.706</v>
       </c>
       <c r="Y100" t="n">
-        <v>2196527</v>
+        <v>2196528</v>
       </c>
     </row>
     <row r="101">
@@ -8658,7 +8658,7 @@
         <v>2103.5</v>
       </c>
       <c r="P101" t="n">
-        <v>384909.5</v>
+        <v>384909.6</v>
       </c>
       <c r="Q101" t="n">
         <v>7882.7</v>
@@ -8670,10 +8670,10 @@
         <v>0</v>
       </c>
       <c r="T101" t="n">
-        <v>6498413</v>
+        <v>6498414</v>
       </c>
       <c r="U101" t="n">
-        <v>6498413</v>
+        <v>6498414</v>
       </c>
       <c r="V101" t="n">
         <v>1000000</v>
@@ -8751,10 +8751,10 @@
         <v>0</v>
       </c>
       <c r="T102" t="n">
-        <v>7078887</v>
+        <v>7078886</v>
       </c>
       <c r="U102" t="n">
-        <v>7078887</v>
+        <v>7078886</v>
       </c>
       <c r="V102" t="n">
         <v>1010000</v>
@@ -8913,10 +8913,10 @@
         <v>0</v>
       </c>
       <c r="T104" t="n">
-        <v>7517179</v>
+        <v>7517181</v>
       </c>
       <c r="U104" t="n">
-        <v>7517179</v>
+        <v>7517181</v>
       </c>
       <c r="V104" t="n">
         <v>1030000</v>
@@ -9063,7 +9063,7 @@
         <v>2134.4</v>
       </c>
       <c r="P106" t="n">
-        <v>387588.2</v>
+        <v>387588.3</v>
       </c>
       <c r="Q106" t="n">
         <v>7997.5</v>
@@ -9144,7 +9144,7 @@
         <v>2168.3</v>
       </c>
       <c r="P107" t="n">
-        <v>387588.2</v>
+        <v>387588.3</v>
       </c>
       <c r="Q107" t="n">
         <v>8118</v>
@@ -9318,10 +9318,10 @@
         <v>0</v>
       </c>
       <c r="T109" t="n">
-        <v>6004060</v>
+        <v>6004059</v>
       </c>
       <c r="U109" t="n">
-        <v>6004060</v>
+        <v>6004059</v>
       </c>
       <c r="V109" t="n">
         <v>1080000</v>
@@ -9408,7 +9408,7 @@
         <v>1090000</v>
       </c>
       <c r="W110" t="n">
-        <v>8.960000000000001</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="X110" t="n">
         <v>13.603</v>
@@ -9495,7 +9495,7 @@
         <v>17.025</v>
       </c>
       <c r="Y111" t="n">
-        <v>2589009</v>
+        <v>2589010</v>
       </c>
     </row>
     <row r="112">
@@ -9576,7 +9576,7 @@
         <v>11.4</v>
       </c>
       <c r="Y112" t="n">
-        <v>2386050</v>
+        <v>2386049</v>
       </c>
     </row>
     <row r="113">
@@ -9642,10 +9642,10 @@
         <v>0</v>
       </c>
       <c r="T113" t="n">
-        <v>7101969</v>
+        <v>7101970</v>
       </c>
       <c r="U113" t="n">
-        <v>7101969</v>
+        <v>7101970</v>
       </c>
       <c r="V113" t="n">
         <v>1120000</v>
@@ -9657,7 +9657,7 @@
         <v>14.679</v>
       </c>
       <c r="Y113" t="n">
-        <v>2577142</v>
+        <v>2577141</v>
       </c>
     </row>
     <row r="114">
@@ -9723,10 +9723,10 @@
         <v>0</v>
       </c>
       <c r="T114" t="n">
-        <v>7877042</v>
+        <v>7877043</v>
       </c>
       <c r="U114" t="n">
-        <v>7877042</v>
+        <v>7877043</v>
       </c>
       <c r="V114" t="n">
         <v>1130000</v>
@@ -9738,7 +9738,7 @@
         <v>16.261</v>
       </c>
       <c r="Y114" t="n">
-        <v>2647303</v>
+        <v>2647302</v>
       </c>
     </row>
     <row r="115">
@@ -9804,10 +9804,10 @@
         <v>0</v>
       </c>
       <c r="T115" t="n">
-        <v>7231596</v>
+        <v>7231597</v>
       </c>
       <c r="U115" t="n">
-        <v>7231596</v>
+        <v>7231597</v>
       </c>
       <c r="V115" t="n">
         <v>1140000</v>
@@ -9819,7 +9819,7 @@
         <v>14.907</v>
       </c>
       <c r="Y115" t="n">
-        <v>2607007</v>
+        <v>2607006</v>
       </c>
     </row>
     <row r="116">
@@ -9900,7 +9900,7 @@
         <v>15.8</v>
       </c>
       <c r="Y116" t="n">
-        <v>2640926</v>
+        <v>2640925</v>
       </c>
     </row>
     <row r="117">
@@ -9966,10 +9966,10 @@
         <v>0</v>
       </c>
       <c r="T117" t="n">
-        <v>8740734</v>
+        <v>8740736</v>
       </c>
       <c r="U117" t="n">
-        <v>8740734</v>
+        <v>8740736</v>
       </c>
       <c r="V117" t="n">
         <v>1160000</v>
@@ -9981,7 +9981,7 @@
         <v>17.974</v>
       </c>
       <c r="Y117" t="n">
-        <v>2766589</v>
+        <v>2766590</v>
       </c>
     </row>
     <row r="118">
@@ -10035,7 +10035,7 @@
         <v>2168.3</v>
       </c>
       <c r="P118" t="n">
-        <v>395333.3</v>
+        <v>395333.4</v>
       </c>
       <c r="Q118" t="n">
         <v>8118</v>
@@ -10047,10 +10047,10 @@
         <v>0</v>
       </c>
       <c r="T118" t="n">
-        <v>9720973</v>
+        <v>9720972</v>
       </c>
       <c r="U118" t="n">
-        <v>9720973</v>
+        <v>9720972</v>
       </c>
       <c r="V118" t="n">
         <v>1170000</v>
@@ -10128,10 +10128,10 @@
         <v>0</v>
       </c>
       <c r="T119" t="n">
-        <v>11444852</v>
+        <v>11444853</v>
       </c>
       <c r="U119" t="n">
-        <v>11444852</v>
+        <v>11444853</v>
       </c>
       <c r="V119" t="n">
         <v>1180000</v>
@@ -10290,10 +10290,10 @@
         <v>0</v>
       </c>
       <c r="T121" t="n">
-        <v>9345550</v>
+        <v>9345549</v>
       </c>
       <c r="U121" t="n">
-        <v>9345550</v>
+        <v>9345549</v>
       </c>
       <c r="V121" t="n">
         <v>1200000</v>
@@ -10305,7 +10305,7 @@
         <v>19.144</v>
       </c>
       <c r="Y121" t="n">
-        <v>2934354</v>
+        <v>2934355</v>
       </c>
     </row>
     <row r="122">
@@ -10452,10 +10452,10 @@
         <v>0</v>
       </c>
       <c r="T123" t="n">
-        <v>7350995</v>
+        <v>7350996</v>
       </c>
       <c r="U123" t="n">
-        <v>7350995</v>
+        <v>7350996</v>
       </c>
       <c r="V123" t="n">
         <v>1220000</v>
@@ -10533,10 +10533,10 @@
         <v>0</v>
       </c>
       <c r="T124" t="n">
-        <v>8576081</v>
+        <v>8576082</v>
       </c>
       <c r="U124" t="n">
-        <v>8576081</v>
+        <v>8576082</v>
       </c>
       <c r="V124" t="n">
         <v>1230000</v>
@@ -10614,10 +10614,10 @@
         <v>0</v>
       </c>
       <c r="T125" t="n">
-        <v>10167703</v>
+        <v>10167704</v>
       </c>
       <c r="U125" t="n">
-        <v>10167703</v>
+        <v>10167704</v>
       </c>
       <c r="V125" t="n">
         <v>1240000</v>
@@ -10695,10 +10695,10 @@
         <v>0</v>
       </c>
       <c r="T126" t="n">
-        <v>12195955</v>
+        <v>12195956</v>
       </c>
       <c r="U126" t="n">
-        <v>12195955</v>
+        <v>12195956</v>
       </c>
       <c r="V126" t="n">
         <v>1250000</v>
@@ -10710,7 +10710,7 @@
         <v>24.828</v>
       </c>
       <c r="Y126" t="n">
-        <v>3862620</v>
+        <v>3862622</v>
       </c>
     </row>
     <row r="127">
@@ -10776,10 +10776,10 @@
         <v>0</v>
       </c>
       <c r="T127" t="n">
-        <v>15247650</v>
+        <v>15247647</v>
       </c>
       <c r="U127" t="n">
-        <v>15247650</v>
+        <v>15247647</v>
       </c>
       <c r="V127" t="n">
         <v>1260000</v>
@@ -10857,10 +10857,10 @@
         <v>0</v>
       </c>
       <c r="T128" t="n">
-        <v>13443231</v>
+        <v>13443232</v>
       </c>
       <c r="U128" t="n">
-        <v>13443231</v>
+        <v>13443232</v>
       </c>
       <c r="V128" t="n">
         <v>1270000</v>
@@ -10938,10 +10938,10 @@
         <v>0</v>
       </c>
       <c r="T129" t="n">
-        <v>12699328</v>
+        <v>12699329</v>
       </c>
       <c r="U129" t="n">
-        <v>12699328</v>
+        <v>12699329</v>
       </c>
       <c r="V129" t="n">
         <v>1280000</v>
@@ -11034,7 +11034,7 @@
         <v>37.565</v>
       </c>
       <c r="Y130" t="n">
-        <v>4396285</v>
+        <v>4396284</v>
       </c>
     </row>
     <row r="131">
@@ -11100,10 +11100,10 @@
         <v>0</v>
       </c>
       <c r="T131" t="n">
-        <v>21134549</v>
+        <v>21134550</v>
       </c>
       <c r="U131" t="n">
-        <v>21134549</v>
+        <v>21134550</v>
       </c>
       <c r="V131" t="n">
         <v>1300000</v>
@@ -11115,7 +11115,7 @@
         <v>42.888</v>
       </c>
       <c r="Y131" t="n">
-        <v>4621798</v>
+        <v>4621800</v>
       </c>
     </row>
     <row r="132">
@@ -11181,10 +11181,10 @@
         <v>0</v>
       </c>
       <c r="T132" t="n">
-        <v>21944520</v>
+        <v>21944519</v>
       </c>
       <c r="U132" t="n">
-        <v>21944520</v>
+        <v>21944519</v>
       </c>
       <c r="V132" t="n">
         <v>1310000</v>
@@ -11196,7 +11196,7 @@
         <v>44.511</v>
       </c>
       <c r="Y132" t="n">
-        <v>4643869</v>
+        <v>4643870</v>
       </c>
     </row>
     <row r="133">
@@ -11262,10 +11262,10 @@
         <v>0</v>
       </c>
       <c r="T133" t="n">
-        <v>23751399</v>
+        <v>23751397</v>
       </c>
       <c r="U133" t="n">
-        <v>23751399</v>
+        <v>23751397</v>
       </c>
       <c r="V133" t="n">
         <v>1320000</v>
@@ -11343,10 +11343,10 @@
         <v>0</v>
       </c>
       <c r="T134" t="n">
-        <v>23809374</v>
+        <v>23809376</v>
       </c>
       <c r="U134" t="n">
-        <v>23809374</v>
+        <v>23809376</v>
       </c>
       <c r="V134" t="n">
         <v>1330000</v>
@@ -11505,10 +11505,10 @@
         <v>0</v>
       </c>
       <c r="T136" t="n">
-        <v>25164171</v>
+        <v>25164173</v>
       </c>
       <c r="U136" t="n">
-        <v>25164171</v>
+        <v>25164173</v>
       </c>
       <c r="V136" t="n">
         <v>1350000</v>
@@ -11520,7 +11520,7 @@
         <v>50.958</v>
       </c>
       <c r="Y136" t="n">
-        <v>4977001</v>
+        <v>4977002</v>
       </c>
     </row>
     <row r="137">
@@ -11586,10 +11586,10 @@
         <v>0</v>
       </c>
       <c r="T137" t="n">
-        <v>29189209</v>
+        <v>29189207</v>
       </c>
       <c r="U137" t="n">
-        <v>29189209</v>
+        <v>29189207</v>
       </c>
       <c r="V137" t="n">
         <v>1360000</v>
@@ -11601,7 +11601,7 @@
         <v>59.089</v>
       </c>
       <c r="Y137" t="n">
-        <v>5298659</v>
+        <v>5298658</v>
       </c>
     </row>
     <row r="138">
@@ -11667,10 +11667,10 @@
         <v>0</v>
       </c>
       <c r="T138" t="n">
-        <v>30149069</v>
+        <v>30149068</v>
       </c>
       <c r="U138" t="n">
-        <v>30149069</v>
+        <v>30149068</v>
       </c>
       <c r="V138" t="n">
         <v>1370000</v>
@@ -11682,7 +11682,7 @@
         <v>61.012</v>
       </c>
       <c r="Y138" t="n">
-        <v>5460240</v>
+        <v>5460239</v>
       </c>
     </row>
     <row r="139">
@@ -11748,10 +11748,10 @@
         <v>0</v>
       </c>
       <c r="T139" t="n">
-        <v>32579498</v>
+        <v>32579500</v>
       </c>
       <c r="U139" t="n">
-        <v>32579498</v>
+        <v>32579500</v>
       </c>
       <c r="V139" t="n">
         <v>1380000</v>
@@ -11829,10 +11829,10 @@
         <v>0</v>
       </c>
       <c r="T140" t="n">
-        <v>27821990</v>
+        <v>27821992</v>
       </c>
       <c r="U140" t="n">
-        <v>27821990</v>
+        <v>27821992</v>
       </c>
       <c r="V140" t="n">
         <v>1390000</v>
@@ -11844,7 +11844,7 @@
         <v>56.265</v>
       </c>
       <c r="Y140" t="n">
-        <v>5386596</v>
+        <v>5386597</v>
       </c>
     </row>
     <row r="141">
@@ -11910,10 +11910,10 @@
         <v>0</v>
       </c>
       <c r="T141" t="n">
-        <v>33553107</v>
+        <v>33553109</v>
       </c>
       <c r="U141" t="n">
-        <v>33553107</v>
+        <v>33553109</v>
       </c>
       <c r="V141" t="n">
         <v>1400000</v>
@@ -11925,7 +11925,7 @@
         <v>67.83499999999999</v>
       </c>
       <c r="Y141" t="n">
-        <v>5820190</v>
+        <v>5820189</v>
       </c>
     </row>
     <row r="142">
@@ -11991,10 +11991,10 @@
         <v>0</v>
       </c>
       <c r="T142" t="n">
-        <v>40473532</v>
+        <v>40473533</v>
       </c>
       <c r="U142" t="n">
-        <v>40473532</v>
+        <v>40473533</v>
       </c>
       <c r="V142" t="n">
         <v>1410000</v>
@@ -12066,16 +12066,16 @@
         <v>8800.9</v>
       </c>
       <c r="R143" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S143" t="n">
         <v>0</v>
       </c>
       <c r="T143" t="n">
-        <v>41964989</v>
+        <v>41964997</v>
       </c>
       <c r="U143" t="n">
-        <v>41964989</v>
+        <v>41964997</v>
       </c>
       <c r="V143" t="n">
         <v>1420000</v>
@@ -12087,7 +12087,7 @@
         <v>84.8</v>
       </c>
       <c r="Y143" t="n">
-        <v>6024911</v>
+        <v>6024912</v>
       </c>
     </row>
     <row r="144">
@@ -12147,16 +12147,16 @@
         <v>8838.1</v>
       </c>
       <c r="R144" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S144" t="n">
         <v>0</v>
       </c>
       <c r="T144" t="n">
-        <v>29465119</v>
+        <v>29465117</v>
       </c>
       <c r="U144" t="n">
-        <v>29465119</v>
+        <v>29465117</v>
       </c>
       <c r="V144" t="n">
         <v>1430000</v>
@@ -12168,7 +12168,7 @@
         <v>59.521</v>
       </c>
       <c r="Y144" t="n">
-        <v>5507902</v>
+        <v>5507901</v>
       </c>
     </row>
     <row r="145">
@@ -12228,16 +12228,16 @@
         <v>8876.299999999999</v>
       </c>
       <c r="R145" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S145" t="n">
         <v>0</v>
       </c>
       <c r="T145" t="n">
-        <v>26366606</v>
+        <v>26366604</v>
       </c>
       <c r="U145" t="n">
-        <v>26366606</v>
+        <v>26366604</v>
       </c>
       <c r="V145" t="n">
         <v>1440000</v>
@@ -12249,7 +12249,7 @@
         <v>53.242</v>
       </c>
       <c r="Y145" t="n">
-        <v>5271359</v>
+        <v>5271358</v>
       </c>
     </row>
     <row r="146">
@@ -12309,16 +12309,16 @@
         <v>8914.299999999999</v>
       </c>
       <c r="R146" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S146" t="n">
         <v>0</v>
       </c>
       <c r="T146" t="n">
-        <v>26733466</v>
+        <v>26733469</v>
       </c>
       <c r="U146" t="n">
-        <v>26733466</v>
+        <v>26733469</v>
       </c>
       <c r="V146" t="n">
         <v>1450000</v>
@@ -12390,16 +12390,16 @@
         <v>8958.799999999999</v>
       </c>
       <c r="R147" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S147" t="n">
         <v>0</v>
       </c>
       <c r="T147" t="n">
-        <v>16522120</v>
+        <v>16522123</v>
       </c>
       <c r="U147" t="n">
-        <v>16522120</v>
+        <v>16522123</v>
       </c>
       <c r="V147" t="n">
         <v>1460000</v>
@@ -12471,16 +12471,16 @@
         <v>9000.700000000001</v>
       </c>
       <c r="R148" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S148" t="n">
         <v>0</v>
       </c>
       <c r="T148" t="n">
-        <v>16839657</v>
+        <v>16839658</v>
       </c>
       <c r="U148" t="n">
-        <v>16839657</v>
+        <v>16839658</v>
       </c>
       <c r="V148" t="n">
         <v>1470000</v>
@@ -12552,16 +12552,16 @@
         <v>9051</v>
       </c>
       <c r="R149" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S149" t="n">
         <v>0</v>
       </c>
       <c r="T149" t="n">
-        <v>10759378</v>
+        <v>10759377</v>
       </c>
       <c r="U149" t="n">
-        <v>10759378</v>
+        <v>10759377</v>
       </c>
       <c r="V149" t="n">
         <v>1480000</v>
@@ -12633,16 +12633,16 @@
         <v>9094.1</v>
       </c>
       <c r="R150" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S150" t="n">
         <v>0</v>
       </c>
       <c r="T150" t="n">
-        <v>15151252</v>
+        <v>15151250</v>
       </c>
       <c r="U150" t="n">
-        <v>15151252</v>
+        <v>15151250</v>
       </c>
       <c r="V150" t="n">
         <v>1490000</v>
@@ -12714,16 +12714,16 @@
         <v>9141.9</v>
       </c>
       <c r="R151" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S151" t="n">
         <v>0</v>
       </c>
       <c r="T151" t="n">
-        <v>11929512</v>
+        <v>11929511</v>
       </c>
       <c r="U151" t="n">
-        <v>11929512</v>
+        <v>11929511</v>
       </c>
       <c r="V151" t="n">
         <v>1500000</v>
@@ -12795,16 +12795,16 @@
         <v>9197.200000000001</v>
       </c>
       <c r="R152" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S152" t="n">
         <v>0</v>
       </c>
       <c r="T152" t="n">
-        <v>8302175</v>
+        <v>8302176</v>
       </c>
       <c r="U152" t="n">
-        <v>8302175</v>
+        <v>8302176</v>
       </c>
       <c r="V152" t="n">
         <v>1510000</v>
@@ -12876,16 +12876,16 @@
         <v>9251.299999999999</v>
       </c>
       <c r="R153" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S153" t="n">
         <v>0</v>
       </c>
       <c r="T153" t="n">
-        <v>8689213</v>
+        <v>8689212</v>
       </c>
       <c r="U153" t="n">
-        <v>8689213</v>
+        <v>8689212</v>
       </c>
       <c r="V153" t="n">
         <v>1520000</v>
@@ -12897,7 +12897,7 @@
         <v>17.435</v>
       </c>
       <c r="Y153" t="n">
-        <v>4319853</v>
+        <v>4319854</v>
       </c>
     </row>
     <row r="154">
@@ -12957,7 +12957,7 @@
         <v>9296.299999999999</v>
       </c>
       <c r="R154" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S154" t="n">
         <v>0</v>
@@ -12978,7 +12978,7 @@
         <v>22.324</v>
       </c>
       <c r="Y154" t="n">
-        <v>4569342</v>
+        <v>4569343</v>
       </c>
     </row>
     <row r="155">
@@ -13038,16 +13038,16 @@
         <v>9346.200000000001</v>
       </c>
       <c r="R155" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S155" t="n">
         <v>0</v>
       </c>
       <c r="T155" t="n">
-        <v>8350213</v>
+        <v>8350214</v>
       </c>
       <c r="U155" t="n">
-        <v>8350213</v>
+        <v>8350214</v>
       </c>
       <c r="V155" t="n">
         <v>1540000</v>
@@ -13059,7 +13059,7 @@
         <v>16.72</v>
       </c>
       <c r="Y155" t="n">
-        <v>4167468</v>
+        <v>4167467</v>
       </c>
     </row>
     <row r="156">
@@ -13119,7 +13119,7 @@
         <v>9388.9</v>
       </c>
       <c r="R156" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S156" t="n">
         <v>0</v>
@@ -13140,7 +13140,7 @@
         <v>22.767</v>
       </c>
       <c r="Y156" t="n">
-        <v>4620997</v>
+        <v>4620998</v>
       </c>
     </row>
     <row r="157">
@@ -13200,16 +13200,16 @@
         <v>9431.200000000001</v>
       </c>
       <c r="R157" t="n">
-        <v>361336.1</v>
+        <v>361336.2</v>
       </c>
       <c r="S157" t="n">
         <v>0</v>
       </c>
       <c r="T157" t="n">
-        <v>11294702</v>
+        <v>11294701</v>
       </c>
       <c r="U157" t="n">
-        <v>11294702</v>
+        <v>11294701</v>
       </c>
       <c r="V157" t="n">
         <v>1560000</v>
@@ -13287,10 +13287,10 @@
         <v>0</v>
       </c>
       <c r="T158" t="n">
-        <v>13994543</v>
+        <v>13994544</v>
       </c>
       <c r="U158" t="n">
-        <v>13994543</v>
+        <v>13994544</v>
       </c>
       <c r="V158" t="n">
         <v>1570000</v>
@@ -13302,7 +13302,7 @@
         <v>27.952</v>
       </c>
       <c r="Y158" t="n">
-        <v>5062380</v>
+        <v>5062381</v>
       </c>
     </row>
     <row r="159">
@@ -13368,10 +13368,10 @@
         <v>0</v>
       </c>
       <c r="T159" t="n">
-        <v>12490340</v>
+        <v>12490341</v>
       </c>
       <c r="U159" t="n">
-        <v>12490340</v>
+        <v>12490341</v>
       </c>
       <c r="V159" t="n">
         <v>1580000</v>
@@ -13383,7 +13383,7 @@
         <v>24.928</v>
       </c>
       <c r="Y159" t="n">
-        <v>5098082</v>
+        <v>5098083</v>
       </c>
     </row>
     <row r="160">
@@ -13437,22 +13437,22 @@
         <v>2632.1</v>
       </c>
       <c r="P160" t="n">
-        <v>400441.7</v>
+        <v>400441.8</v>
       </c>
       <c r="Q160" t="n">
         <v>9431.200000000001</v>
       </c>
       <c r="R160" t="n">
-        <v>362213.8</v>
+        <v>362213.9</v>
       </c>
       <c r="S160" t="n">
         <v>0</v>
       </c>
       <c r="T160" t="n">
-        <v>16469314</v>
+        <v>16469315</v>
       </c>
       <c r="U160" t="n">
-        <v>16469314</v>
+        <v>16469315</v>
       </c>
       <c r="V160" t="n">
         <v>1590000</v>
@@ -13518,22 +13518,22 @@
         <v>2645.8</v>
       </c>
       <c r="P161" t="n">
-        <v>400441.7</v>
+        <v>400441.8</v>
       </c>
       <c r="Q161" t="n">
         <v>9464.4</v>
       </c>
       <c r="R161" t="n">
-        <v>362213.8</v>
+        <v>362213.9</v>
       </c>
       <c r="S161" t="n">
         <v>0</v>
       </c>
       <c r="T161" t="n">
-        <v>19163121</v>
+        <v>19163120</v>
       </c>
       <c r="U161" t="n">
-        <v>19163121</v>
+        <v>19163120</v>
       </c>
       <c r="V161" t="n">
         <v>1600000</v>
@@ -13545,7 +13545,7 @@
         <v>38.202</v>
       </c>
       <c r="Y161" t="n">
-        <v>5867328</v>
+        <v>5867327</v>
       </c>
     </row>
     <row r="162">
@@ -13599,7 +13599,7 @@
         <v>2645.8</v>
       </c>
       <c r="P162" t="n">
-        <v>400669.3</v>
+        <v>400669.4</v>
       </c>
       <c r="Q162" t="n">
         <v>9464.4</v>
@@ -13611,10 +13611,10 @@
         <v>0</v>
       </c>
       <c r="T162" t="n">
-        <v>21397102</v>
+        <v>21397100</v>
       </c>
       <c r="U162" t="n">
-        <v>21397102</v>
+        <v>21397100</v>
       </c>
       <c r="V162" t="n">
         <v>1610000</v>
@@ -13626,7 +13626,7 @@
         <v>42.635</v>
       </c>
       <c r="Y162" t="n">
-        <v>6103803</v>
+        <v>6103801</v>
       </c>
     </row>
     <row r="163">
@@ -13707,7 +13707,7 @@
         <v>38.189</v>
       </c>
       <c r="Y163" t="n">
-        <v>6023272</v>
+        <v>6023271</v>
       </c>
     </row>
     <row r="164">
@@ -13773,10 +13773,10 @@
         <v>0</v>
       </c>
       <c r="T164" t="n">
-        <v>15966068</v>
+        <v>15966069</v>
       </c>
       <c r="U164" t="n">
-        <v>15966068</v>
+        <v>15966069</v>
       </c>
       <c r="V164" t="n">
         <v>1630000</v>
@@ -13788,7 +13788,7 @@
         <v>31.777</v>
       </c>
       <c r="Y164" t="n">
-        <v>5727289</v>
+        <v>5727288</v>
       </c>
     </row>
     <row r="165">
@@ -13854,10 +13854,10 @@
         <v>0</v>
       </c>
       <c r="T165" t="n">
-        <v>13930308</v>
+        <v>13930310</v>
       </c>
       <c r="U165" t="n">
-        <v>13930308</v>
+        <v>13930310</v>
       </c>
       <c r="V165" t="n">
         <v>1640000</v>
@@ -13929,7 +13929,7 @@
         <v>9464.4</v>
       </c>
       <c r="R166" t="n">
-        <v>363439.2</v>
+        <v>363439.3</v>
       </c>
       <c r="S166" t="n">
         <v>0</v>
@@ -14016,10 +14016,10 @@
         <v>0</v>
       </c>
       <c r="T167" t="n">
-        <v>23911805</v>
+        <v>23911806</v>
       </c>
       <c r="U167" t="n">
-        <v>23911805</v>
+        <v>23911806</v>
       </c>
       <c r="V167" t="n">
         <v>1660000</v>
@@ -14097,10 +14097,10 @@
         <v>0</v>
       </c>
       <c r="T168" t="n">
-        <v>24676081</v>
+        <v>24676082</v>
       </c>
       <c r="U168" t="n">
-        <v>24676081</v>
+        <v>24676082</v>
       </c>
       <c r="V168" t="n">
         <v>1670000</v>
@@ -14178,10 +14178,10 @@
         <v>0</v>
       </c>
       <c r="T169" t="n">
-        <v>30353798</v>
+        <v>30353797</v>
       </c>
       <c r="U169" t="n">
-        <v>30353798</v>
+        <v>30353797</v>
       </c>
       <c r="V169" t="n">
         <v>1680000</v>
@@ -14193,7 +14193,7 @@
         <v>60.269</v>
       </c>
       <c r="Y169" t="n">
-        <v>7090605</v>
+        <v>7090606</v>
       </c>
     </row>
     <row r="170">
@@ -14259,10 +14259,10 @@
         <v>0</v>
       </c>
       <c r="T170" t="n">
-        <v>32116992</v>
+        <v>32116993</v>
       </c>
       <c r="U170" t="n">
-        <v>32116992</v>
+        <v>32116993</v>
       </c>
       <c r="V170" t="n">
         <v>1690000</v>
@@ -14274,7 +14274,7 @@
         <v>63.75</v>
       </c>
       <c r="Y170" t="n">
-        <v>7190999</v>
+        <v>7190998</v>
       </c>
     </row>
     <row r="171">
@@ -14340,10 +14340,10 @@
         <v>0</v>
       </c>
       <c r="T171" t="n">
-        <v>27237246</v>
+        <v>27237247</v>
       </c>
       <c r="U171" t="n">
-        <v>27237246</v>
+        <v>27237247</v>
       </c>
       <c r="V171" t="n">
         <v>1700000</v>
@@ -14421,10 +14421,10 @@
         <v>0</v>
       </c>
       <c r="T172" t="n">
-        <v>33233012</v>
+        <v>33233015</v>
       </c>
       <c r="U172" t="n">
-        <v>33233012</v>
+        <v>33233015</v>
       </c>
       <c r="V172" t="n">
         <v>1710000</v>
@@ -14436,7 +14436,7 @@
         <v>65.92100000000001</v>
       </c>
       <c r="Y172" t="n">
-        <v>7320104</v>
+        <v>7320103</v>
       </c>
     </row>
     <row r="173">
@@ -14496,16 +14496,16 @@
         <v>9464.4</v>
       </c>
       <c r="R173" t="n">
-        <v>364313.9</v>
+        <v>364314</v>
       </c>
       <c r="S173" t="n">
         <v>0</v>
       </c>
       <c r="T173" t="n">
-        <v>38280842</v>
+        <v>38280846</v>
       </c>
       <c r="U173" t="n">
-        <v>38280842</v>
+        <v>38280846</v>
       </c>
       <c r="V173" t="n">
         <v>1720000</v>
@@ -14517,7 +14517,7 @@
         <v>75.914</v>
       </c>
       <c r="Y173" t="n">
-        <v>7803713</v>
+        <v>7803714</v>
       </c>
     </row>
     <row r="174">
@@ -14583,10 +14583,10 @@
         <v>0</v>
       </c>
       <c r="T174" t="n">
-        <v>33090702</v>
+        <v>33090703</v>
       </c>
       <c r="U174" t="n">
-        <v>33090702</v>
+        <v>33090703</v>
       </c>
       <c r="V174" t="n">
         <v>1730000</v>
@@ -14598,7 +14598,7 @@
         <v>65.602</v>
       </c>
       <c r="Y174" t="n">
-        <v>7682749</v>
+        <v>7682748</v>
       </c>
     </row>
     <row r="175">
@@ -14637,7 +14637,7 @@
         <v>0</v>
       </c>
       <c r="K175" t="n">
-        <v>471.85</v>
+        <v>471.84</v>
       </c>
       <c r="L175" t="n">
         <v>33.75</v>
@@ -14658,16 +14658,16 @@
         <v>9464.4</v>
       </c>
       <c r="R175" t="n">
-        <v>364557.9</v>
+        <v>364558</v>
       </c>
       <c r="S175" t="n">
         <v>0</v>
       </c>
       <c r="T175" t="n">
-        <v>31128408</v>
+        <v>31128411</v>
       </c>
       <c r="U175" t="n">
-        <v>31128408</v>
+        <v>31128411</v>
       </c>
       <c r="V175" t="n">
         <v>1740000</v>
@@ -14745,10 +14745,10 @@
         <v>0</v>
       </c>
       <c r="T176" t="n">
-        <v>31268446</v>
+        <v>31268447</v>
       </c>
       <c r="U176" t="n">
-        <v>31268446</v>
+        <v>31268447</v>
       </c>
       <c r="V176" t="n">
         <v>1750000</v>
@@ -14826,10 +14826,10 @@
         <v>0</v>
       </c>
       <c r="T177" t="n">
-        <v>28245894</v>
+        <v>28245897</v>
       </c>
       <c r="U177" t="n">
-        <v>28245894</v>
+        <v>28245897</v>
       </c>
       <c r="V177" t="n">
         <v>1760000</v>
@@ -14841,7 +14841,7 @@
         <v>55.941</v>
       </c>
       <c r="Y177" t="n">
-        <v>7932325</v>
+        <v>7932326</v>
       </c>
     </row>
     <row r="178">
@@ -14895,7 +14895,7 @@
         <v>2656.2</v>
       </c>
       <c r="P178" t="n">
-        <v>403536.8</v>
+        <v>403536.9</v>
       </c>
       <c r="Q178" t="n">
         <v>9485.299999999999</v>
@@ -14988,10 +14988,10 @@
         <v>0</v>
       </c>
       <c r="T179" t="n">
-        <v>29357463</v>
+        <v>29357462</v>
       </c>
       <c r="U179" t="n">
-        <v>29357463</v>
+        <v>29357462</v>
       </c>
       <c r="V179" t="n">
         <v>1780000</v>
@@ -15003,7 +15003,7 @@
         <v>58.103</v>
       </c>
       <c r="Y179" t="n">
-        <v>8414739</v>
+        <v>8414738</v>
       </c>
     </row>
     <row r="180">
@@ -15084,7 +15084,7 @@
         <v>59.4</v>
       </c>
       <c r="Y180" t="n">
-        <v>8606773</v>
+        <v>8606772</v>
       </c>
     </row>
     <row r="181">
@@ -15150,10 +15150,10 @@
         <v>0</v>
       </c>
       <c r="T181" t="n">
-        <v>26776824</v>
+        <v>26776825</v>
       </c>
       <c r="U181" t="n">
-        <v>26776824</v>
+        <v>26776825</v>
       </c>
       <c r="V181" t="n">
         <v>1800000</v>
@@ -15231,10 +15231,10 @@
         <v>0</v>
       </c>
       <c r="T182" t="n">
-        <v>20550299</v>
+        <v>20550300</v>
       </c>
       <c r="U182" t="n">
-        <v>20550299</v>
+        <v>20550300</v>
       </c>
       <c r="V182" t="n">
         <v>1810000</v>
@@ -15246,7 +15246,7 @@
         <v>40.624</v>
       </c>
       <c r="Y182" t="n">
-        <v>7758039</v>
+        <v>7758040</v>
       </c>
     </row>
     <row r="183">
@@ -15393,10 +15393,10 @@
         <v>0</v>
       </c>
       <c r="T184" t="n">
-        <v>23599915</v>
+        <v>23599916</v>
       </c>
       <c r="U184" t="n">
-        <v>23599915</v>
+        <v>23599916</v>
       </c>
       <c r="V184" t="n">
         <v>1830000</v>
@@ -15555,10 +15555,10 @@
         <v>0</v>
       </c>
       <c r="T186" t="n">
-        <v>31150712</v>
+        <v>31150711</v>
       </c>
       <c r="U186" t="n">
-        <v>31150712</v>
+        <v>31150711</v>
       </c>
       <c r="V186" t="n">
         <v>1850000</v>
@@ -15630,7 +15630,7 @@
         <v>9553.6</v>
       </c>
       <c r="R187" t="n">
-        <v>366057.3</v>
+        <v>366057.4</v>
       </c>
       <c r="S187" t="n">
         <v>0</v>
@@ -15717,10 +15717,10 @@
         <v>0</v>
       </c>
       <c r="T188" t="n">
-        <v>38314372</v>
+        <v>38314373</v>
       </c>
       <c r="U188" t="n">
-        <v>38314372</v>
+        <v>38314373</v>
       </c>
       <c r="V188" t="n">
         <v>1870000</v>
@@ -15798,10 +15798,10 @@
         <v>0</v>
       </c>
       <c r="T189" t="n">
-        <v>46173492</v>
+        <v>46173493</v>
       </c>
       <c r="U189" t="n">
-        <v>46173492</v>
+        <v>46173493</v>
       </c>
       <c r="V189" t="n">
         <v>1880000</v>
@@ -15960,10 +15960,10 @@
         <v>0</v>
       </c>
       <c r="T191" t="n">
-        <v>41792364</v>
+        <v>41792365</v>
       </c>
       <c r="U191" t="n">
-        <v>41792364</v>
+        <v>41792365</v>
       </c>
       <c r="V191" t="n">
         <v>1900000</v>
@@ -16041,10 +16041,10 @@
         <v>0</v>
       </c>
       <c r="T192" t="n">
-        <v>49996613</v>
+        <v>49996614</v>
       </c>
       <c r="U192" t="n">
-        <v>49996613</v>
+        <v>49996614</v>
       </c>
       <c r="V192" t="n">
         <v>1910000</v>
@@ -16122,10 +16122,10 @@
         <v>0</v>
       </c>
       <c r="T193" t="n">
-        <v>48544371</v>
+        <v>48544372</v>
       </c>
       <c r="U193" t="n">
-        <v>48544371</v>
+        <v>48544372</v>
       </c>
       <c r="V193" t="n">
         <v>1920000</v>
@@ -16203,10 +16203,10 @@
         <v>0</v>
       </c>
       <c r="T194" t="n">
-        <v>39666029</v>
+        <v>39666030</v>
       </c>
       <c r="U194" t="n">
-        <v>39666029</v>
+        <v>39666030</v>
       </c>
       <c r="V194" t="n">
         <v>1930000</v>
@@ -16284,10 +16284,10 @@
         <v>0</v>
       </c>
       <c r="T195" t="n">
-        <v>78944925</v>
+        <v>78944926</v>
       </c>
       <c r="U195" t="n">
-        <v>78944925</v>
+        <v>78944926</v>
       </c>
       <c r="V195" t="n">
         <v>1940000</v>
@@ -16365,10 +16365,10 @@
         <v>0</v>
       </c>
       <c r="T196" t="n">
-        <v>124244778</v>
+        <v>124244779</v>
       </c>
       <c r="U196" t="n">
-        <v>124244778</v>
+        <v>124244779</v>
       </c>
       <c r="V196" t="n">
         <v>1950000</v>
@@ -16446,10 +16446,10 @@
         <v>0</v>
       </c>
       <c r="T197" t="n">
-        <v>103894489</v>
+        <v>103894490</v>
       </c>
       <c r="U197" t="n">
-        <v>103894489</v>
+        <v>103894490</v>
       </c>
       <c r="V197" t="n">
         <v>1960000</v>
@@ -16582,7 +16582,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>$103,894,489</t>
+          <t>$103,894,490</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -16592,7 +16592,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>$101,660,686</t>
+          <t>$101,660,687</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -16602,7 +16602,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>$205,415,389</t>
+          <t>$205,415,390</t>
         </is>
       </c>
     </row>
@@ -16614,7 +16614,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>$101,934,489</t>
+          <t>$101,934,490</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -16624,7 +16624,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>$99,700,686</t>
+          <t>$99,700,687</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -16634,7 +16634,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>$203,455,389</t>
+          <t>$203,455,390</t>
         </is>
       </c>
     </row>

</xml_diff>